<commit_message>
Update Pray For text; fix Thread View tour scroll-to-top on every step
- Content: regenerate content-overrides.js from workbook (Column AB "Pray
  For" now leads each prayer with "Pray for ..."). Adjust the two UI
  labels so they don't double up: Study session header "Before we begin,
  pray for:" -> "Before we begin:"; drop the redundant trailing period in
  the Meditate prayer-time lede when the text already ends in punctuation.

- Thread View tour: every step carried scrollId "thread-view-section", so
  GuidedTour re-navigated on each step, jumping to the page top then back
  down to the section before highlighting the target -- a disorienting
  bounce. Track the last-scrolled section (navScrollRef) and only
  re-navigate when the view or target section actually changes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RECAP MODE - Data Entry USE THIS v9 (synced).xlsx
+++ b/RECAP MODE - Data Entry USE THIS v9 (synced).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ClaudeLocal\OTOverviewAG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{703E27E0-AA83-4639-8996-1918A2A26298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA7DF321-7AF3-4FC2-8D93-19D3F72E455A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -204,9 +204,6 @@
     <t>John 5:39 — the purpose of the whole Old Testament is to know ___.</t>
   </si>
   <si>
-    <t>God to help us see Jesus and love Him more.</t>
-  </si>
-  <si>
     <t>As you reflect on Why OT? (OT Overview Why OT?), what does this passage reveal about God’s character that you can praise Him for?</t>
   </si>
   <si>
@@ -280,9 +277,6 @@
   <si>
     <t>• We often view God's rule as restrictive and rigid, while He shows himself as truly good, generous and life-giving.
 • Cross-ref to Revelation 21-22 to show the bookend: Eden restored as a city.</t>
-  </si>
-  <si>
-    <t>God to help us see His good rule and perfect kingdom order.</t>
   </si>
   <si>
     <t>As you reflect on Creation (Genesis 1-2), what does this passage reveal about God’s character that you can praise Him for?</t>
@@ -347,9 +341,6 @@
     <t>Salvation</t>
   </si>
   <si>
-    <t>eyes to see how God truly views sin, giving thanks for Jesus who dealt with the problem of sin completely.</t>
-  </si>
-  <si>
     <t>As you reflect on Fall (Genesis 3), what does this passage reveal about God’s character that you can praise Him for?</t>
   </si>
   <si>
@@ -421,9 +412,6 @@
     <t>Promises</t>
   </si>
   <si>
-    <t>eyes to see sin for what it truly is, but also giving thanks for Jesus who dealt with the problem of sin completely.</t>
-  </si>
-  <si>
     <t>As you reflect on Noah (Genesis 6-9), what does this passage reveal about God’s character that you can praise Him for?</t>
   </si>
   <si>
@@ -487,9 +475,6 @@
     <t>Luke 1 — in Christ comes the true reversal of the ___.</t>
   </si>
   <si>
-    <t>God to help us see His character through His promises.</t>
-  </si>
-  <si>
     <t>As you reflect on Abrahamic Covenant (Genesis 12 ; 15 ; 17), what does this passage reveal about God’s character that you can praise Him for?</t>
   </si>
   <si>
@@ -555,9 +540,6 @@
   </si>
   <si>
     <t>1 Corinthians 5:7 — Christ, our Passover ___, has been sacrificed.</t>
-  </si>
-  <si>
-    <t>God to show us His holiness, and also to appreciate Jesus' perfect sacrifice as the Passover lamb.</t>
   </si>
   <si>
     <t>As you reflect on Passover (Exodus 11-13), what does this passage reveal about God’s character that you can praise Him for?</t>
@@ -635,9 +617,6 @@
   </si>
   <si>
     <t>Promises &amp; Kingdom</t>
-  </si>
-  <si>
-    <t>us to appreciate God's holiness and mercy, ultimately appreciating His new covenant in Jesus.</t>
   </si>
   <si>
     <t>As you reflect on Mosaic Covenant (Exodus 19-20), what does this passage reveal about God’s character that you can praise Him for?</t>
@@ -788,9 +767,6 @@
     <t>Promises &amp; Salvation</t>
   </si>
   <si>
-    <t>us to appreciate Jesus - God's perfect favoured mediator, and to follow in Jesus' footsteps to be holy in Him.</t>
-  </si>
-  <si>
     <t>As you reflect on Golden Calf &amp; Renewal (Exodus 32-34), what does this passage reveal about God’s character that you can praise Him for?</t>
   </si>
   <si>
@@ -862,9 +838,6 @@
     <t>Hebrews 9 — Jesus is the perfect great high ___, both sacrifice and sin-bearer.</t>
   </si>
   <si>
-    <t>us to appreciate God's holiness in the Day of Atonement; giving thanks to Jesus, our great high priest, who has restored our relationship with God.</t>
-  </si>
-  <si>
     <t>As you reflect on Day of Atonement (Leviticus 16), what does this passage reveal about God’s character that you can praise Him for?</t>
   </si>
   <si>
@@ -928,9 +901,6 @@
     <t>Kingdom &amp; Promises</t>
   </si>
   <si>
-    <t>us to appreciate God's holiness and mercy; especially Him cleansing us from inside out and giving us His Spirit, through Jesus' life and death.</t>
-  </si>
-  <si>
     <t>As you reflect on Blessings &amp; Curses (Deuteronomy 28-30), what does this passage reveal about God’s character that you can praise Him for?</t>
   </si>
   <si>
@@ -2330,6 +2300,36 @@
   </si>
   <si>
     <t>Pause and speak to God. Consider His love for me. Take time to behold all the riches we have in the gospel.</t>
+  </si>
+  <si>
+    <t>Pray for God to help us see Jesus and love Him more.</t>
+  </si>
+  <si>
+    <t>Pray for God to help us see His good rule and perfect kingdom order.</t>
+  </si>
+  <si>
+    <t>Pray for eyes to see how God truly views sin, giving thanks for Jesus who dealt with the problem of sin completely.</t>
+  </si>
+  <si>
+    <t>Pray for eyes to see sin for what it truly is, but also giving thanks for Jesus who dealt with the problem of sin completely.</t>
+  </si>
+  <si>
+    <t>Pray for God to help us see His character through His promises.</t>
+  </si>
+  <si>
+    <t>Pray for God to show us His holiness, and also to appreciate Jesus' perfect sacrifice as the Passover lamb.</t>
+  </si>
+  <si>
+    <t>Pray for us to appreciate God's holiness and mercy, ultimately appreciating His new covenant in Jesus.</t>
+  </si>
+  <si>
+    <t>Pray for us to appreciate Jesus - God's perfect favoured mediator, and to follow in Jesus' footsteps to be holy in Him.</t>
+  </si>
+  <si>
+    <t>Pray for us to appreciate God's holiness in the Day of Atonement; giving thanks to Jesus, our great high priest, who has restored our relationship with God.</t>
+  </si>
+  <si>
+    <t>Pray for us to appreciate God's holiness and mercy; especially Him cleansing us from inside out and giving us His Spirit, through Jesus' life and death.</t>
   </si>
 </sst>
 </file>
@@ -2562,14 +2562,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2907,6 +2907,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="2">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{B691C7A0-7CA0-463D-887B-FAEA15CD6B3B}">
+  <we:reference id="wa200010725" version="1.0.0.1" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200010725" version="1.0.0.1" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;a7edc66e-11e7-4913-b4a6-1f61cb1c17f9&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
@@ -2920,431 +2942,431 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="21" t="s">
-        <v>294</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
+      <c r="A1" s="23" t="s">
+        <v>284</v>
+      </c>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="20" t="s">
-        <v>295</v>
-      </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
+      <c r="A2" s="22" t="s">
+        <v>285</v>
+      </c>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="20" t="s">
-        <v>296</v>
-      </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
+      <c r="A4" s="22" t="s">
+        <v>286</v>
+      </c>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="B5" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
       <c r="C5" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="B6" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
       <c r="C6" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="B7" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="C7" t="s">
-        <v>305</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
       <c r="B8" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="C8" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
-        <v>309</v>
-      </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
+      <c r="A10" s="22" t="s">
+        <v>299</v>
+      </c>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="B11" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="C11" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="B12" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="C12" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="B13" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="C13" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B14" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
       <c r="C14" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>321</v>
+        <v>311</v>
       </c>
       <c r="B15" t="s">
-        <v>322</v>
+        <v>312</v>
       </c>
       <c r="C15" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
       <c r="B16" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
       <c r="C16" t="s">
-        <v>326</v>
+        <v>316</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>327</v>
+        <v>317</v>
       </c>
       <c r="B17" t="s">
-        <v>328</v>
+        <v>318</v>
       </c>
       <c r="C17" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="B18" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
       <c r="C18" t="s">
-        <v>332</v>
+        <v>322</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>333</v>
+        <v>323</v>
       </c>
       <c r="B19" t="s">
-        <v>334</v>
+        <v>324</v>
       </c>
       <c r="C19" t="s">
-        <v>335</v>
+        <v>325</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
       <c r="B20" t="s">
-        <v>337</v>
+        <v>327</v>
       </c>
       <c r="C20" t="s">
-        <v>338</v>
+        <v>328</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>339</v>
+        <v>329</v>
       </c>
       <c r="B21" t="s">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="C21" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" s="20"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
+      <c r="A22" s="22"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>342</v>
+        <v>332</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>343</v>
+        <v>333</v>
       </c>
       <c r="B24" t="s">
-        <v>344</v>
+        <v>334</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>345</v>
+        <v>335</v>
       </c>
       <c r="B25" t="s">
-        <v>346</v>
+        <v>336</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>347</v>
+        <v>337</v>
       </c>
       <c r="B26" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>349</v>
+        <v>339</v>
       </c>
       <c r="B27" t="s">
-        <v>350</v>
+        <v>340</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>351</v>
+        <v>341</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>352</v>
+        <v>342</v>
       </c>
       <c r="B30" t="s">
-        <v>353</v>
+        <v>343</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>354</v>
+        <v>344</v>
       </c>
       <c r="B31" t="s">
-        <v>355</v>
+        <v>345</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>356</v>
+        <v>346</v>
       </c>
       <c r="B32" t="s">
-        <v>357</v>
+        <v>347</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>358</v>
+        <v>348</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>359</v>
+        <v>349</v>
       </c>
       <c r="B35" t="s">
-        <v>360</v>
+        <v>350</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
       <c r="B36" t="s">
-        <v>362</v>
+        <v>352</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>363</v>
+        <v>353</v>
       </c>
       <c r="B37" t="s">
-        <v>364</v>
+        <v>354</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>365</v>
+        <v>355</v>
       </c>
       <c r="B38" t="s">
-        <v>366</v>
+        <v>356</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>367</v>
+        <v>357</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>368</v>
+        <v>358</v>
       </c>
       <c r="B41" t="s">
-        <v>369</v>
+        <v>359</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>370</v>
+        <v>360</v>
       </c>
       <c r="B42" t="s">
-        <v>371</v>
+        <v>361</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>372</v>
+        <v>362</v>
       </c>
       <c r="B43" t="s">
-        <v>373</v>
+        <v>363</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>374</v>
+        <v>364</v>
       </c>
       <c r="B44" t="s">
-        <v>375</v>
+        <v>365</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>376</v>
+        <v>366</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="93" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>377</v>
+        <v>367</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>378</v>
+        <v>368</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>379</v>
+        <v>369</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>380</v>
+        <v>370</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>381</v>
+        <v>371</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="62" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>383</v>
+        <v>373</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>384</v>
+        <v>374</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="62" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>387</v>
+        <v>377</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>390</v>
+        <v>380</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>391</v>
+        <v>381</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>392</v>
+        <v>382</v>
       </c>
       <c r="B56" t="s">
-        <v>393</v>
+        <v>383</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>394</v>
+        <v>384</v>
       </c>
       <c r="B57" t="s">
-        <v>395</v>
+        <v>385</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>396</v>
+        <v>386</v>
       </c>
       <c r="B58" t="s">
-        <v>397</v>
+        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -3589,19 +3611,19 @@
       <c r="Z2" s="12"/>
       <c r="AA2" s="12"/>
       <c r="AB2" s="12" t="s">
+        <v>723</v>
+      </c>
+      <c r="AC2" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="AC2" s="12" t="s">
+      <c r="AD2" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="AD2" s="12" t="s">
+      <c r="AE2" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="AE2" s="12" t="s">
+      <c r="AF2" s="12" t="s">
         <v>62</v>
-      </c>
-      <c r="AF2" s="12" t="s">
-        <v>63</v>
       </c>
       <c r="AG2" s="12"/>
       <c r="AH2" s="12"/>
@@ -3609,7 +3631,7 @@
       <c r="AJ2" s="12"/>
       <c r="AK2" s="12"/>
       <c r="AL2" s="12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AM2" s="12"/>
       <c r="AN2" s="18"/>
@@ -3620,49 +3642,49 @@
         <v>2</v>
       </c>
       <c r="B3" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="D3" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="E3" s="13" t="s">
+        <v>677</v>
+      </c>
+      <c r="F3" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="E3" s="13" t="s">
-        <v>687</v>
-      </c>
-      <c r="F3" s="13" t="s">
+      <c r="G3" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="H3" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="I3" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="J3" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="J3" s="13" t="s">
+      <c r="K3" s="13" t="s">
         <v>72</v>
-      </c>
-      <c r="K3" s="13" t="s">
-        <v>73</v>
       </c>
       <c r="L3" s="13"/>
       <c r="M3" s="13"/>
       <c r="N3" s="13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O3" s="13"/>
       <c r="P3" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q3" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="Q3" s="13" t="s">
+      <c r="R3" s="13" t="s">
         <v>76</v>
-      </c>
-      <c r="R3" s="13" t="s">
-        <v>77</v>
       </c>
       <c r="S3" s="13"/>
       <c r="T3" s="13"/>
@@ -3670,37 +3692,37 @@
         <v>55</v>
       </c>
       <c r="V3" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="W3" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="W3" s="13" t="s">
+      <c r="X3" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="X3" s="13" t="s">
+      <c r="Y3" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="Y3" s="13" t="s">
+      <c r="Z3" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="Z3" s="13" t="s">
+      <c r="AA3" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="AA3" s="13" t="s">
+      <c r="AB3" s="13" t="s">
+        <v>724</v>
+      </c>
+      <c r="AC3" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="AB3" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC3" s="13" t="s">
-        <v>85</v>
-      </c>
       <c r="AD3" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE3" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="AE3" s="13" t="s">
+      <c r="AF3" s="13" t="s">
         <v>62</v>
-      </c>
-      <c r="AF3" s="13" t="s">
-        <v>63</v>
       </c>
       <c r="AG3" s="13"/>
       <c r="AH3" s="13"/>
@@ -3709,11 +3731,11 @@
       <c r="AK3" s="13"/>
       <c r="AL3" s="13"/>
       <c r="AM3" s="13"/>
-      <c r="AN3" s="22" t="s">
-        <v>716</v>
-      </c>
-      <c r="AO3" s="22" t="s">
-        <v>722</v>
+      <c r="AN3" s="20" t="s">
+        <v>706</v>
+      </c>
+      <c r="AO3" s="20" t="s">
+        <v>712</v>
       </c>
     </row>
     <row r="4" spans="1:41" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3721,91 +3743,91 @@
         <v>3</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C4" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="F4" s="12" t="s">
+        <v>678</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="F4" s="12" t="s">
-        <v>688</v>
-      </c>
-      <c r="G4" s="12" t="s">
+      <c r="I4" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="K4" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="L4" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="M4" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="N4" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="L4" s="12" t="s">
+      <c r="O4" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="M4" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="N4" s="12" t="s">
+      <c r="P4" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="Q4" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="P4" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q4" s="12" t="s">
-        <v>98</v>
-      </c>
       <c r="R4" s="12" t="s">
-        <v>690</v>
+        <v>680</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>691</v>
+        <v>681</v>
       </c>
       <c r="T4" s="12"/>
       <c r="U4" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="V4" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="W4" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="V4" s="12" t="s">
+      <c r="X4" s="12" t="s">
         <v>100</v>
-      </c>
-      <c r="W4" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="X4" s="12" t="s">
-        <v>102</v>
       </c>
       <c r="Y4" s="12"/>
       <c r="Z4" s="12" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="AA4" s="12"/>
       <c r="AB4" s="12" t="s">
-        <v>104</v>
+        <v>725</v>
       </c>
       <c r="AC4" s="12" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="AD4" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE4" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="AE4" s="12" t="s">
+      <c r="AF4" s="12" t="s">
         <v>62</v>
-      </c>
-      <c r="AF4" s="12" t="s">
-        <v>63</v>
       </c>
       <c r="AG4" s="12"/>
       <c r="AH4" s="12"/>
@@ -3814,11 +3836,11 @@
       <c r="AK4" s="12"/>
       <c r="AL4" s="12"/>
       <c r="AM4" s="12"/>
-      <c r="AN4" s="23" t="s">
-        <v>717</v>
+      <c r="AN4" s="21" t="s">
+        <v>707</v>
       </c>
       <c r="AO4" s="12" t="s">
-        <v>723</v>
+        <v>713</v>
       </c>
     </row>
     <row r="5" spans="1:41" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3826,91 +3848,91 @@
         <v>4</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C5" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="F5" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="G5" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="H5" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="I5" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="J5" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="K5" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="I5" s="13" t="s">
+      <c r="L5" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="J5" s="13" t="s">
+      <c r="M5" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="N5" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="L5" s="13" t="s">
+      <c r="O5" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="M5" s="13" t="s">
+      <c r="P5" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="N5" s="13" t="s">
+      <c r="Q5" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="O5" s="13" t="s">
+      <c r="R5" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="P5" s="13" t="s">
+      <c r="S5" s="13" t="s">
         <v>119</v>
-      </c>
-      <c r="Q5" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="R5" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="S5" s="13" t="s">
-        <v>122</v>
       </c>
       <c r="T5" s="13"/>
       <c r="U5" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="V5" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="W5" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="X5" s="13" t="s">
         <v>123</v>
-      </c>
-      <c r="V5" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="W5" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="X5" s="13" t="s">
-        <v>126</v>
       </c>
       <c r="Y5" s="13"/>
       <c r="Z5" s="13" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="AA5" s="13"/>
       <c r="AB5" s="13" t="s">
-        <v>128</v>
+        <v>726</v>
       </c>
       <c r="AC5" s="13" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="AD5" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE5" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="AE5" s="13" t="s">
+      <c r="AF5" s="13" t="s">
         <v>62</v>
-      </c>
-      <c r="AF5" s="13" t="s">
-        <v>63</v>
       </c>
       <c r="AG5" s="13"/>
       <c r="AH5" s="13"/>
@@ -3920,10 +3942,10 @@
       <c r="AL5" s="13"/>
       <c r="AM5" s="13"/>
       <c r="AN5" s="13" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="AO5" s="13" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:41" ht="31" customHeight="1" x14ac:dyDescent="0.35">
@@ -3931,91 +3953,91 @@
         <v>5</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C6" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="G6" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="H6" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="I6" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="J6" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="K6" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="L6" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="M6" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="J6" s="12" t="s">
+      <c r="N6" s="12" t="s">
         <v>137</v>
-      </c>
-      <c r="K6" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="L6" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="M6" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="N6" s="12" t="s">
-        <v>141</v>
       </c>
       <c r="O6" s="12"/>
       <c r="P6" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q6" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="R6" s="12" t="s">
+        <v>682</v>
+      </c>
+      <c r="S6" s="12" t="s">
+        <v>683</v>
+      </c>
+      <c r="T6" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="U6" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="V6" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="Q6" s="12" t="s">
+      <c r="W6" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="R6" s="12" t="s">
-        <v>692</v>
-      </c>
-      <c r="S6" s="12" t="s">
-        <v>693</v>
-      </c>
-      <c r="T6" s="12" t="s">
+      <c r="X6" s="12" t="s">
         <v>144</v>
-      </c>
-      <c r="U6" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="V6" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="W6" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="X6" s="12" t="s">
-        <v>148</v>
       </c>
       <c r="Y6" s="12"/>
       <c r="Z6" s="12" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="AA6" s="12"/>
       <c r="AB6" s="12" t="s">
-        <v>149</v>
+        <v>727</v>
       </c>
       <c r="AC6" s="12" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="AD6" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE6" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="AE6" s="12" t="s">
+      <c r="AF6" s="12" t="s">
         <v>62</v>
-      </c>
-      <c r="AF6" s="12" t="s">
-        <v>63</v>
       </c>
       <c r="AG6" s="12"/>
       <c r="AH6" s="12"/>
@@ -4024,11 +4046,11 @@
       <c r="AK6" s="12"/>
       <c r="AL6" s="12"/>
       <c r="AM6" s="12"/>
-      <c r="AN6" s="23" t="s">
-        <v>718</v>
-      </c>
-      <c r="AO6" s="23" t="s">
-        <v>719</v>
+      <c r="AN6" s="21" t="s">
+        <v>708</v>
+      </c>
+      <c r="AO6" s="21" t="s">
+        <v>709</v>
       </c>
     </row>
     <row r="7" spans="1:41" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4036,89 +4058,89 @@
         <v>6</v>
       </c>
       <c r="B7" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="G7" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="H7" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="I7" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="J7" s="13" t="s">
         <v>154</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="H7" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="I7" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="J7" s="13" t="s">
-        <v>159</v>
       </c>
       <c r="K7" s="13"/>
       <c r="L7" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="M7" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="N7" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="O7" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="P7" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q7" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="M7" s="13" t="s">
+      <c r="R7" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="N7" s="13" t="s">
+      <c r="S7" s="13" t="s">
         <v>162</v>
-      </c>
-      <c r="O7" s="13" t="s">
-        <v>163</v>
-      </c>
-      <c r="P7" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="Q7" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="R7" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="S7" s="13" t="s">
-        <v>167</v>
       </c>
       <c r="T7" s="13"/>
       <c r="U7" s="13" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="V7" s="13" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="W7" s="13" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="X7" s="13" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="Y7" s="13"/>
       <c r="Z7" s="13" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="AA7" s="13"/>
       <c r="AB7" s="13" t="s">
-        <v>171</v>
+        <v>728</v>
       </c>
       <c r="AC7" s="13" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="AD7" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE7" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="AE7" s="13" t="s">
+      <c r="AF7" s="13" t="s">
         <v>62</v>
-      </c>
-      <c r="AF7" s="13" t="s">
-        <v>63</v>
       </c>
       <c r="AG7" s="13"/>
       <c r="AH7" s="13"/>
@@ -4127,11 +4149,11 @@
       <c r="AK7" s="13"/>
       <c r="AL7" s="13"/>
       <c r="AM7" s="13"/>
-      <c r="AN7" s="22" t="s">
-        <v>721</v>
-      </c>
-      <c r="AO7" s="22" t="s">
-        <v>720</v>
+      <c r="AN7" s="20" t="s">
+        <v>711</v>
+      </c>
+      <c r="AO7" s="20" t="s">
+        <v>710</v>
       </c>
     </row>
     <row r="8" spans="1:41" ht="124" customHeight="1" x14ac:dyDescent="0.35">
@@ -4139,91 +4161,91 @@
         <v>7</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C8" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="I8" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="J8" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="K8" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="L8" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="M8" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="N8" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="O8" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="J8" s="12" t="s">
+      <c r="P8" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="K8" s="12" t="s">
+      <c r="Q8" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="L8" s="12" t="s">
+      <c r="R8" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="M8" s="12" t="s">
+      <c r="S8" s="12" t="s">
         <v>183</v>
-      </c>
-      <c r="N8" s="12" t="s">
-        <v>184</v>
-      </c>
-      <c r="O8" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="P8" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="Q8" s="12" t="s">
-        <v>187</v>
-      </c>
-      <c r="R8" s="12" t="s">
-        <v>188</v>
-      </c>
-      <c r="S8" s="12" t="s">
-        <v>189</v>
       </c>
       <c r="T8" s="12"/>
       <c r="U8" s="12" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="V8" s="12" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="W8" s="12" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="X8" s="12" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="Y8" s="12"/>
       <c r="Z8" s="12" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="AA8" s="12"/>
       <c r="AB8" s="12" t="s">
-        <v>195</v>
+        <v>729</v>
       </c>
       <c r="AC8" s="12" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="AD8" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE8" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="AE8" s="12" t="s">
+      <c r="AF8" s="12" t="s">
         <v>62</v>
-      </c>
-      <c r="AF8" s="12" t="s">
-        <v>63</v>
       </c>
       <c r="AG8" s="12"/>
       <c r="AH8" s="12"/>
@@ -4232,11 +4254,11 @@
       <c r="AK8" s="12"/>
       <c r="AL8" s="12"/>
       <c r="AM8" s="12"/>
-      <c r="AN8" s="23" t="s">
-        <v>724</v>
-      </c>
-      <c r="AO8" s="23" t="s">
-        <v>725</v>
+      <c r="AN8" s="21" t="s">
+        <v>714</v>
+      </c>
+      <c r="AO8" s="21" t="s">
+        <v>715</v>
       </c>
     </row>
     <row r="9" spans="1:41" ht="77.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4244,93 +4266,93 @@
         <v>8</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C9" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="I9" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="J9" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="K9" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="L9" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="M9" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="N9" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="O9" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="P9" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="Q9" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="R9" s="13" t="s">
         <v>205</v>
       </c>
-      <c r="L9" s="13" t="s">
+      <c r="S9" s="13" t="s">
+        <v>684</v>
+      </c>
+      <c r="T9" s="13" t="s">
+        <v>685</v>
+      </c>
+      <c r="U9" s="13" t="s">
         <v>206</v>
       </c>
-      <c r="M9" s="13" t="s">
+      <c r="V9" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="N9" s="13" t="s">
+      <c r="W9" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="O9" s="13" t="s">
+      <c r="X9" s="13" t="s">
         <v>209</v>
-      </c>
-      <c r="P9" s="13" t="s">
-        <v>210</v>
-      </c>
-      <c r="Q9" s="13" t="s">
-        <v>211</v>
-      </c>
-      <c r="R9" s="13" t="s">
-        <v>212</v>
-      </c>
-      <c r="S9" s="13" t="s">
-        <v>694</v>
-      </c>
-      <c r="T9" s="13" t="s">
-        <v>695</v>
-      </c>
-      <c r="U9" s="13" t="s">
-        <v>213</v>
-      </c>
-      <c r="V9" s="13" t="s">
-        <v>214</v>
-      </c>
-      <c r="W9" s="13" t="s">
-        <v>215</v>
-      </c>
-      <c r="X9" s="13" t="s">
-        <v>216</v>
       </c>
       <c r="Y9" s="13"/>
       <c r="Z9" s="13" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="AA9" s="13"/>
       <c r="AB9" s="13" t="s">
-        <v>195</v>
+        <v>729</v>
       </c>
       <c r="AC9" s="13" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="AD9" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE9" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="AE9" s="13" t="s">
+      <c r="AF9" s="13" t="s">
         <v>62</v>
-      </c>
-      <c r="AF9" s="13" t="s">
-        <v>63</v>
       </c>
       <c r="AG9" s="13"/>
       <c r="AH9" s="13"/>
@@ -4339,11 +4361,11 @@
       <c r="AK9" s="13"/>
       <c r="AL9" s="13"/>
       <c r="AM9" s="13"/>
-      <c r="AN9" s="22" t="s">
-        <v>726</v>
-      </c>
-      <c r="AO9" s="22" t="s">
-        <v>729</v>
+      <c r="AN9" s="20" t="s">
+        <v>716</v>
+      </c>
+      <c r="AO9" s="20" t="s">
+        <v>719</v>
       </c>
     </row>
     <row r="10" spans="1:41" ht="170.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4351,91 +4373,91 @@
         <v>9</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C10" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="I10" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="J10" s="12" t="s">
         <v>218</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="K10" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="L10" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="M10" s="12" t="s">
         <v>221</v>
       </c>
-      <c r="G10" s="12" t="s">
+      <c r="N10" s="12" t="s">
         <v>222</v>
       </c>
-      <c r="H10" s="12" t="s">
+      <c r="O10" s="12" t="s">
         <v>223</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="P10" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="J10" s="12" t="s">
+      <c r="Q10" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="K10" s="12" t="s">
+      <c r="R10" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="L10" s="12" t="s">
+      <c r="S10" s="12" t="s">
         <v>227</v>
-      </c>
-      <c r="M10" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="N10" s="12" t="s">
-        <v>229</v>
-      </c>
-      <c r="O10" s="12" t="s">
-        <v>230</v>
-      </c>
-      <c r="P10" s="12" t="s">
-        <v>231</v>
-      </c>
-      <c r="Q10" s="12" t="s">
-        <v>232</v>
-      </c>
-      <c r="R10" s="12" t="s">
-        <v>233</v>
-      </c>
-      <c r="S10" s="12" t="s">
-        <v>234</v>
       </c>
       <c r="T10" s="12"/>
       <c r="U10" s="12" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="V10" s="12" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="W10" s="12" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="X10" s="12" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="Y10" s="12"/>
       <c r="Z10" s="12" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="AA10" s="12"/>
       <c r="AB10" s="12" t="s">
-        <v>240</v>
+        <v>730</v>
       </c>
       <c r="AC10" s="12" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="AD10" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE10" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="AE10" s="12" t="s">
+      <c r="AF10" s="12" t="s">
         <v>62</v>
-      </c>
-      <c r="AF10" s="12" t="s">
-        <v>63</v>
       </c>
       <c r="AG10" s="12"/>
       <c r="AH10" s="12"/>
@@ -4444,11 +4466,11 @@
       <c r="AK10" s="12"/>
       <c r="AL10" s="12"/>
       <c r="AM10" s="12"/>
-      <c r="AN10" s="23" t="s">
-        <v>727</v>
-      </c>
-      <c r="AO10" s="23" t="s">
-        <v>728</v>
+      <c r="AN10" s="21" t="s">
+        <v>717</v>
+      </c>
+      <c r="AO10" s="21" t="s">
+        <v>718</v>
       </c>
     </row>
     <row r="11" spans="1:41" ht="201.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4456,89 +4478,89 @@
         <v>10</v>
       </c>
       <c r="B11" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>235</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>238</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="H11" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="I11" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="J11" s="13" t="s">
         <v>242</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="K11" s="13" t="s">
         <v>243</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="L11" s="13" t="s">
         <v>244</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>245</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>246</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>247</v>
-      </c>
-      <c r="H11" s="13" t="s">
-        <v>248</v>
-      </c>
-      <c r="I11" s="13" t="s">
-        <v>249</v>
-      </c>
-      <c r="J11" s="13" t="s">
-        <v>250</v>
-      </c>
-      <c r="K11" s="13" t="s">
-        <v>251</v>
-      </c>
-      <c r="L11" s="13" t="s">
-        <v>252</v>
       </c>
       <c r="M11" s="13"/>
       <c r="N11" s="13" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="O11" s="13" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="P11" s="13" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="Q11" s="13" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="R11" s="13" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="S11" s="13" t="s">
-        <v>698</v>
+        <v>688</v>
       </c>
       <c r="T11" s="13"/>
       <c r="U11" s="13" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="V11" s="13" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="W11" s="13" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="X11" s="13" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="Y11" s="13"/>
       <c r="Z11" s="13" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="AA11" s="13"/>
       <c r="AB11" s="13" t="s">
-        <v>262</v>
+        <v>731</v>
       </c>
       <c r="AC11" s="13" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="AD11" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE11" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="AE11" s="13" t="s">
+      <c r="AF11" s="13" t="s">
         <v>62</v>
-      </c>
-      <c r="AF11" s="13" t="s">
-        <v>63</v>
       </c>
       <c r="AG11" s="13"/>
       <c r="AH11" s="13"/>
@@ -4547,11 +4569,11 @@
       <c r="AK11" s="13"/>
       <c r="AL11" s="13"/>
       <c r="AM11" s="13"/>
-      <c r="AN11" s="22" t="s">
-        <v>724</v>
-      </c>
-      <c r="AO11" s="22" t="s">
-        <v>730</v>
+      <c r="AN11" s="20" t="s">
+        <v>714</v>
+      </c>
+      <c r="AO11" s="20" t="s">
+        <v>720</v>
       </c>
     </row>
     <row r="12" spans="1:41" ht="263.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4559,91 +4581,91 @@
         <v>11</v>
       </c>
       <c r="B12" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>256</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="I12" s="12" t="s">
+        <v>705</v>
+      </c>
+      <c r="J12" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="K12" s="12" t="s">
+        <v>263</v>
+      </c>
+      <c r="L12" s="12" t="s">
         <v>264</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="M12" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="N12" s="12" t="s">
         <v>265</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="O12" s="12" t="s">
         <v>266</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="P12" s="12" t="s">
         <v>267</v>
       </c>
-      <c r="F12" s="12" t="s">
-        <v>268</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="H12" s="12" t="s">
-        <v>270</v>
-      </c>
-      <c r="I12" s="12" t="s">
-        <v>715</v>
-      </c>
-      <c r="J12" s="12" t="s">
-        <v>271</v>
-      </c>
-      <c r="K12" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="L12" s="12" t="s">
-        <v>273</v>
-      </c>
-      <c r="M12" s="12" t="s">
-        <v>273</v>
-      </c>
-      <c r="N12" s="12" t="s">
-        <v>274</v>
-      </c>
-      <c r="O12" s="12" t="s">
-        <v>275</v>
-      </c>
-      <c r="P12" s="12" t="s">
-        <v>276</v>
-      </c>
       <c r="Q12" s="12" t="s">
-        <v>699</v>
+        <v>689</v>
       </c>
       <c r="R12" s="12" t="s">
-        <v>696</v>
+        <v>686</v>
       </c>
       <c r="S12" s="12" t="s">
-        <v>697</v>
+        <v>687</v>
       </c>
       <c r="T12" s="12"/>
       <c r="U12" s="12" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="V12" s="12" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="W12" s="12" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="X12" s="12" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="Y12" s="12"/>
       <c r="Z12" s="12" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="AA12" s="12"/>
       <c r="AB12" s="12" t="s">
-        <v>282</v>
+        <v>732</v>
       </c>
       <c r="AC12" s="12" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="AD12" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE12" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="AE12" s="12" t="s">
+      <c r="AF12" s="12" t="s">
         <v>62</v>
-      </c>
-      <c r="AF12" s="12" t="s">
-        <v>63</v>
       </c>
       <c r="AG12" s="12"/>
       <c r="AH12" s="12"/>
@@ -4652,11 +4674,11 @@
       <c r="AK12" s="12"/>
       <c r="AL12" s="12"/>
       <c r="AM12" s="12"/>
-      <c r="AN12" s="23" t="s">
-        <v>731</v>
-      </c>
-      <c r="AO12" s="23" t="s">
-        <v>732</v>
+      <c r="AN12" s="21" t="s">
+        <v>721</v>
+      </c>
+      <c r="AO12" s="21" t="s">
+        <v>722</v>
       </c>
     </row>
     <row r="13" spans="1:41" ht="87.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4664,24 +4686,24 @@
         <v>12</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
       <c r="I13" s="13" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="J13" s="13"/>
       <c r="K13" s="13"/>
@@ -4695,10 +4717,10 @@
       <c r="S13" s="13"/>
       <c r="T13" s="13"/>
       <c r="U13" s="13" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="V13" s="13" t="s">
-        <v>291</v>
+        <v>281</v>
       </c>
       <c r="W13" s="13"/>
       <c r="X13" s="13"/>
@@ -4707,16 +4729,16 @@
       <c r="AA13" s="13"/>
       <c r="AB13" s="13"/>
       <c r="AC13" s="13" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
       <c r="AD13" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE13" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="AE13" s="13" t="s">
+      <c r="AF13" s="13" t="s">
         <v>62</v>
-      </c>
-      <c r="AF13" s="13" t="s">
-        <v>63</v>
       </c>
       <c r="AG13" s="13"/>
       <c r="AH13" s="13"/>
@@ -4724,10 +4746,10 @@
       <c r="AJ13" s="13"/>
       <c r="AK13" s="13"/>
       <c r="AL13" s="13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AM13" s="13" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="AN13" s="19"/>
       <c r="AO13" s="19"/>
@@ -4775,49 +4797,49 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
+        <v>388</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>392</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>394</v>
+      </c>
+      <c r="I1" s="15" t="s">
+        <v>395</v>
+      </c>
+      <c r="J1" s="15" t="s">
+        <v>396</v>
+      </c>
+      <c r="K1" s="15" t="s">
+        <v>397</v>
+      </c>
+      <c r="L1" s="16" t="s">
         <v>398</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="M1" s="16" t="s">
         <v>399</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="N1" s="16" t="s">
         <v>400</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="O1" s="7" t="s">
         <v>401</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="P1" s="11" t="s">
         <v>402</v>
-      </c>
-      <c r="G1" s="14" t="s">
-        <v>403</v>
-      </c>
-      <c r="H1" s="14" t="s">
-        <v>404</v>
-      </c>
-      <c r="I1" s="15" t="s">
-        <v>405</v>
-      </c>
-      <c r="J1" s="15" t="s">
-        <v>406</v>
-      </c>
-      <c r="K1" s="15" t="s">
-        <v>407</v>
-      </c>
-      <c r="L1" s="16" t="s">
-        <v>408</v>
-      </c>
-      <c r="M1" s="16" t="s">
-        <v>409</v>
-      </c>
-      <c r="N1" s="16" t="s">
-        <v>410</v>
-      </c>
-      <c r="O1" s="7" t="s">
-        <v>411</v>
-      </c>
-      <c r="P1" s="11" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -4834,7 +4856,7 @@
         <v>49</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>413</v>
+        <v>403</v>
       </c>
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
@@ -4862,7 +4884,7 @@
         <v>50</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>414</v>
+        <v>404</v>
       </c>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
@@ -4890,7 +4912,7 @@
         <v>51</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>415</v>
+        <v>405</v>
       </c>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
@@ -4909,46 +4931,46 @@
         <v>2</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C5" s="13">
         <v>1</v>
       </c>
       <c r="D5" s="13" t="s">
+        <v>406</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>407</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>408</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>409</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>410</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>679</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>411</v>
+      </c>
+      <c r="K5" s="13" t="s">
+        <v>412</v>
+      </c>
+      <c r="L5" s="13" t="s">
+        <v>413</v>
+      </c>
+      <c r="M5" s="13" t="s">
+        <v>414</v>
+      </c>
+      <c r="N5" s="13" t="s">
+        <v>415</v>
+      </c>
+      <c r="O5" s="13" t="s">
         <v>416</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>417</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>418</v>
-      </c>
-      <c r="G5" s="13" t="s">
-        <v>419</v>
-      </c>
-      <c r="H5" s="13" t="s">
-        <v>420</v>
-      </c>
-      <c r="I5" s="13" t="s">
-        <v>689</v>
-      </c>
-      <c r="J5" s="13" t="s">
-        <v>421</v>
-      </c>
-      <c r="K5" s="13" t="s">
-        <v>422</v>
-      </c>
-      <c r="L5" s="13" t="s">
-        <v>423</v>
-      </c>
-      <c r="M5" s="13" t="s">
-        <v>424</v>
-      </c>
-      <c r="N5" s="13" t="s">
-        <v>425</v>
-      </c>
-      <c r="O5" s="13" t="s">
-        <v>426</v>
       </c>
       <c r="P5" s="13"/>
     </row>
@@ -4957,46 +4979,46 @@
         <v>2</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C6" s="12">
         <v>2</v>
       </c>
       <c r="D6" s="12" t="s">
+        <v>417</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>418</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>419</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>420</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>421</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>422</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>423</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>424</v>
+      </c>
+      <c r="L6" s="12" t="s">
+        <v>425</v>
+      </c>
+      <c r="M6" s="12" t="s">
+        <v>426</v>
+      </c>
+      <c r="N6" s="12" t="s">
         <v>427</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="O6" s="12" t="s">
         <v>428</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>429</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>430</v>
-      </c>
-      <c r="H6" s="12" t="s">
-        <v>431</v>
-      </c>
-      <c r="I6" s="12" t="s">
-        <v>432</v>
-      </c>
-      <c r="J6" s="12" t="s">
-        <v>433</v>
-      </c>
-      <c r="K6" s="12" t="s">
-        <v>434</v>
-      </c>
-      <c r="L6" s="12" t="s">
-        <v>435</v>
-      </c>
-      <c r="M6" s="12" t="s">
-        <v>436</v>
-      </c>
-      <c r="N6" s="12" t="s">
-        <v>437</v>
-      </c>
-      <c r="O6" s="12" t="s">
-        <v>438</v>
       </c>
       <c r="P6" s="12"/>
     </row>
@@ -5005,38 +5027,38 @@
         <v>3</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C7" s="13">
         <v>1</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>439</v>
+        <v>429</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>441</v>
+        <v>431</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>442</v>
+        <v>432</v>
       </c>
       <c r="H7" s="13"/>
       <c r="I7" s="13" t="s">
-        <v>443</v>
+        <v>433</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>444</v>
+        <v>434</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>445</v>
+        <v>435</v>
       </c>
       <c r="L7" s="13"/>
       <c r="M7" s="13"/>
       <c r="N7" s="13"/>
       <c r="O7" s="13" t="s">
-        <v>445</v>
+        <v>435</v>
       </c>
       <c r="P7" s="13"/>
     </row>
@@ -5045,40 +5067,40 @@
         <v>3</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C8" s="12">
         <v>2</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>446</v>
+        <v>436</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>447</v>
+        <v>437</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>448</v>
+        <v>438</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>449</v>
+        <v>439</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>451</v>
+        <v>441</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>452</v>
+        <v>442</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>453</v>
+        <v>443</v>
       </c>
       <c r="L8" s="12"/>
       <c r="M8" s="12"/>
       <c r="N8" s="12"/>
       <c r="O8" s="12" t="s">
-        <v>454</v>
+        <v>444</v>
       </c>
       <c r="P8" s="12"/>
     </row>
@@ -5087,34 +5109,34 @@
         <v>3</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C9" s="13">
         <v>3</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>455</v>
+        <v>445</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>456</v>
+        <v>446</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>457</v>
+        <v>447</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>458</v>
+        <v>448</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>459</v>
+        <v>449</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>460</v>
+        <v>450</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>461</v>
+        <v>451</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>462</v>
+        <v>452</v>
       </c>
       <c r="L9" s="13"/>
       <c r="M9" s="13"/>
@@ -5127,42 +5149,42 @@
         <v>4</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C10" s="12">
         <v>1</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>463</v>
+        <v>453</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>464</v>
+        <v>454</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>465</v>
+        <v>455</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>466</v>
+        <v>456</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>467</v>
+        <v>457</v>
       </c>
       <c r="I10" s="12" t="s">
-        <v>468</v>
+        <v>458</v>
       </c>
       <c r="J10" s="12"/>
       <c r="K10" s="12" t="s">
-        <v>469</v>
+        <v>459</v>
       </c>
       <c r="L10" s="12" t="s">
-        <v>470</v>
+        <v>460</v>
       </c>
       <c r="M10" s="12"/>
       <c r="N10" s="12" t="s">
-        <v>471</v>
+        <v>461</v>
       </c>
       <c r="O10" s="12" t="s">
-        <v>472</v>
+        <v>462</v>
       </c>
       <c r="P10" s="12"/>
     </row>
@@ -5171,46 +5193,46 @@
         <v>4</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C11" s="13">
         <v>2</v>
       </c>
       <c r="D11" s="13" t="s">
+        <v>463</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>464</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>465</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>466</v>
+      </c>
+      <c r="H11" s="13" t="s">
+        <v>467</v>
+      </c>
+      <c r="I11" s="13" t="s">
+        <v>468</v>
+      </c>
+      <c r="J11" s="13" t="s">
+        <v>469</v>
+      </c>
+      <c r="K11" s="13" t="s">
+        <v>470</v>
+      </c>
+      <c r="L11" s="13" t="s">
+        <v>471</v>
+      </c>
+      <c r="M11" s="13" t="s">
+        <v>472</v>
+      </c>
+      <c r="N11" s="13" t="s">
         <v>473</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="O11" s="13" t="s">
         <v>474</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>475</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>476</v>
-      </c>
-      <c r="H11" s="13" t="s">
-        <v>477</v>
-      </c>
-      <c r="I11" s="13" t="s">
-        <v>478</v>
-      </c>
-      <c r="J11" s="13" t="s">
-        <v>479</v>
-      </c>
-      <c r="K11" s="13" t="s">
-        <v>480</v>
-      </c>
-      <c r="L11" s="13" t="s">
-        <v>481</v>
-      </c>
-      <c r="M11" s="13" t="s">
-        <v>482</v>
-      </c>
-      <c r="N11" s="13" t="s">
-        <v>483</v>
-      </c>
-      <c r="O11" s="13" t="s">
-        <v>484</v>
       </c>
       <c r="P11" s="13"/>
     </row>
@@ -5219,46 +5241,46 @@
         <v>4</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C12" s="12">
         <v>3</v>
       </c>
       <c r="D12" s="12" t="s">
+        <v>475</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>476</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>477</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>478</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>479</v>
+      </c>
+      <c r="I12" s="12" t="s">
+        <v>480</v>
+      </c>
+      <c r="J12" s="12" t="s">
+        <v>481</v>
+      </c>
+      <c r="K12" s="12" t="s">
+        <v>482</v>
+      </c>
+      <c r="L12" s="12" t="s">
+        <v>483</v>
+      </c>
+      <c r="M12" s="12" t="s">
+        <v>484</v>
+      </c>
+      <c r="N12" s="12" t="s">
         <v>485</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="O12" s="12" t="s">
         <v>486</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>487</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="H12" s="12" t="s">
-        <v>489</v>
-      </c>
-      <c r="I12" s="12" t="s">
-        <v>490</v>
-      </c>
-      <c r="J12" s="12" t="s">
-        <v>491</v>
-      </c>
-      <c r="K12" s="12" t="s">
-        <v>492</v>
-      </c>
-      <c r="L12" s="12" t="s">
-        <v>493</v>
-      </c>
-      <c r="M12" s="12" t="s">
-        <v>494</v>
-      </c>
-      <c r="N12" s="12" t="s">
-        <v>495</v>
-      </c>
-      <c r="O12" s="12" t="s">
-        <v>496</v>
       </c>
       <c r="P12" s="12"/>
     </row>
@@ -5267,40 +5289,40 @@
         <v>5</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C13" s="13">
         <v>1</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>497</v>
+        <v>487</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>498</v>
+        <v>488</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>499</v>
+        <v>489</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>501</v>
+        <v>491</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>502</v>
+        <v>492</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>503</v>
+        <v>493</v>
       </c>
       <c r="K13" s="13" t="s">
-        <v>504</v>
+        <v>494</v>
       </c>
       <c r="L13" s="13"/>
       <c r="M13" s="13"/>
       <c r="N13" s="13"/>
       <c r="O13" s="13" t="s">
-        <v>505</v>
+        <v>495</v>
       </c>
       <c r="P13" s="13"/>
     </row>
@@ -5309,40 +5331,40 @@
         <v>5</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C14" s="12">
         <v>2</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>506</v>
+        <v>496</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>507</v>
+        <v>497</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>508</v>
+        <v>498</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>509</v>
+        <v>499</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>510</v>
+        <v>500</v>
       </c>
       <c r="I14" s="12" t="s">
-        <v>511</v>
+        <v>501</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="K14" s="12" t="s">
-        <v>513</v>
+        <v>503</v>
       </c>
       <c r="L14" s="12"/>
       <c r="M14" s="12"/>
       <c r="N14" s="12"/>
       <c r="O14" s="12" t="s">
-        <v>514</v>
+        <v>504</v>
       </c>
       <c r="P14" s="12"/>
     </row>
@@ -5351,38 +5373,38 @@
         <v>5</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C15" s="13">
         <v>3</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>515</v>
+        <v>505</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>516</v>
+        <v>506</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>517</v>
+        <v>507</v>
       </c>
       <c r="G15" s="13"/>
       <c r="H15" s="13" t="s">
-        <v>518</v>
+        <v>508</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>519</v>
+        <v>509</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>520</v>
+        <v>510</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>521</v>
+        <v>511</v>
       </c>
       <c r="L15" s="13"/>
       <c r="M15" s="13"/>
       <c r="N15" s="13"/>
       <c r="O15" s="13" t="s">
-        <v>522</v>
+        <v>512</v>
       </c>
       <c r="P15" s="13"/>
     </row>
@@ -5391,44 +5413,44 @@
         <v>6</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C16" s="12">
         <v>1</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>523</v>
+        <v>513</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>524</v>
+        <v>514</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>525</v>
+        <v>515</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>526</v>
+        <v>516</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>527</v>
+        <v>517</v>
       </c>
       <c r="I16" s="12" t="s">
-        <v>528</v>
+        <v>518</v>
       </c>
       <c r="J16" s="12"/>
       <c r="K16" s="12" t="s">
-        <v>529</v>
+        <v>519</v>
       </c>
       <c r="L16" s="12" t="s">
-        <v>530</v>
+        <v>520</v>
       </c>
       <c r="M16" s="12" t="s">
-        <v>531</v>
+        <v>521</v>
       </c>
       <c r="N16" s="12" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="O16" s="12" t="s">
-        <v>533</v>
+        <v>523</v>
       </c>
       <c r="P16" s="12"/>
     </row>
@@ -5437,25 +5459,25 @@
         <v>6</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C17" s="13">
         <v>2</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>534</v>
+        <v>524</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>535</v>
+        <v>525</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>536</v>
+        <v>526</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>537</v>
+        <v>527</v>
       </c>
       <c r="I17" s="13"/>
       <c r="J17" s="13"/>
@@ -5464,7 +5486,7 @@
       <c r="M17" s="13"/>
       <c r="N17" s="13"/>
       <c r="O17" s="13" t="s">
-        <v>538</v>
+        <v>528</v>
       </c>
       <c r="P17" s="13"/>
     </row>
@@ -5473,46 +5495,46 @@
         <v>6</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C18" s="12">
         <v>3</v>
       </c>
       <c r="D18" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>531</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>532</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>533</v>
+      </c>
+      <c r="I18" s="12" t="s">
+        <v>534</v>
+      </c>
+      <c r="J18" s="12" t="s">
+        <v>535</v>
+      </c>
+      <c r="K18" s="12" t="s">
+        <v>536</v>
+      </c>
+      <c r="L18" s="12" t="s">
+        <v>537</v>
+      </c>
+      <c r="M18" s="12" t="s">
+        <v>538</v>
+      </c>
+      <c r="N18" s="12" t="s">
         <v>539</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="O18" s="12" t="s">
         <v>540</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>541</v>
-      </c>
-      <c r="G18" s="12" t="s">
-        <v>542</v>
-      </c>
-      <c r="H18" s="12" t="s">
-        <v>543</v>
-      </c>
-      <c r="I18" s="12" t="s">
-        <v>544</v>
-      </c>
-      <c r="J18" s="12" t="s">
-        <v>545</v>
-      </c>
-      <c r="K18" s="12" t="s">
-        <v>546</v>
-      </c>
-      <c r="L18" s="12" t="s">
-        <v>547</v>
-      </c>
-      <c r="M18" s="12" t="s">
-        <v>548</v>
-      </c>
-      <c r="N18" s="12" t="s">
-        <v>549</v>
-      </c>
-      <c r="O18" s="12" t="s">
-        <v>550</v>
       </c>
       <c r="P18" s="12"/>
     </row>
@@ -5521,46 +5543,46 @@
         <v>7</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C19" s="13">
         <v>1</v>
       </c>
       <c r="D19" s="13" t="s">
+        <v>541</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>542</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>543</v>
+      </c>
+      <c r="G19" s="13" t="s">
+        <v>544</v>
+      </c>
+      <c r="H19" s="13" t="s">
+        <v>545</v>
+      </c>
+      <c r="I19" s="13" t="s">
+        <v>546</v>
+      </c>
+      <c r="J19" s="13" t="s">
+        <v>547</v>
+      </c>
+      <c r="K19" s="13" t="s">
+        <v>548</v>
+      </c>
+      <c r="L19" s="13" t="s">
+        <v>549</v>
+      </c>
+      <c r="M19" s="13" t="s">
+        <v>550</v>
+      </c>
+      <c r="N19" s="13" t="s">
         <v>551</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="O19" s="13" t="s">
         <v>552</v>
-      </c>
-      <c r="F19" s="13" t="s">
-        <v>553</v>
-      </c>
-      <c r="G19" s="13" t="s">
-        <v>554</v>
-      </c>
-      <c r="H19" s="13" t="s">
-        <v>555</v>
-      </c>
-      <c r="I19" s="13" t="s">
-        <v>556</v>
-      </c>
-      <c r="J19" s="13" t="s">
-        <v>557</v>
-      </c>
-      <c r="K19" s="13" t="s">
-        <v>558</v>
-      </c>
-      <c r="L19" s="13" t="s">
-        <v>559</v>
-      </c>
-      <c r="M19" s="13" t="s">
-        <v>560</v>
-      </c>
-      <c r="N19" s="13" t="s">
-        <v>561</v>
-      </c>
-      <c r="O19" s="13" t="s">
-        <v>562</v>
       </c>
       <c r="P19" s="13"/>
     </row>
@@ -5569,38 +5591,38 @@
         <v>7</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C20" s="12">
         <v>2</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>563</v>
+        <v>553</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>564</v>
+        <v>554</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>565</v>
+        <v>555</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>566</v>
+        <v>556</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>567</v>
+        <v>557</v>
       </c>
       <c r="I20" s="12" t="s">
-        <v>568</v>
+        <v>558</v>
       </c>
       <c r="J20" s="12"/>
       <c r="K20" s="12" t="s">
-        <v>569</v>
+        <v>559</v>
       </c>
       <c r="L20" s="12"/>
       <c r="M20" s="12"/>
       <c r="N20" s="12"/>
       <c r="O20" s="12" t="s">
-        <v>570</v>
+        <v>560</v>
       </c>
       <c r="P20" s="12"/>
     </row>
@@ -5609,40 +5631,40 @@
         <v>7</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C21" s="13">
         <v>3</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>571</v>
+        <v>561</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>572</v>
+        <v>562</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>573</v>
+        <v>563</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>574</v>
+        <v>564</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>575</v>
+        <v>565</v>
       </c>
       <c r="I21" s="13" t="s">
-        <v>576</v>
+        <v>566</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>577</v>
+        <v>567</v>
       </c>
       <c r="K21" s="13" t="s">
-        <v>578</v>
+        <v>568</v>
       </c>
       <c r="L21" s="13"/>
       <c r="M21" s="13"/>
       <c r="N21" s="13"/>
       <c r="O21" s="13" t="s">
-        <v>579</v>
+        <v>569</v>
       </c>
       <c r="P21" s="13"/>
     </row>
@@ -5651,25 +5673,25 @@
         <v>7</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C22" s="12">
         <v>4</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>580</v>
+        <v>570</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>581</v>
+        <v>571</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>582</v>
+        <v>572</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>583</v>
+        <v>573</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>584</v>
+        <v>574</v>
       </c>
       <c r="I22" s="12"/>
       <c r="J22" s="12"/>
@@ -5678,7 +5700,7 @@
       <c r="M22" s="12"/>
       <c r="N22" s="12"/>
       <c r="O22" s="12" t="s">
-        <v>585</v>
+        <v>575</v>
       </c>
       <c r="P22" s="12"/>
     </row>
@@ -5687,40 +5709,40 @@
         <v>8</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="C23" s="13">
         <v>1</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>588</v>
+        <v>578</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>589</v>
+        <v>579</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>590</v>
+        <v>580</v>
       </c>
       <c r="I23" s="13" t="s">
-        <v>591</v>
+        <v>581</v>
       </c>
       <c r="J23" s="13" t="s">
-        <v>592</v>
+        <v>582</v>
       </c>
       <c r="K23" s="13" t="s">
-        <v>593</v>
+        <v>583</v>
       </c>
       <c r="L23" s="13"/>
       <c r="M23" s="13"/>
       <c r="N23" s="13"/>
       <c r="O23" s="13" t="s">
-        <v>594</v>
+        <v>584</v>
       </c>
       <c r="P23" s="13"/>
     </row>
@@ -5729,46 +5751,46 @@
         <v>8</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="C24" s="12">
         <v>2</v>
       </c>
       <c r="D24" s="12" t="s">
+        <v>585</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>586</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>587</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>588</v>
+      </c>
+      <c r="H24" s="12" t="s">
+        <v>589</v>
+      </c>
+      <c r="I24" s="12" t="s">
+        <v>590</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>591</v>
+      </c>
+      <c r="K24" s="12" t="s">
+        <v>592</v>
+      </c>
+      <c r="L24" s="12" t="s">
+        <v>593</v>
+      </c>
+      <c r="M24" s="12" t="s">
+        <v>594</v>
+      </c>
+      <c r="N24" s="12" t="s">
         <v>595</v>
       </c>
-      <c r="E24" s="12" t="s">
+      <c r="O24" s="12" t="s">
         <v>596</v>
-      </c>
-      <c r="F24" s="12" t="s">
-        <v>597</v>
-      </c>
-      <c r="G24" s="12" t="s">
-        <v>598</v>
-      </c>
-      <c r="H24" s="12" t="s">
-        <v>599</v>
-      </c>
-      <c r="I24" s="12" t="s">
-        <v>600</v>
-      </c>
-      <c r="J24" s="12" t="s">
-        <v>601</v>
-      </c>
-      <c r="K24" s="12" t="s">
-        <v>602</v>
-      </c>
-      <c r="L24" s="12" t="s">
-        <v>603</v>
-      </c>
-      <c r="M24" s="12" t="s">
-        <v>604</v>
-      </c>
-      <c r="N24" s="12" t="s">
-        <v>605</v>
-      </c>
-      <c r="O24" s="12" t="s">
-        <v>606</v>
       </c>
       <c r="P24" s="12"/>
     </row>
@@ -5777,25 +5799,25 @@
         <v>8</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="C25" s="13">
         <v>3</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>607</v>
+        <v>597</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>608</v>
+        <v>598</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>609</v>
+        <v>599</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>610</v>
+        <v>600</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>611</v>
+        <v>601</v>
       </c>
       <c r="I25" s="13"/>
       <c r="J25" s="13"/>
@@ -5804,7 +5826,7 @@
       <c r="M25" s="13"/>
       <c r="N25" s="13"/>
       <c r="O25" s="13" t="s">
-        <v>612</v>
+        <v>602</v>
       </c>
       <c r="P25" s="13"/>
     </row>
@@ -5813,46 +5835,46 @@
         <v>9</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="C26" s="12">
         <v>1</v>
       </c>
       <c r="D26" s="12" t="s">
+        <v>603</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>604</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>605</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>606</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>607</v>
+      </c>
+      <c r="I26" s="12" t="s">
+        <v>608</v>
+      </c>
+      <c r="J26" s="12" t="s">
+        <v>609</v>
+      </c>
+      <c r="K26" s="12" t="s">
+        <v>610</v>
+      </c>
+      <c r="L26" s="12" t="s">
+        <v>611</v>
+      </c>
+      <c r="M26" s="12" t="s">
+        <v>612</v>
+      </c>
+      <c r="N26" s="12" t="s">
         <v>613</v>
       </c>
-      <c r="E26" s="12" t="s">
+      <c r="O26" s="12" t="s">
         <v>614</v>
-      </c>
-      <c r="F26" s="12" t="s">
-        <v>615</v>
-      </c>
-      <c r="G26" s="12" t="s">
-        <v>616</v>
-      </c>
-      <c r="H26" s="12" t="s">
-        <v>617</v>
-      </c>
-      <c r="I26" s="12" t="s">
-        <v>618</v>
-      </c>
-      <c r="J26" s="12" t="s">
-        <v>619</v>
-      </c>
-      <c r="K26" s="12" t="s">
-        <v>620</v>
-      </c>
-      <c r="L26" s="12" t="s">
-        <v>621</v>
-      </c>
-      <c r="M26" s="12" t="s">
-        <v>622</v>
-      </c>
-      <c r="N26" s="12" t="s">
-        <v>623</v>
-      </c>
-      <c r="O26" s="12" t="s">
-        <v>624</v>
       </c>
       <c r="P26" s="12"/>
     </row>
@@ -5861,25 +5883,25 @@
         <v>9</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="C27" s="13">
         <v>2</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>625</v>
+        <v>615</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>626</v>
+        <v>616</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>627</v>
+        <v>617</v>
       </c>
       <c r="G27" s="13" t="s">
-        <v>628</v>
+        <v>618</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>629</v>
+        <v>619</v>
       </c>
       <c r="I27" s="13"/>
       <c r="J27" s="13"/>
@@ -5888,7 +5910,7 @@
       <c r="M27" s="13"/>
       <c r="N27" s="13"/>
       <c r="O27" s="13" t="s">
-        <v>630</v>
+        <v>620</v>
       </c>
       <c r="P27" s="13"/>
     </row>
@@ -5897,40 +5919,40 @@
         <v>9</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="C28" s="12">
         <v>3</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>631</v>
+        <v>621</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>632</v>
+        <v>622</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>633</v>
+        <v>623</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>634</v>
+        <v>624</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>635</v>
+        <v>625</v>
       </c>
       <c r="I28" s="12" t="s">
-        <v>636</v>
+        <v>626</v>
       </c>
       <c r="J28" s="12" t="s">
-        <v>637</v>
+        <v>627</v>
       </c>
       <c r="K28" s="12" t="s">
-        <v>638</v>
+        <v>628</v>
       </c>
       <c r="L28" s="12"/>
       <c r="M28" s="12"/>
       <c r="N28" s="12"/>
       <c r="O28" s="12" t="s">
-        <v>639</v>
+        <v>629</v>
       </c>
       <c r="P28" s="12"/>
     </row>
@@ -5939,44 +5961,44 @@
         <v>10</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="C29" s="13">
         <v>1</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>640</v>
+        <v>630</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>641</v>
+        <v>631</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>642</v>
+        <v>632</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>643</v>
+        <v>633</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>644</v>
+        <v>634</v>
       </c>
       <c r="I29" s="13" t="s">
-        <v>645</v>
+        <v>635</v>
       </c>
       <c r="J29" s="13" t="s">
-        <v>646</v>
+        <v>636</v>
       </c>
       <c r="K29" s="13" t="s">
-        <v>647</v>
+        <v>637</v>
       </c>
       <c r="L29" s="13" t="s">
-        <v>648</v>
+        <v>638</v>
       </c>
       <c r="M29" s="13"/>
       <c r="N29" s="13" t="s">
-        <v>649</v>
+        <v>639</v>
       </c>
       <c r="O29" s="13" t="s">
-        <v>650</v>
+        <v>640</v>
       </c>
       <c r="P29" s="13"/>
     </row>
@@ -5985,40 +6007,40 @@
         <v>10</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="C30" s="12">
         <v>2</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>651</v>
+        <v>641</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>652</v>
+        <v>642</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>653</v>
+        <v>643</v>
       </c>
       <c r="G30" s="12" t="s">
-        <v>654</v>
+        <v>644</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>655</v>
+        <v>645</v>
       </c>
       <c r="I30" s="12" t="s">
-        <v>656</v>
+        <v>646</v>
       </c>
       <c r="J30" s="12" t="s">
-        <v>657</v>
+        <v>647</v>
       </c>
       <c r="K30" s="12" t="s">
-        <v>658</v>
+        <v>648</v>
       </c>
       <c r="L30" s="12"/>
       <c r="M30" s="12"/>
       <c r="N30" s="12"/>
       <c r="O30" s="12" t="s">
-        <v>659</v>
+        <v>649</v>
       </c>
       <c r="P30" s="12"/>
     </row>
@@ -6027,25 +6049,25 @@
         <v>10</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="C31" s="13">
         <v>3</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>660</v>
+        <v>650</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>661</v>
+        <v>651</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>662</v>
+        <v>652</v>
       </c>
       <c r="G31" s="13" t="s">
-        <v>663</v>
+        <v>653</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>664</v>
+        <v>654</v>
       </c>
       <c r="I31" s="13"/>
       <c r="J31" s="13"/>
@@ -6054,7 +6076,7 @@
       <c r="M31" s="13"/>
       <c r="N31" s="13"/>
       <c r="O31" s="13" t="s">
-        <v>665</v>
+        <v>655</v>
       </c>
       <c r="P31" s="13"/>
     </row>
@@ -6063,44 +6085,44 @@
         <v>11</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="C32" s="12">
         <v>1</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>666</v>
+        <v>656</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>667</v>
+        <v>657</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>668</v>
+        <v>658</v>
       </c>
       <c r="G32" s="12"/>
       <c r="H32" s="12" t="s">
-        <v>669</v>
+        <v>659</v>
       </c>
       <c r="I32" s="12" t="s">
-        <v>670</v>
+        <v>660</v>
       </c>
       <c r="J32" s="12" t="s">
-        <v>671</v>
+        <v>661</v>
       </c>
       <c r="K32" s="12" t="s">
-        <v>672</v>
+        <v>662</v>
       </c>
       <c r="L32" s="12" t="s">
-        <v>673</v>
+        <v>663</v>
       </c>
       <c r="M32" s="12" t="s">
-        <v>674</v>
+        <v>664</v>
       </c>
       <c r="N32" s="12" t="s">
-        <v>675</v>
+        <v>665</v>
       </c>
       <c r="O32" s="12" t="s">
-        <v>700</v>
+        <v>690</v>
       </c>
       <c r="P32" s="12"/>
     </row>
@@ -6109,40 +6131,40 @@
         <v>11</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="C33" s="13">
         <v>2</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>676</v>
+        <v>666</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>677</v>
+        <v>667</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>701</v>
+        <v>691</v>
       </c>
       <c r="G33" s="13"/>
       <c r="H33" s="13" t="s">
-        <v>702</v>
+        <v>692</v>
       </c>
       <c r="I33" s="13" t="s">
-        <v>703</v>
+        <v>693</v>
       </c>
       <c r="J33" s="13"/>
       <c r="K33" s="13" t="s">
-        <v>704</v>
+        <v>694</v>
       </c>
       <c r="L33" s="13" t="s">
-        <v>705</v>
+        <v>695</v>
       </c>
       <c r="M33" s="13"/>
       <c r="N33" s="13" t="s">
-        <v>706</v>
+        <v>696</v>
       </c>
       <c r="O33" s="13" t="s">
-        <v>707</v>
+        <v>697</v>
       </c>
       <c r="P33" s="13"/>
     </row>
@@ -6151,40 +6173,40 @@
         <v>11</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="C34" s="12">
         <v>3</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>678</v>
+        <v>668</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>679</v>
+        <v>669</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>708</v>
+        <v>698</v>
       </c>
       <c r="G34" s="12"/>
       <c r="H34" s="12" t="s">
-        <v>709</v>
+        <v>699</v>
       </c>
       <c r="I34" s="12" t="s">
-        <v>710</v>
+        <v>700</v>
       </c>
       <c r="J34" s="12"/>
       <c r="K34" s="12" t="s">
-        <v>711</v>
+        <v>701</v>
       </c>
       <c r="L34" s="12" t="s">
-        <v>712</v>
+        <v>702</v>
       </c>
       <c r="M34" s="12"/>
       <c r="N34" s="12" t="s">
-        <v>713</v>
+        <v>703</v>
       </c>
       <c r="O34" s="12" t="s">
-        <v>714</v>
+        <v>704</v>
       </c>
       <c r="P34" s="12"/>
     </row>
@@ -6212,13 +6234,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>680</v>
+        <v>670</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>681</v>
+        <v>671</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>682</v>
+        <v>672</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -6226,10 +6248,10 @@
         <v>2</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>683</v>
+        <v>673</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>684</v>
+        <v>674</v>
       </c>
       <c r="D2" s="12"/>
     </row>
@@ -6238,10 +6260,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>685</v>
+        <v>675</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>686</v>
+        <v>676</v>
       </c>
       <c r="D3" s="13"/>
     </row>

</xml_diff>

<commit_message>
Add Second Half of the OT Overview (Sessions 13–22)
Content (workbook → generated overlay):
- Merge Sessions 13–22 and their 33 divisions into the Data Entry master,
  built from the actual study docs/slides. Sessions 1–12 untouched.
- Division suggested answers trimmed to 1–2 sentences to match 1–12 style.
- Regenerate assets/js/content-overrides.js (22 sessions, 66 divisions).

Site wiring:
- data.js: register sessions 13–22 in OT_SESSIONS (+ image fallbacks);
  content comes from the workbook overlay.
- 05-app.js: Pentateuch pages (Intro/Big Picture/Matrix) keep sessions 1–12
  only, so they render exactly as before; Home + Recap Mode get all 22.
  Home hero now references the Second Half.
- 04-recap.js: add a "The Second Half — Part 2" picker group (Sessions 13–22);
  keep Session 12's embedded Pentateuch view scoped to 1–12.

Saved-answer behaviour and the 1–12 experience are unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RECAP MODE - Data Entry USE THIS v9 (synced).xlsx
+++ b/RECAP MODE - Data Entry USE THIS v9 (synced).xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sessions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Division Questions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Further Study" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Division Questions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Further Study" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -186,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -253,6 +253,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -677,7 +680,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -753,7 +755,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -1009,7 +1010,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
@@ -1053,7 +1053,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
@@ -1109,7 +1108,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
@@ -1165,7 +1163,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
@@ -1257,7 +1254,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
@@ -1320,7 +1316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO13"/>
+  <dimension ref="A1:AO23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.5"/>
   <cols>
     <col width="8" customWidth="1" style="22" min="1" max="1"/>
@@ -3506,6 +3502,1809 @@
       <c r="AN13" s="19" t="n"/>
       <c r="AO13" s="19" t="n"/>
     </row>
+    <row r="14">
+      <c r="A14" s="24" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>Judges</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>The Need for a King</t>
+        </is>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>Israel had God’s law, God’s land, and God-raised judges — so why did they keep spiralling back into sin?</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t>Because the problem was never just their circumstances — it was their hearts. The judges brought only temporary rescue, then died and the cycle repeated. Israel needed more than a deliverer for a moment; they needed a righteous King, chosen by God, who fears God and keeps His law — pointing forward to Jesus.</t>
+        </is>
+      </c>
+      <c r="G14" s="24" t="inlineStr">
+        <is>
+          <t>Context: After Moses (Deuteronomy) and Joshua, Israel has entered Canaan but has not fully driven out the nations. Judges 1 and 2 give parallel accounts — chapter 1 a factual record of the incomplete conquest, chapter 2 the spiritual interpretation. Notice the downward spiral, and watch how the book ends craving a king.</t>
+        </is>
+      </c>
+      <c r="H14" s="24" t="inlineStr">
+        <is>
+          <t>Judges 1 | The Failure of the Military Conquest
+Judges 2 | The Spiritual Failure &amp; the Cycle
+1 Samuel 8; 13:14; Deuteronomy 17:14-20 | The Need for a Righteous King</t>
+        </is>
+      </c>
+      <c r="I14" s="24" t="inlineStr">
+        <is>
+          <t>God’s people keep disobeying Him even under the judges; a better and lasting solution is needed — a righteous King who points them back to God.</t>
+        </is>
+      </c>
+      <c r="J14" s="24" t="inlineStr">
+        <is>
+          <t>Judges 21:25 — In those days there was no king in Israel. Everyone did what was right in his own eyes.</t>
+        </is>
+      </c>
+      <c r="K14" s="24" t="inlineStr">
+        <is>
+          <t>Under the judges, Israel abandons God’s **kingdom order** — ‘everyone did what was right in his own eyes’ (Judges 21:25) — and even begins to lose the land God had given them.</t>
+        </is>
+      </c>
+      <c r="L14" s="24" t="inlineStr">
+        <is>
+          <t>When His people cry out, God repeatedly **raises up judges to rescue** them — yet the rescue is only temporary: the judges die and the cycle repeats.</t>
+        </is>
+      </c>
+      <c r="M14" s="24" t="inlineStr">
+        <is>
+          <t>The failure of the judges sharpens the hope for God’s **promise of a righteous King**, chosen by God, who fears Him and keeps His law (Deut 17; 1 Sam 13:14).</t>
+        </is>
+      </c>
+      <c r="N14" s="24" t="inlineStr">
+        <is>
+          <t>God is patient and merciful — He keeps raising rescuers for a people who keep rebelling — and He is working toward a lasting solution: a righteous King after His own heart.</t>
+        </is>
+      </c>
+      <c r="O14" s="24" t="inlineStr">
+        <is>
+          <t>Israel’s problem is not their circumstances but their hearts. Even when rescued, they will not listen (Judges 2:17); they choose disobedience and spiral downward, becoming like the nations around them.</t>
+        </is>
+      </c>
+      <c r="P14" s="24" t="inlineStr">
+        <is>
+          <t>Acts 5:29-32; Acts 13:22-23</t>
+        </is>
+      </c>
+      <c r="Q14" s="24" t="inlineStr">
+        <is>
+          <t>God raised up Jesus as Leader and Saviour — the truly righteous King after God’s own heart, perfectly obedient, who deals with the heart problem the judges never could.</t>
+        </is>
+      </c>
+      <c r="R14" s="24" t="inlineStr">
+        <is>
+          <t>What does Judges add to your understanding of sin and the human heart?</t>
+        </is>
+      </c>
+      <c r="S14" s="24" t="inlineStr">
+        <is>
+          <t>How might a righteous Leader and Saviour — not just better circumstances — be the solution to a sinful heart?</t>
+        </is>
+      </c>
+      <c r="T14" s="24" t="inlineStr">
+        <is>
+          <t>How do the judges and the cry for a king show us our need for Jesus as Leader and Saviour?</t>
+        </is>
+      </c>
+      <c r="U14" s="24" t="inlineStr">
+        <is>
+          <t>king</t>
+        </is>
+      </c>
+      <c r="V14" s="24" t="inlineStr">
+        <is>
+          <t>Judges ends with a cry: there was no ___ in Israel, and everyone did what was right in his own eyes.</t>
+        </is>
+      </c>
+      <c r="W14" s="24" t="inlineStr">
+        <is>
+          <t>Jesus</t>
+        </is>
+      </c>
+      <c r="X14" s="24" t="inlineStr">
+        <is>
+          <t>Acts 5 — God raised up ___ as Leader and Saviour, the righteous King.</t>
+        </is>
+      </c>
+      <c r="Y14" s="24" t="inlineStr"/>
+      <c r="Z14" s="24" t="inlineStr">
+        <is>
+          <t>Kingdom</t>
+        </is>
+      </c>
+      <c r="AA14" s="24" t="inlineStr">
+        <is>
+          <t>• Judges 1 and 2 are parallel accounts of the same period (note Joshua’s death in 1:1 and 2:8): ch.1 records the military failure, ch.2 interprets it spiritually.
+• Land connects back to the Abrahamic promise — losing it is the covenant blessing going into reverse.</t>
+        </is>
+      </c>
+      <c r="AB14" s="24" t="inlineStr">
+        <is>
+          <t>Pray that God would show us the depth of our own heart’s rebellion, and give us fresh love for Jesus, our righteous King and Saviour.</t>
+        </is>
+      </c>
+      <c r="AC14" s="24" t="inlineStr">
+        <is>
+          <t>As you reflect on The Need for a King (Judges 1-2), what does this passage reveal about God’s character that you can praise Him for?</t>
+        </is>
+      </c>
+      <c r="AD14" s="24" t="inlineStr">
+        <is>
+          <t>In light of what you’ve studied, where have you fallen short of God’s design? Where have you resisted His good rule?</t>
+        </is>
+      </c>
+      <c r="AE14" s="24" t="inlineStr">
+        <is>
+          <t>What can you thank God for in light of this passage — especially how Christ fulfils what you’ve studied?</t>
+        </is>
+      </c>
+      <c r="AF14" s="24" t="inlineStr">
+        <is>
+          <t>What do you need from God as you apply this truth to your life this week?</t>
+        </is>
+      </c>
+      <c r="AG14" s="24" t="inlineStr"/>
+      <c r="AH14" s="24" t="inlineStr"/>
+      <c r="AI14" s="24" t="inlineStr"/>
+      <c r="AJ14" s="24" t="inlineStr"/>
+      <c r="AK14" s="24" t="inlineStr"/>
+      <c r="AL14" s="24" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="AM14" s="24" t="inlineStr"/>
+      <c r="AN14" s="24" t="inlineStr">
+        <is>
+          <t>Where do you see the pattern of Judges — rebellion, temporary rescue, then drifting back — in your own heart?</t>
+        </is>
+      </c>
+      <c r="AO14" s="24" t="inlineStr">
+        <is>
+          <t>Jesus is the righteous King who obeyed perfectly and saves us. Pause and thank Him for being the Leader your heart most needs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="24" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>2 Samuel</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>Davidic Covenant</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>Israel wanted a king ‘like the nations’. What kind of king does the Lord actually want — and what makes David different from Saul?</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>God wants a king who is His own sovereign choice, who sees himself as God’s servant, fears Him and loves His house. Against this, God makes a covenant with David: not that David will build God a house, but that God will build David a ‘house’ — an everlasting dynasty and kingdom, established by God’s own faithfulness, not the king’s.</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="inlineStr">
+        <is>
+          <t>Context: After the spiral of Judges and the failure of Saul (who would not obey God), we come to David. The passage falls into two halves: God’s promise to David (v.1-17) and David’s response of prayer (v.18-29). Notice how often God says ‘I will’, and how often David calls himself ‘your servant’.</t>
+        </is>
+      </c>
+      <c r="H15" s="24" t="inlineStr">
+        <is>
+          <t>Deuteronomy 17:14-20; 1 Samuel 8; 13; 15 | The king the Lord wants (recap)
+2 Samuel 7:1-17 | God’s promise to David
+2 Samuel 7:18-29 | David’s response</t>
+        </is>
+      </c>
+      <c r="I15" s="24" t="inlineStr">
+        <is>
+          <t>The faithful God will Himself establish an everlasting kingdom through the line of David, God’s chosen servant-king — a kingdom that brings ultimate peace to His people.</t>
+        </is>
+      </c>
+      <c r="J15" s="24" t="inlineStr">
+        <is>
+          <t>2 Samuel 7:16 — And your house and your kingdom shall be made sure forever before me. Your throne shall be established forever.</t>
+        </is>
+      </c>
+      <c r="K15" s="24" t="inlineStr">
+        <is>
+          <t>God promises to establish David’s **throne and kingdom forever** (v.16) — not a kingdom that depends on the king, but one secured by God Himself.</t>
+        </is>
+      </c>
+      <c r="L15" s="24" t="inlineStr">
+        <is>
+          <t>God gives His people **rest from their enemies** and a king who serves Him — a foretaste of the ultimate peace His forever-kingdom will bring.</t>
+        </is>
+      </c>
+      <c r="M15" s="24" t="inlineStr">
+        <is>
+          <t>The **Davidic Covenant**: God’s repeated ‘I will’ — a great name, a place for His people, and an offspring whose kingdom endures forever (echoing the Abrahamic promise that all nations will be blessed).</t>
+        </is>
+      </c>
+      <c r="N15" s="24" t="inlineStr">
+        <is>
+          <t>God is the faithful promise-keeper who Himself establishes His kingdom. He chooses and delights in a king who is His servant, and binds the future of all nations to this covenant.</t>
+        </is>
+      </c>
+      <c r="O15" s="24" t="inlineStr">
+        <is>
+          <t>Even David, the king after God’s own heart, is not the forever-king — he will die, and later kings will fail. The covenant’s certainty rests on God’s faithfulness, not the king’s.</t>
+        </is>
+      </c>
+      <c r="P15" s="24" t="inlineStr">
+        <is>
+          <t>John 2:13-22; Luke 1:32-33</t>
+        </is>
+      </c>
+      <c r="Q15" s="24" t="inlineStr">
+        <is>
+          <t>Jesus is the promised offspring of David — the servant-King who honours God and loves His Father’s house — whose kingdom truly lasts forever.</t>
+        </is>
+      </c>
+      <c r="R15" s="24" t="inlineStr">
+        <is>
+          <t>How have you seen Jesus to be the true Davidic King — the one who honours God and loves His house?</t>
+        </is>
+      </c>
+      <c r="S15" s="24" t="inlineStr">
+        <is>
+          <t>Think of the person you’d most willingly follow. How does Jesus, as God’s chosen King, compare?</t>
+        </is>
+      </c>
+      <c r="T15" s="24" t="inlineStr">
+        <is>
+          <t>Why does it matter to you, as a Christian today, that you have such a King? What are you grateful for as you think of Him?</t>
+        </is>
+      </c>
+      <c r="U15" s="24" t="inlineStr">
+        <is>
+          <t>forever</t>
+        </is>
+      </c>
+      <c r="V15" s="24" t="inlineStr">
+        <is>
+          <t>2 Samuel 7 — God promises that David’s throne and kingdom will be established ___.</t>
+        </is>
+      </c>
+      <c r="W15" s="24" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="X15" s="24" t="inlineStr">
+        <is>
+          <t>John 2 — Jesus is the promised offspring of ___, the servant-King who loves His Father’s house.</t>
+        </is>
+      </c>
+      <c r="Y15" s="24" t="inlineStr"/>
+      <c r="Z15" s="24" t="inlineStr">
+        <is>
+          <t>Promises</t>
+        </is>
+      </c>
+      <c r="AA15" s="24" t="inlineStr">
+        <is>
+          <t>• Play up the repeated ‘I will’ (God) versus ‘your servant’ (David): the kingdom’s security rests on God, and the king God wants is a servant.
+• Feedback from the study team: let the group sit with the OT picture of the king before jumping to Jesus; keep the ‘house = God’s people’ idea as an optional deeper layer.</t>
+        </is>
+      </c>
+      <c r="AB15" s="24" t="inlineStr">
+        <is>
+          <t>Pray that we would adore King Jesus more — the faithful, servant-hearted King God promised — and rest in the certainty of His forever-kingdom.</t>
+        </is>
+      </c>
+      <c r="AC15" s="24" t="inlineStr">
+        <is>
+          <t>As you reflect on the Davidic Covenant (2 Samuel 7), what does this passage reveal about God’s character that you can praise Him for?</t>
+        </is>
+      </c>
+      <c r="AD15" s="24" t="inlineStr">
+        <is>
+          <t>In light of what you’ve studied, where have you fallen short of God’s design? Where have you resisted His good rule?</t>
+        </is>
+      </c>
+      <c r="AE15" s="24" t="inlineStr">
+        <is>
+          <t>What can you thank God for in light of this passage — especially how Christ fulfils what you’ve studied?</t>
+        </is>
+      </c>
+      <c r="AF15" s="24" t="inlineStr">
+        <is>
+          <t>What do you need from God as you apply this truth to your life this week?</t>
+        </is>
+      </c>
+      <c r="AG15" s="24" t="inlineStr"/>
+      <c r="AH15" s="24" t="inlineStr"/>
+      <c r="AI15" s="24" t="inlineStr"/>
+      <c r="AJ15" s="24" t="inlineStr"/>
+      <c r="AK15" s="24" t="inlineStr"/>
+      <c r="AL15" s="24" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="AM15" s="24" t="inlineStr"/>
+      <c r="AN15" s="24" t="inlineStr">
+        <is>
+          <t>God’s ‘I will’ secures the kingdom, not the king’s performance. Where do you need to rest in God’s faithfulness rather than your own?</t>
+        </is>
+      </c>
+      <c r="AO15" s="24" t="inlineStr">
+        <is>
+          <t>How does Jesus compare with the kind of leader you’d most want to follow? Sit with what you’re grateful for in Him as your King.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>1 Kings</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>The Temple</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>God promised David a ‘house’. When Solomon finishes the magnificent Temple, has the promise been fulfilled — and is everything now secure?</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>God’s promise to David is genuinely fulfilled: Solomon, David’s son, builds the house and God’s glory fills it. Yet the Temple’s significance is not its grandeur but the Lord’s presence — and even at Israel’s peak, Solomon’s own prayer keeps returning to sin, forgiveness and exile. The forever-house depends on a faithfulness Solomon himself will not keep.</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="inlineStr">
+        <is>
+          <t>Context: Solomon has succeeded David and, after huge effort (1 Kings 5-6), completes the Temple. Connect back to Sinai and the Tabernacle — this is about the presence of the Lord dwelling with His people. Watch how Solomon’s dedication prayer, at the very peak of Israel’s power, is preoccupied with sin and the need for God to hear and forgive.</t>
+        </is>
+      </c>
+      <c r="H16" s="24" t="inlineStr">
+        <is>
+          <t>1 Kings 8:1-21 | A house filled with the Lord’s presence
+1 Kings 8:22-53 | A house where God hears His people
+1 Kings 8:54-66 | Solomon blesses and consecrates the house</t>
+        </is>
+      </c>
+      <c r="I16" s="24" t="inlineStr">
+        <is>
+          <t>The faithful and holy God fulfils His covenant promise to David by filling His house with His presence — yet the future of that house depends on the king’s faithfulness.</t>
+        </is>
+      </c>
+      <c r="J16" s="24" t="inlineStr">
+        <is>
+          <t>1 Kings 8:56 — Blessed be the Lord who has given rest to his people Israel, according to all that he promised. Not one word has failed of all his good promise, which he spoke by Moses his servant.</t>
+        </is>
+      </c>
+      <c r="K16" s="24" t="inlineStr">
+        <is>
+          <t>God’s **glory fills the Temple** (v.10-11) — the King of the universe comes to dwell in the midst of His people, the goal of His kingdom since Eden and Sinai.</t>
+        </is>
+      </c>
+      <c r="L16" s="24" t="inlineStr">
+        <is>
+          <t>The house is where God **hears and forgives** His people when they pray toward it — Solomon’s prayer already anticipates sin, defeat and even exile, and pleads for mercy.</t>
+        </is>
+      </c>
+      <c r="M16" s="24" t="inlineStr">
+        <is>
+          <t>God has **kept His promise** to David: ‘Not one word has failed of all his good promise’ (v.56). The son of David has built the house for the Lord’s name.</t>
+        </is>
+      </c>
+      <c r="N16" s="24" t="inlineStr">
+        <is>
+          <t>God is faithful and holy — He keeps every word of His promise and comes to dwell with His people, while remaining so holy that heaven itself cannot contain Him.</t>
+        </is>
+      </c>
+      <c r="O16" s="24" t="inlineStr">
+        <is>
+          <t>Even at Israel’s peak the problem of sin remains: ‘there is no one who does not sin’ (v.46). The builder-king Solomon is fallible and will later turn from the Lord (1 Kings 11); the physical Temple cannot be the forever-house.</t>
+        </is>
+      </c>
+      <c r="P16" s="24" t="inlineStr">
+        <is>
+          <t>Hebrews 3:1-6; Ephesians 2:22</t>
+        </is>
+      </c>
+      <c r="Q16" s="24" t="inlineStr">
+        <is>
+          <t>Jesus is the faithful Son over God’s house — greater than Moses and Solomon, the perfect priest-King — and by His Spirit we ourselves become the house where God dwells.</t>
+        </is>
+      </c>
+      <c r="R16" s="24" t="inlineStr">
+        <is>
+          <t>How does seeing God keep every word of His promise to David move your heart to trust Him?</t>
+        </is>
+      </c>
+      <c r="S16" s="24" t="inlineStr">
+        <is>
+          <t>Solomon’s prayer keeps returning to sin and forgiveness. How does that deepen your longing for the perfect priest-King, Jesus?</t>
+        </is>
+      </c>
+      <c r="T16" s="24" t="inlineStr">
+        <is>
+          <t>Jesus is faithful over God’s house as a Son, and by His Spirit we are that house (Eph 2:22). How does that shape how you live this week?</t>
+        </is>
+      </c>
+      <c r="U16" s="24" t="inlineStr">
+        <is>
+          <t>glory</t>
+        </is>
+      </c>
+      <c r="V16" s="24" t="inlineStr">
+        <is>
+          <t>The Temple’s significance is not its grandeur but the Lord’s ___ filling it.</t>
+        </is>
+      </c>
+      <c r="W16" s="24" t="inlineStr">
+        <is>
+          <t>Son</t>
+        </is>
+      </c>
+      <c r="X16" s="24" t="inlineStr">
+        <is>
+          <t>Hebrews 3 — Christ is faithful over God’s house as a ___.</t>
+        </is>
+      </c>
+      <c r="Y16" s="24" t="inlineStr"/>
+      <c r="Z16" s="24" t="inlineStr">
+        <is>
+          <t>Promises</t>
+        </is>
+      </c>
+      <c r="AA16" s="24" t="inlineStr">
+        <is>
+          <t>• The point of the Temple is presence, not architecture — tie back to Sinai and the Tabernacle (the Sinai-vs-Tabernacle picture used earlier in the series).
+• Response song used in the study: ‘O Come, O Come, Emmanuel’ (Sovereign Grace Music) — note it covers more than the Incarnation.</t>
+        </is>
+      </c>
+      <c r="AB16" s="24" t="inlineStr">
+        <is>
+          <t>Pray that we would treasure God’s faithful presence with us, and appreciate Jesus, the perfect priest-King who makes us God’s dwelling place.</t>
+        </is>
+      </c>
+      <c r="AC16" s="24" t="inlineStr">
+        <is>
+          <t>As you reflect on the Temple (1 Kings 8), what does this passage reveal about God’s character that you can praise Him for?</t>
+        </is>
+      </c>
+      <c r="AD16" s="24" t="inlineStr">
+        <is>
+          <t>In light of what you’ve studied, where have you fallen short of God’s design? Where have you resisted His good rule?</t>
+        </is>
+      </c>
+      <c r="AE16" s="24" t="inlineStr">
+        <is>
+          <t>What can you thank God for in light of this passage — especially how Christ fulfils what you’ve studied?</t>
+        </is>
+      </c>
+      <c r="AF16" s="24" t="inlineStr">
+        <is>
+          <t>What do you need from God as you apply this truth to your life this week?</t>
+        </is>
+      </c>
+      <c r="AG16" s="24" t="inlineStr"/>
+      <c r="AH16" s="24" t="inlineStr"/>
+      <c r="AI16" s="24" t="inlineStr"/>
+      <c r="AJ16" s="24" t="inlineStr"/>
+      <c r="AK16" s="24" t="inlineStr"/>
+      <c r="AL16" s="24" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="AM16" s="24" t="inlineStr"/>
+      <c r="AN16" s="24" t="inlineStr">
+        <is>
+          <t>God kept every word of His promise to David. Where are you tempted to doubt God’s faithfulness — and how does Solomon’s prayer reassure you?</t>
+        </is>
+      </c>
+      <c r="AO16" s="24" t="inlineStr">
+        <is>
+          <t>By His Spirit, you are the house where God dwells. Sit with that privilege and thank Jesus, the faithful Son over God’s house.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>8-11</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>The Glory Departs</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>If God’s glory once filled Solomon’s Temple, what would have to go so wrong for that glory to leave it?</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t>Israel filled God’s own Temple with idols — breaking His commandments in His very presence. Their sinful hearts made the relationship impossible to sustain, so God justly judges them and His glory departs the Temple in stages. Yet He does not abandon His people: He follows them into exile and promises to remove their heart of stone and give them a new heart and Spirit.</t>
+        </is>
+      </c>
+      <c r="G17" s="24" t="inlineStr">
+        <is>
+          <t>Context: After the high of Solomon’s Temple, the kings and people spiral into idolatry (even Solomon’s heart turned, 1 Kings 11). Ezekiel — a priest taken into the first wave of Babylonian exile — receives visions five years in. Notice the escalating ‘abominations’ inside the Temple, the staged departure of God’s glory, and the surprising glimmer of hope at the end.</t>
+        </is>
+      </c>
+      <c r="H17" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel 8:1-17 | Israel turns God’s sanctuary into a house of idols
+Ezekiel 8:18-9:11 | Judgement for the abominations
+Ezekiel 10 | The glory of God leaves the temple
+Ezekiel 11 | Impending judgement — and a glimmer of hope</t>
+        </is>
+      </c>
+      <c r="I17" s="24" t="inlineStr">
+        <is>
+          <t>Israel cannot sustain their relationship with God on their own because of their sinful hearts; God justly judges their sin yet does not abandon them — He promises a new heart and spirit so they can follow Him.</t>
+        </is>
+      </c>
+      <c r="J17" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel 11:19 — And I will give them one heart, and a new spirit I will put within them. I will remove the heart of stone from their flesh and give them a heart of flesh.</t>
+        </is>
+      </c>
+      <c r="K17" s="24" t="inlineStr">
+        <is>
+          <t>Israel drives God out of His own **kingdom**: they fill the Temple — the place of His presence — with idols, so God’s glory departs in stages (Eze 10).</t>
+        </is>
+      </c>
+      <c r="L17" s="24" t="inlineStr">
+        <is>
+          <t>God does not abandon His people — He **follows them into exile** (11:16) and promises to bring back a remnant, transformed.</t>
+        </is>
+      </c>
+      <c r="M17" s="24" t="inlineStr">
+        <is>
+          <t>God promises a **new heart and a new spirit** (11:19; 36:26-27), removing the heart of stone so His people can finally love and follow Him — fulfilled when the Spirit is given (John 14-15).</t>
+        </is>
+      </c>
+      <c r="N17" s="24" t="inlineStr">
+        <is>
+          <t>God is holy and just — He will not overlook sin, even His people’s — yet He is astonishingly gracious and merciful, refusing to abandon them and promising to change them from the inside out.</t>
+        </is>
+      </c>
+      <c r="O17" s="24" t="inlineStr">
+        <is>
+          <t>Israel cannot sustain their relationship with God on their own. The problem is the heart — they worship God outwardly while practising idolatry secretly, so a mere change of circumstances will never be enough.</t>
+        </is>
+      </c>
+      <c r="P17" s="24" t="inlineStr">
+        <is>
+          <t>John 14:15-17; John 15:26; Ezekiel 36:26-27</t>
+        </is>
+      </c>
+      <c r="Q17" s="24" t="inlineStr">
+        <is>
+          <t>The new heart and Spirit Ezekiel promised are given to us in Christ: the Holy Spirit now dwells in believers, guiding us to love and follow God.</t>
+        </is>
+      </c>
+      <c r="R17" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel 8 shows people worshipping God publicly while serving idols privately. Where is there a gap between the Christian life you present and the life you actually live?</t>
+        </is>
+      </c>
+      <c r="S17" s="24" t="inlineStr">
+        <is>
+          <t>If the Holy Spirit were increasingly shaping your heart, what would become noticeably different about how you live?</t>
+        </is>
+      </c>
+      <c r="T17" s="24" t="inlineStr">
+        <is>
+          <t>How does the promise of a new heart and Spirit move you to thank God for the Spirit within you?</t>
+        </is>
+      </c>
+      <c r="U17" s="24" t="inlineStr">
+        <is>
+          <t>heart</t>
+        </is>
+      </c>
+      <c r="V17" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel 11 — God promises to remove the heart of stone and give a new ___ and spirit.</t>
+        </is>
+      </c>
+      <c r="W17" s="24" t="inlineStr">
+        <is>
+          <t>Spirit</t>
+        </is>
+      </c>
+      <c r="X17" s="24" t="inlineStr">
+        <is>
+          <t>John 14 — the ___ Ezekiel promised now dwells in every believer.</t>
+        </is>
+      </c>
+      <c r="Y17" s="24" t="inlineStr"/>
+      <c r="Z17" s="24" t="inlineStr">
+        <is>
+          <t>Promises</t>
+        </is>
+      </c>
+      <c r="AA17" s="24" t="inlineStr">
+        <is>
+          <t>• Intro illustration used in the study: an Airbnb guest who trashes your home, invites the very people you barred, and swaps your photos for a stranger’s — a picture of what Israel did to God’s house.
+• Let the weight of the glory departing land before reaching the hope in ch.11.</t>
+        </is>
+      </c>
+      <c r="AB17" s="24" t="inlineStr">
+        <is>
+          <t>Thank God for the Holy Spirit within us, who constantly guides us toward God; pray for hearts that love and follow Him wholly, without hidden idols.</t>
+        </is>
+      </c>
+      <c r="AC17" s="24" t="inlineStr">
+        <is>
+          <t>As you reflect on The Glory Departs (Ezekiel 8-11), what does this passage reveal about God’s character that you can praise Him for?</t>
+        </is>
+      </c>
+      <c r="AD17" s="24" t="inlineStr">
+        <is>
+          <t>In light of what you’ve studied, where have you fallen short of God’s design? Where have you resisted His good rule?</t>
+        </is>
+      </c>
+      <c r="AE17" s="24" t="inlineStr">
+        <is>
+          <t>What can you thank God for in light of this passage — especially how Christ fulfils what you’ve studied?</t>
+        </is>
+      </c>
+      <c r="AF17" s="24" t="inlineStr">
+        <is>
+          <t>What do you need from God as you apply this truth to your life this week?</t>
+        </is>
+      </c>
+      <c r="AG17" s="24" t="inlineStr"/>
+      <c r="AH17" s="24" t="inlineStr"/>
+      <c r="AI17" s="24" t="inlineStr"/>
+      <c r="AJ17" s="24" t="inlineStr"/>
+      <c r="AK17" s="24" t="inlineStr"/>
+      <c r="AL17" s="24" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="AM17" s="24" t="inlineStr"/>
+      <c r="AN17" s="24" t="inlineStr">
+        <is>
+          <t>Where might there be hidden idols in the ‘temple’ of your own heart? Bring them honestly to God.</t>
+        </is>
+      </c>
+      <c r="AO17" s="24" t="inlineStr">
+        <is>
+          <t>God has given you a new heart and His Spirit. Thank Him, and ask the Spirit to make you more like Jesus this week.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>Psalms</t>
+        </is>
+      </c>
+      <c r="C18" s="24" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="inlineStr">
+        <is>
+          <t>Clinging to the Promise</t>
+        </is>
+      </c>
+      <c r="E18" s="24" t="inlineStr">
+        <is>
+          <t>When God’s promises seem to have failed — the king defeated, the people in exile — what do you do with your disappointment and your faith?</t>
+        </is>
+      </c>
+      <c r="F18" s="24" t="inlineStr">
+        <is>
+          <t>You do what the psalmist does: you cling. Psalm 89 holds raw tension — pages of praise for God’s steadfast love and His forever-promise to David, then the brutal reality that God has judged and cast the king down. It ends not with answers but a cry: ‘How long, O Lord?’ — pleading God to remember His promises. It is the honest prayer of faith clinging to God when fulfilment feels far away.</t>
+        </is>
+      </c>
+      <c r="G18" s="24" t="inlineStr">
+        <is>
+          <t>Context: We are in the exile (cf. Ezekiel 8-11); the Davidic kingdom has collapsed. Psalms are Israel’s songs and prayers — this is Book 3 (Ps 73-89), ‘the dark book’, where God’s judgement falls on king and people and they plead His covenant. Notice the ‘Selah’ breaks that divide the psalm, and the jarring turn from praise to lament.</t>
+        </is>
+      </c>
+      <c r="H18" s="24" t="inlineStr">
+        <is>
+          <t>Psalm 89:1-4 | Praising God’s promise of an eternal kingdom to David
+Psalm 89:5-18 | Praising the God who strengthens the King
+Psalm 89:19-37 | God’s steadfast love and forever-promise to David
+Psalm 89:38-45 | God has judged His King, kingdom and people
+Psalm 89:46-52 | ‘How long, O Lord?’ — pleading the promises</t>
+        </is>
+      </c>
+      <c r="I18" s="24" t="inlineStr">
+        <is>
+          <t>In exile, with the Davidic kingdom in ruins, the psalmist clings to God’s covenant promises to David and cries out for Him to remember them and rescue His people.</t>
+        </is>
+      </c>
+      <c r="J18" s="24" t="inlineStr">
+        <is>
+          <t>Psalm 89:1 — I will sing of the steadfast love of the Lord, forever; with my mouth I will make known your faithfulness to all generations.</t>
+        </is>
+      </c>
+      <c r="K18" s="24" t="inlineStr">
+        <is>
+          <t>The psalm mourns a **kingdom in ruins** — God has cast the Davidic throne ‘to the ground’ (v.44) — yet clings to His promise that David’s throne would endure forever (v.4, 36-37).</t>
+        </is>
+      </c>
+      <c r="L18" s="24" t="inlineStr">
+        <is>
+          <t>From exile the psalmist **cries for rescue** — ‘How long, O Lord?’ (v.46) — appealing not to Israel’s merit but to God’s steadfast love of old.</t>
+        </is>
+      </c>
+      <c r="M18" s="24" t="inlineStr">
+        <is>
+          <t>The whole psalm leans on God’s **covenant promise to David** (v.3-4, 28-37) — His steadfast love and faithfulness, sworn by oath — as the one unshakeable ground of hope in the dark.</t>
+        </is>
+      </c>
+      <c r="N18" s="24" t="inlineStr">
+        <is>
+          <t>God is the maker of steadfast-love promises, faithful and true, who swears by an oath and cannot lie — even when His people cannot yet see how He will keep His word.</t>
+        </is>
+      </c>
+      <c r="O18" s="24" t="inlineStr">
+        <is>
+          <t>God’s people sit in exile under His judgement, the kingdom collapsed, feeling cast off and shamed — left clinging to promises whose fulfilment seems impossibly far away (‘How long?’).</t>
+        </is>
+      </c>
+      <c r="P18" s="24" t="inlineStr">
+        <is>
+          <t>Luke 24:44; 1 Peter 2:11-12</t>
+        </is>
+      </c>
+      <c r="Q18" s="24" t="inlineStr">
+        <is>
+          <t>Jesus is the Davidic King who truly bore being cast off, shamed and judged (Ps 89:38-45) — but His rejection led to salvation, not condemnation. He is the promise kept; and we, living as ‘exiles’ now, cling to Him until He brings us home.</t>
+        </is>
+      </c>
+      <c r="R18" s="24" t="inlineStr">
+        <is>
+          <t>Psalm 89 is a prayer for rescue in exile. How might it be a prayer for Christians living as ‘exiles’ in the world today (1 Peter 2:11-12)?</t>
+        </is>
+      </c>
+      <c r="S18" s="24" t="inlineStr">
+        <is>
+          <t>‘How long, O Lord?’ — where in your life are you waiting on God’s promises, and what helps you keep clinging rather than letting go?</t>
+        </is>
+      </c>
+      <c r="T18" s="24" t="inlineStr">
+        <is>
+          <t>How does seeing Jesus bear rejection and judgement — yet for our salvation — shape how you view your own suffering and sin?</t>
+        </is>
+      </c>
+      <c r="U18" s="24" t="inlineStr">
+        <is>
+          <t>steadfast</t>
+        </is>
+      </c>
+      <c r="V18" s="24" t="inlineStr">
+        <is>
+          <t>Psalm 89 clings to God’s ___ love and His covenant promise to David.</t>
+        </is>
+      </c>
+      <c r="W18" s="24" t="inlineStr">
+        <is>
+          <t>exiles</t>
+        </is>
+      </c>
+      <c r="X18" s="24" t="inlineStr">
+        <is>
+          <t>1 Peter 2 — we live as ___ now, clinging to the promises kept in King Jesus.</t>
+        </is>
+      </c>
+      <c r="Y18" s="24" t="inlineStr"/>
+      <c r="Z18" s="24" t="inlineStr">
+        <is>
+          <t>Promises</t>
+        </is>
+      </c>
+      <c r="AA18" s="24" t="inlineStr">
+        <is>
+          <t>• The emotional honesty is the point — Psalm 89 lets God’s people lament without pretending all is well.
+• The king judged in vv.38-45 foreshadows Jesus, but with the opposite outcome: His rejection brings salvation, not judgement (the contrast to draw in the Consolidation).</t>
+        </is>
+      </c>
+      <c r="AB18" s="24" t="inlineStr">
+        <is>
+          <t>Pray that we would cling to God’s promises in King Jesus through our own ‘exile’ — that He would show us His steadfast love in our afflictions and bring us home to His Kingdom.</t>
+        </is>
+      </c>
+      <c r="AC18" s="24" t="inlineStr">
+        <is>
+          <t>As you reflect on Clinging to the Promise (Psalm 89), what does this passage reveal about God’s character that you can praise Him for?</t>
+        </is>
+      </c>
+      <c r="AD18" s="24" t="inlineStr">
+        <is>
+          <t>In light of what you’ve studied, where have you fallen short of God’s design? Where have you resisted His good rule?</t>
+        </is>
+      </c>
+      <c r="AE18" s="24" t="inlineStr">
+        <is>
+          <t>What can you thank God for in light of this passage — especially how Christ fulfils what you’ve studied?</t>
+        </is>
+      </c>
+      <c r="AF18" s="24" t="inlineStr">
+        <is>
+          <t>What do you need from God as you apply this truth to your life this week?</t>
+        </is>
+      </c>
+      <c r="AG18" s="24" t="inlineStr"/>
+      <c r="AH18" s="24" t="inlineStr"/>
+      <c r="AI18" s="24" t="inlineStr"/>
+      <c r="AJ18" s="24" t="inlineStr"/>
+      <c r="AK18" s="24" t="inlineStr"/>
+      <c r="AL18" s="24" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="AM18" s="24" t="inlineStr"/>
+      <c r="AN18" s="24" t="inlineStr">
+        <is>
+          <t>Bring your own ‘How long, O Lord?’ honestly to God. What promise are you clinging to in the waiting?</t>
+        </is>
+      </c>
+      <c r="AO18" s="24" t="inlineStr">
+        <is>
+          <t>Jesus bore rejection and judgement for you, and rose. Sit with His steadfast love as your anchor in exile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="24" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah</t>
+        </is>
+      </c>
+      <c r="C19" s="24" t="inlineStr">
+        <is>
+          <t>9; 11; 25; 40</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="inlineStr">
+        <is>
+          <t>God’s King Who Saves</t>
+        </is>
+      </c>
+      <c r="E19" s="24" t="inlineStr">
+        <is>
+          <t>By now the Davidic king has disappointed again and again. What more could Isaiah possibly add to the ‘job description’ of the coming King — and why would it matter to you?</t>
+        </is>
+      </c>
+      <c r="F19" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah massively expands the King’s CV. This King is God Himself (Isa 9:6), permanently anointed by the Spirit (11:2), a righteous judge of the whole earth who even begins to reverse the Fall (11:6-9). And through Him God brings global, cosmic salvation: a feast for all peoples, death swallowed up forever, iniquity pardoned (Isa 25; 40). The real problem was never just exile — it is sin and death — and the answer is King Jesus.</t>
+        </is>
+      </c>
+      <c r="G19" s="24" t="inlineStr">
+        <is>
+          <t>Context: Isaiah comes BEFORE Ezekiel — we step back to before Judah’s exile (Isaiah ~740 BC onward; the northern kingdom falls to Assyria in 722 BC). Two discussions tonight: Isaiah 9 &amp; 11 (who the King is), then Isaiah 25 &amp; 40 (what God does through Him). Watch how far beyond 2 Samuel 7 this goes — and keep the surprising ‘light from Galilee’ (9:1-2) in mind.</t>
+        </is>
+      </c>
+      <c r="H19" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 9:1-7 | The King is God Himself
+Isaiah 11:1-16 | The Spirit-anointed King who renews creation
+Isaiah 25:1-12 | A feast for all peoples; death swallowed up
+Isaiah 40:1-5 | Comfort: iniquity pardoned, the Lord comes</t>
+        </is>
+      </c>
+      <c r="I19" s="24" t="inlineStr">
+        <is>
+          <t>The promised Davidic King is God Himself, Spirit-anointed to rule the whole earth; and through Him God brings a global, cosmic salvation — death swallowed up and iniquity pardoned — reaching the deepest problem of all: sin and death.</t>
+        </is>
+      </c>
+      <c r="J19" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 9:6 — For to us a child is born, to us a son is given; and the government shall be upon his shoulder, and his name shall be called Wonderful Counselor, Mighty God, Everlasting Father, Prince of Peace.</t>
+        </is>
+      </c>
+      <c r="K19" s="24" t="inlineStr">
+        <is>
+          <t>The coming King rules the **whole earth** in righteousness (11:3-4) — judge not just of Israel but of all nations — and His government and peace will have **no end** (9:7).</t>
+        </is>
+      </c>
+      <c r="L19" s="24" t="inlineStr">
+        <is>
+          <t>Through this King God brings a **global and cosmic salvation**: a feast for all peoples, **death swallowed up forever**, every tear wiped away (25:6-8), and iniquity itself pardoned (40:2).</t>
+        </is>
+      </c>
+      <c r="M19" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah expands the Davidic **promise** beyond anything in 2 Samuel 7 — the King is **God Himself** (9:6), the Spirit rests on Him permanently (11:2), and He undoes the Fall (11:6-9); ‘the zeal of the Lord of hosts will do this’ (9:7).</t>
+        </is>
+      </c>
+      <c r="N19" s="24" t="inlineStr">
+        <is>
+          <t>God is so committed to saving His people that He will come in person as the Davidic King — Mighty God, Prince of Peace — to deal with sin and death at their root, for all peoples, guaranteeing it by His own zeal.</t>
+        </is>
+      </c>
+      <c r="O19" s="24" t="inlineStr">
+        <is>
+          <t>The real problem was never merely exile but sin and death — the curse of Genesis 3 that no human king could lift. Humanity needs more than rescue from Babylon; it needs death swallowed and iniquity pardoned.</t>
+        </is>
+      </c>
+      <c r="P19" s="24" t="inlineStr">
+        <is>
+          <t>Matthew 4:13-16; 1 Corinthians 15:54; Hebrews 2:14-15; Revelation 21:4</t>
+        </is>
+      </c>
+      <c r="Q19" s="24" t="inlineStr">
+        <is>
+          <t>Jesus is this King: God come in person, beginning in Galilee (Matt 4), the Spirit resting on Him (John 1:32-33), who at the cross pardons our iniquity and in His resurrection swallows up death forever (1 Cor 15:54).</t>
+        </is>
+      </c>
+      <c r="R19" s="24" t="inlineStr">
+        <is>
+          <t>What do you most appreciate from all that King Jesus has done?</t>
+        </is>
+      </c>
+      <c r="S19" s="24" t="inlineStr">
+        <is>
+          <t>How does seeing the Big Problem as sin and death — not just our circumstances — shape the way you feel and think about your own sin?</t>
+        </is>
+      </c>
+      <c r="T19" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah said this King would be ‘God Himself’ come to save. How does it move you that God would come in person for you?</t>
+        </is>
+      </c>
+      <c r="U19" s="24" t="inlineStr">
+        <is>
+          <t>death</t>
+        </is>
+      </c>
+      <c r="V19" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 25:8 — through His King, God will swallow up ___ forever.</t>
+        </is>
+      </c>
+      <c r="W19" s="24" t="inlineStr">
+        <is>
+          <t>Galilee</t>
+        </is>
+      </c>
+      <c r="X19" s="24" t="inlineStr">
+        <is>
+          <t>Matthew 4 — Jesus, the light of Isaiah 9, begins His ministry in ___.</t>
+        </is>
+      </c>
+      <c r="Y19" s="24" t="inlineStr"/>
+      <c r="Z19" s="24" t="inlineStr">
+        <is>
+          <t>Salvation</t>
+        </is>
+      </c>
+      <c r="AA19" s="24" t="inlineStr">
+        <is>
+          <t>• Hold back the ‘light from Galilee’ (9:1-2) and the Spirit ‘resting’ (11:2) until the NT reveal lands — they are the clues by which Jesus is recognised as the true Davidic King.
+• Weight the application on Discussion 2 (what Jesus has done: sin pardoned, death undone).</t>
+        </is>
+      </c>
+      <c r="AB19" s="24" t="inlineStr">
+        <is>
+          <t>Pray that we would behold King Jesus — God come in person — and treasure the salvation He brings: our sin pardoned and death itself swallowed up.</t>
+        </is>
+      </c>
+      <c r="AC19" s="24" t="inlineStr">
+        <is>
+          <t>As you reflect on God’s King Who Saves (Isaiah 9; 11; 25; 40), what does this passage reveal about God’s character that you can praise Him for?</t>
+        </is>
+      </c>
+      <c r="AD19" s="24" t="inlineStr">
+        <is>
+          <t>In light of what you’ve studied, where have you fallen short of God’s design? Where have you resisted His good rule?</t>
+        </is>
+      </c>
+      <c r="AE19" s="24" t="inlineStr">
+        <is>
+          <t>What can you thank God for in light of this passage — especially how Christ fulfils what you’ve studied?</t>
+        </is>
+      </c>
+      <c r="AF19" s="24" t="inlineStr">
+        <is>
+          <t>What do you need from God as you apply this truth to your life this week?</t>
+        </is>
+      </c>
+      <c r="AG19" s="24" t="inlineStr"/>
+      <c r="AH19" s="24" t="inlineStr"/>
+      <c r="AI19" s="24" t="inlineStr"/>
+      <c r="AJ19" s="24" t="inlineStr"/>
+      <c r="AK19" s="24" t="inlineStr"/>
+      <c r="AL19" s="24" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="AM19" s="24" t="inlineStr"/>
+      <c r="AN19" s="24" t="inlineStr">
+        <is>
+          <t>The deepest problem is sin and death, not just hard circumstances. How does that reframe what you most need from God?</t>
+        </is>
+      </c>
+      <c r="AO19" s="24" t="inlineStr">
+        <is>
+          <t>Behold King Jesus — God come in person, who pardons your sin and has swallowed death. Sit in wonder and thank Him.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>52-54</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>The Suffering Servant</t>
+        </is>
+      </c>
+      <c r="E20" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah has shown us a King who is God Himself, who will swallow up death and pardon sin. But HOW will God actually pardon sin? How can a holy God forgive guilty people?</t>
+        </is>
+      </c>
+      <c r="F20" s="24" t="inlineStr">
+        <is>
+          <t>Through His Servant — and in a way no one expected. The fourth Servant Song (52:13-53:12) shows the Servant ‘high and lifted up’ yet ‘despised and rejected’, ‘pierced for our transgressions’, the Lord laying ‘on him the iniquity of us all’. He bears our sin as a substitute so that ‘the righteous one, my servant, makes many to be accounted righteous.’ This is how the King saves — by suffering in our place.</t>
+        </is>
+      </c>
+      <c r="G20" s="24" t="inlineStr">
+        <is>
+          <t>Context: ‘Servant’ runs through Isaiah (Abraham, Moses, David, Israel) with obedience as its key mark; chapters 42-53 unveil ‘the Servant’ in four Songs. Isaiah 52-54 flows: God’s coming salvation (52:1-12), the fourth Servant Song (52:13-53:12), and a call to respond — ‘Sing!’ (54). Read chapter 53 slowly; watch who the Servant suffers for.</t>
+        </is>
+      </c>
+      <c r="H20" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 52:1-12 | God’s coming salvation — good news proclaimed
+Isaiah 52:13-53:12 | The fourth Servant Song
+Isaiah 54 | The response: ‘Sing!’</t>
+        </is>
+      </c>
+      <c r="I20" s="24" t="inlineStr">
+        <is>
+          <t>God’s salvation comes through His Servant, who though exalted is despised and rejected, bearing the sin of many as a substitute to make them righteous.</t>
+        </is>
+      </c>
+      <c r="J20" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 53:5 — But he was pierced for our transgressions; he was crushed for our iniquities; upon him was the chastisement that brought us peace, and with his wounds we are healed.</t>
+        </is>
+      </c>
+      <c r="K20" s="24" t="inlineStr">
+        <is>
+          <t>The herald announces ‘Your God reigns’ (52:7) — but the King establishes His reign not by force; the exalted Servant is also the rejected one (52:13-14), high and lifted up through suffering.</t>
+        </is>
+      </c>
+      <c r="L20" s="24" t="inlineStr">
+        <is>
+          <t>The Servant **bears our sins as a substitute**: ‘pierced for our transgressions… the Lord has laid on him the iniquity of us all’ (53:5-6), pouring out his soul to death to make many righteous (53:11-12). This is how God saves.</t>
+        </is>
+      </c>
+      <c r="M20" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 54 is the **response and promise**: the barren one bursts into song with many offspring, an everlasting covenant of peace and steadfast love that will not depart (54:1,10), and ‘many are now servants of the Lord’ like the Servant (54:17).</t>
+        </is>
+      </c>
+      <c r="N20" s="24" t="inlineStr">
+        <is>
+          <t>God is both perfectly just and astonishingly gracious: He Himself provides the Servant to bear the sin He cannot overlook — satisfying justice while pardoning sinners — out of steadfast love that will never depart.</t>
+        </is>
+      </c>
+      <c r="O20" s="24" t="inlineStr">
+        <is>
+          <t>‘All we like sheep have gone astray; we have turned — every one — to his own way’ (53:6). We cannot make ourselves righteous; we esteemed the Servant ‘not’, yet it was our griefs and iniquities he carried.</t>
+        </is>
+      </c>
+      <c r="P20" s="24" t="inlineStr">
+        <is>
+          <t>John 12:30-34; 2 Corinthians 5:21</t>
+        </is>
+      </c>
+      <c r="Q20" s="24" t="inlineStr">
+        <is>
+          <t>Jesus is the Suffering Servant: ‘lifted up’ on the cross to draw all people (John 12:32); ‘God made him to be sin who knew no sin, so that in him we might become the righteousness of God’ (2 Cor 5:21) — the great exchange Isaiah foretold.</t>
+        </is>
+      </c>
+      <c r="R20" s="24" t="inlineStr">
+        <is>
+          <t>How has God spoken to you through the Suffering Servant Song today?</t>
+        </is>
+      </c>
+      <c r="S20" s="24" t="inlineStr">
+        <is>
+          <t>What about Christ do you see more clearly, or treasure more, through this Song?</t>
+        </is>
+      </c>
+      <c r="T20" s="24" t="inlineStr">
+        <is>
+          <t>‘The Lord has laid on him the iniquity of us all.’ How does it change you to know your sin was laid on Jesus, and His righteousness credited to you (2 Cor 5:21)?</t>
+        </is>
+      </c>
+      <c r="U20" s="24" t="inlineStr">
+        <is>
+          <t>iniquity</t>
+        </is>
+      </c>
+      <c r="V20" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 53:6 — the Lord has laid on him the ___ of us all.</t>
+        </is>
+      </c>
+      <c r="W20" s="24" t="inlineStr">
+        <is>
+          <t>righteousness</t>
+        </is>
+      </c>
+      <c r="X20" s="24" t="inlineStr">
+        <is>
+          <t>2 Corinthians 5:21 — God made him to be sin, so that in him we might become the ___ of God.</t>
+        </is>
+      </c>
+      <c r="Y20" s="24" t="inlineStr"/>
+      <c r="Z20" s="24" t="inlineStr">
+        <is>
+          <t>Salvation</t>
+        </is>
+      </c>
+      <c r="AA20" s="24" t="inlineStr">
+        <is>
+          <t>• Let Isaiah 53 breathe — read it slowly and let its weight land before the NT reveal.
+• The ‘high and lifted up’ language (52:13) deliberately echoes God’s own exaltation in Isaiah (6:1; 33:10; 57:15): the Servant’s exaltation IS God’s.</t>
+        </is>
+      </c>
+      <c r="AB20" s="24" t="inlineStr">
+        <is>
+          <t>Pray that we would behold Christ our Suffering Servant — pierced for our transgressions — and treasure the great exchange: our sin on Him, His righteousness on us.</t>
+        </is>
+      </c>
+      <c r="AC20" s="24" t="inlineStr">
+        <is>
+          <t>As you reflect on The Suffering Servant (Isaiah 52-54), what does this passage reveal about God’s character that you can praise Him for?</t>
+        </is>
+      </c>
+      <c r="AD20" s="24" t="inlineStr">
+        <is>
+          <t>In light of what you’ve studied, where have you fallen short of God’s design? Where have you resisted His good rule?</t>
+        </is>
+      </c>
+      <c r="AE20" s="24" t="inlineStr">
+        <is>
+          <t>What can you thank God for in light of this passage — especially how Christ fulfils what you’ve studied?</t>
+        </is>
+      </c>
+      <c r="AF20" s="24" t="inlineStr">
+        <is>
+          <t>What do you need from God as you apply this truth to your life this week?</t>
+        </is>
+      </c>
+      <c r="AG20" s="24" t="inlineStr"/>
+      <c r="AH20" s="24" t="inlineStr"/>
+      <c r="AI20" s="24" t="inlineStr"/>
+      <c r="AJ20" s="24" t="inlineStr"/>
+      <c r="AK20" s="24" t="inlineStr"/>
+      <c r="AL20" s="24" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="AM20" s="24" t="inlineStr"/>
+      <c r="AN20" s="24" t="inlineStr">
+        <is>
+          <t>Read Isaiah 53 slowly as a prayer. Which line most makes you see your sin — and His love — clearly?</t>
+        </is>
+      </c>
+      <c r="AO20" s="24" t="inlineStr">
+        <is>
+          <t>Your sin was laid on Jesus; His righteousness is credited to you. Behold Him and let your heart respond in worship.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>Jeremiah</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>The New Covenant</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>Every covenant so far has run aground on the same rock — the human heart. If the problem is the heart, what would God have to do to finally fix it?</t>
+        </is>
+      </c>
+      <c r="F21" s="24" t="inlineStr">
+        <is>
+          <t>He would have to make a new kind of covenant. In Jeremiah 31, into the darkness of exile, God promises a New Covenant ‘not like’ the Sinai one Israel broke: He will put His law within them and write it on their hearts, He will be their God and they His people, all will know Him, and — the foundation — ‘I will forgive their iniquity and remember their sin no more.’ He will re-establish His people, forgive their sin, and give them a transformed heart to obey.</t>
+        </is>
+      </c>
+      <c r="G21" s="24" t="inlineStr">
+        <is>
+          <t>Context: Jeremiah prophesies in Judah’s final years and into the exile (Ezekiel’s era). Chapters 30-33 are the ‘Book of Consolation’ — hope spoken into the dark. The passage is divided by the repeated ‘behold, the days are coming’ (v.27, v.31, v.38). Notice how this covenant differs from every earlier one, and where its security lies.</t>
+        </is>
+      </c>
+      <c r="H21" s="24" t="inlineStr">
+        <is>
+          <t>Jeremiah 31:27-30 | ‘The days are coming’ — hope and questions
+Jeremiah 31:31-37 | The New Covenant
+Jeremiah 31:38-40 | God’s new holy city</t>
+        </is>
+      </c>
+      <c r="I21" s="24" t="inlineStr">
+        <is>
+          <t>God promises to establish a New Covenant with His people: He will faithfully re-establish them, forgive their sin, and give them a heart transformed to obey Him — unlike the covenant they broke.</t>
+        </is>
+      </c>
+      <c r="J21" s="24" t="inlineStr">
+        <is>
+          <t>Jeremiah 31:33 — I will put my law within them, and I will write it on their hearts. And I will be their God, and they shall be my people.</t>
+        </is>
+      </c>
+      <c r="K21" s="24" t="inlineStr">
+        <is>
+          <t>God pledges to **re-establish His scattered people** — to ‘build and to plant’ them again (v.28) and be their God — the kingdom relationship remade.</t>
+        </is>
+      </c>
+      <c r="L21" s="24" t="inlineStr">
+        <is>
+          <t>At the heart of the New Covenant is **full forgiveness**: ‘I will forgive their iniquity, and I will remember their sin no more’ (31:34) — the root problem dealt with at last.</t>
+        </is>
+      </c>
+      <c r="M21" s="24" t="inlineStr">
+        <is>
+          <t>God promises a **New Covenant** ‘not like’ the broken Sinai one (31:31-32): He will **write His law on their hearts** and transform them so that all, from least to greatest, truly know Him (31:33-34).</t>
+        </is>
+      </c>
+      <c r="N21" s="24" t="inlineStr">
+        <is>
+          <t>God is the faithful, steadfast-love God who will not give up on His people — He takes the initiative to do for them what they could never do for themselves: change the heart and forgive the sin.</t>
+        </is>
+      </c>
+      <c r="O21" s="24" t="inlineStr">
+        <is>
+          <t>Every covenant Israel made, they broke — ‘my covenant that they broke, though I was their husband’ (31:32). The problem is the heart; external law could command obedience but never create it.</t>
+        </is>
+      </c>
+      <c r="P21" s="24" t="inlineStr">
+        <is>
+          <t>Matthew 26:28; Romans 6:17-18; Hebrews 8:6-13</t>
+        </is>
+      </c>
+      <c r="Q21" s="24" t="inlineStr">
+        <is>
+          <t>Jesus inaugurates this New Covenant in His blood — ‘my blood of the covenant… for the forgiveness of sins’ (Matt 26:28). By His death our sin is forgiven and remembered no more, and by His Spirit He transforms our hearts so we become ‘obedient from the heart’ (Rom 6:17-18).</t>
+        </is>
+      </c>
+      <c r="R21" s="24" t="inlineStr">
+        <is>
+          <t>The New Covenant is founded on sins ‘remembered no more’. How does it change you to know your sin is not just forgiven but forgotten by God?</t>
+        </is>
+      </c>
+      <c r="S21" s="24" t="inlineStr">
+        <is>
+          <t>God promises to write His law on your heart and transform it — not just hand you rules. Where do you long for God to change what you WANT, not just what you do?</t>
+        </is>
+      </c>
+      <c r="T21" s="24" t="inlineStr">
+        <is>
+          <t>If you are in Christ, you live in this New Covenant now. How do its promises encourage you to live ‘as those who have become obedient from the heart’ (Rom 6:17)?</t>
+        </is>
+      </c>
+      <c r="U21" s="24" t="inlineStr">
+        <is>
+          <t>hearts</t>
+        </is>
+      </c>
+      <c r="V21" s="24" t="inlineStr">
+        <is>
+          <t>Jeremiah 31:33 — God will write His law on their ___.</t>
+        </is>
+      </c>
+      <c r="W21" s="24" t="inlineStr">
+        <is>
+          <t>blood</t>
+        </is>
+      </c>
+      <c r="X21" s="24" t="inlineStr">
+        <is>
+          <t>Matthew 26:28 — ‘this is my ___ of the covenant… for the forgiveness of sins.’</t>
+        </is>
+      </c>
+      <c r="Y21" s="24" t="inlineStr"/>
+      <c r="Z21" s="24" t="inlineStr">
+        <is>
+          <t>Promises</t>
+        </is>
+      </c>
+      <c r="AA21" s="24" t="inlineStr">
+        <is>
+          <t>• The passage is divided by the ‘behold, the days are coming’ markers (v.27, 31, 38); vv.35-37 add ‘Thus says the Lord’ twice — the covenant is as sure as creation.
+• The study compares the New Covenant with the Abrahamic (Gen 17:1-9) and Sinai (Ex 19:1-6; Deut 30:1-10) covenants — same promise, now written on the heart.</t>
+        </is>
+      </c>
+      <c r="AB21" s="24" t="inlineStr">
+        <is>
+          <t>Thank God for the New Covenant in Jesus’ blood — our sin remembered no more and our hearts transformed to obey; pray we would live as people who truly know Him.</t>
+        </is>
+      </c>
+      <c r="AC21" s="24" t="inlineStr">
+        <is>
+          <t>As you reflect on The New Covenant (Jeremiah 31), what does this passage reveal about God’s character that you can praise Him for?</t>
+        </is>
+      </c>
+      <c r="AD21" s="24" t="inlineStr">
+        <is>
+          <t>In light of what you’ve studied, where have you fallen short of God’s design? Where have you resisted His good rule?</t>
+        </is>
+      </c>
+      <c r="AE21" s="24" t="inlineStr">
+        <is>
+          <t>What can you thank God for in light of this passage — especially how Christ fulfils what you’ve studied?</t>
+        </is>
+      </c>
+      <c r="AF21" s="24" t="inlineStr">
+        <is>
+          <t>What do you need from God as you apply this truth to your life this week?</t>
+        </is>
+      </c>
+      <c r="AG21" s="24" t="inlineStr"/>
+      <c r="AH21" s="24" t="inlineStr"/>
+      <c r="AI21" s="24" t="inlineStr"/>
+      <c r="AJ21" s="24" t="inlineStr"/>
+      <c r="AK21" s="24" t="inlineStr"/>
+      <c r="AL21" s="24" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="AM21" s="24" t="inlineStr"/>
+      <c r="AN21" s="24" t="inlineStr">
+        <is>
+          <t>God promises to change your heart and to forget your sin. Which do you need to hear more today — and why?</t>
+        </is>
+      </c>
+      <c r="AO21" s="24" t="inlineStr">
+        <is>
+          <t>In Christ the New Covenant is yours: sin remembered no more, a heart transformed to obey. Rest in that and thank Him.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>43; 47</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>The New Temple</t>
+        </is>
+      </c>
+      <c r="E22" s="24" t="inlineStr">
+        <is>
+          <t>In Ezekiel 8-11 we watched God’s glory leave the temple — the worst possible judgement. Could that ever be undone? Would God ever come back?</t>
+        </is>
+      </c>
+      <c r="F22" s="24" t="inlineStr">
+        <is>
+          <t>Yes — and gloriously. God shows Ezekiel a new temple, and ‘the glory of the Lord filled the temple’ as it returns from the east (43:1-5) — the exact reversal of its departure. But it is more than a building: its very design teaches God’s people to obey (ch.43), and from it flows a river that grows ever deeper, bringing life and healing everywhere — remaking a whole new creation, like Eden renewed (ch.47). God will dwell with His people again, forever.</t>
+        </is>
+      </c>
+      <c r="G22" s="24" t="inlineStr">
+        <is>
+          <t>Context: Same Ezekiel, now the hope-filled climax of his visions (chs. 40-48). Remember the devastating departure of God’s glory in chapters 8-11 — this is its answer. Watch where the glory comes FROM, and trace what the river does as it flows. (43:3 deliberately sets this vision beside the vision of the city’s destruction and the Chebar vision.)</t>
+        </is>
+      </c>
+      <c r="H22" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel 43:1-12 | The glory of the Lord returns to the new temple
+Ezekiel 47:1-12 | The river of life flows from the temple</t>
+        </is>
+      </c>
+      <c r="I22" s="24" t="inlineStr">
+        <is>
+          <t>God will build a new temple — His glory returning to dwell with His people — that is more than a building: it teaches His law for obedience and pours out waters of new life, remaking creation like Eden renewed.</t>
+        </is>
+      </c>
+      <c r="J22" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel 43:7 — Son of man, this is the place of my throne and the place of the soles of my feet, where I will dwell in the midst of the people of Israel forever.</t>
+        </is>
+      </c>
+      <c r="K22" s="24" t="inlineStr">
+        <is>
+          <t>God’s **glory returns** from the east — the very place it left in chapters 8-11 — and fills the temple (a throwback to Exodus 40 and 1 Kings 8): ‘this is the place of my throne… where I will dwell… forever’ (43:7).</t>
+        </is>
+      </c>
+      <c r="L22" s="24" t="inlineStr">
+        <is>
+          <t>A **river of life** flows from the temple, impossibly deepening as it goes, bringing healing and teeming life — even reviving the Dead Sea (47:1-12). God’s presence makes a dead world alive, like Eden renewed.</t>
+        </is>
+      </c>
+      <c r="M22" s="24" t="inlineStr">
+        <is>
+          <t>The vision answers the covenant hope: God dwelling with His people, His law known and obeyed (the temple’s very design, 43:10-12), the curse reversed and creation healed — the New Covenant made visible.</t>
+        </is>
+      </c>
+      <c r="N22" s="24" t="inlineStr">
+        <is>
+          <t>God is faithful and gracious beyond the judgement: the holy God who had to leave now returns to dwell with His people forever, teaching them to obey and making even the dead places teem with life.</t>
+        </is>
+      </c>
+      <c r="O22" s="24" t="inlineStr">
+        <is>
+          <t>Israel could not keep God’s presence by their own faithfulness — they drove His glory out (chs. 8-11). Seeing God’s holy design is meant to make them ashamed of their sin; the new temple and river are God’s gift, not their achievement.</t>
+        </is>
+      </c>
+      <c r="P22" s="24" t="inlineStr">
+        <is>
+          <t>John 7:37-39; Revelation 21:22-22:5</t>
+        </is>
+      </c>
+      <c r="Q22" s="24" t="inlineStr">
+        <is>
+          <t>Jesus is the true temple (John 2) from whom ‘rivers of living water’ flow by the Spirit (John 7:37-39); His church becomes God’s dwelling, and the vision finds its end in Revelation 21-22 — no temple needed, for God dwells with His people, the river of life flowing from His throne.</t>
+        </is>
+      </c>
+      <c r="R22" s="24" t="inlineStr">
+        <is>
+          <t>How is Ezekiel’s vision of the new temple fulfilled through Christ and then His church?</t>
+        </is>
+      </c>
+      <c r="S22" s="24" t="inlineStr">
+        <is>
+          <t>What does it mean for you to have the living waters of God’s Spirit in you — and flowing out to others?</t>
+        </is>
+      </c>
+      <c r="T22" s="24" t="inlineStr">
+        <is>
+          <t>What do you think or feel as you picture the new temple Ezekiel saw — God’s glory back, dwelling with His people forever?</t>
+        </is>
+      </c>
+      <c r="U22" s="24" t="inlineStr">
+        <is>
+          <t>glory</t>
+        </is>
+      </c>
+      <c r="V22" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel 43:5 — the ___ of the Lord filled the temple (returning from the east, as it had left in chapters 8-11).</t>
+        </is>
+      </c>
+      <c r="W22" s="24" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="X22" s="24" t="inlineStr">
+        <is>
+          <t>John 7 — from Jesus flow rivers of living ___ by the Spirit.</t>
+        </is>
+      </c>
+      <c r="Y22" s="24" t="inlineStr"/>
+      <c r="Z22" s="24" t="inlineStr">
+        <is>
+          <t>Kingdom</t>
+        </is>
+      </c>
+      <c r="AA22" s="24" t="inlineStr">
+        <is>
+          <t>• This vision is the deliberate reversal of Session 16 (Ezekiel 8-11): the glory that departed to the east returns from the east; the river undoes the curse — pointing to Revelation 21-22.
+• ‘Knowing the design/measurements’ of the temple (43:10-12) stands for knowing and keeping God’s law — linking this vision to the New Covenant.</t>
+        </is>
+      </c>
+      <c r="AB22" s="24" t="inlineStr">
+        <is>
+          <t>Praise God that His glory returns by grace to dwell with His people, and that in Jesus the river of life flows to us by the Spirit; pray for His life to heal and overflow to others.</t>
+        </is>
+      </c>
+      <c r="AC22" s="24" t="inlineStr">
+        <is>
+          <t>As you reflect on The New Temple (Ezekiel 43; 47), what does this passage reveal about God’s character that you can praise Him for?</t>
+        </is>
+      </c>
+      <c r="AD22" s="24" t="inlineStr">
+        <is>
+          <t>In light of what you’ve studied, where have you fallen short of God’s design? Where have you resisted His good rule?</t>
+        </is>
+      </c>
+      <c r="AE22" s="24" t="inlineStr">
+        <is>
+          <t>What can you thank God for in light of this passage — especially how Christ fulfils what you’ve studied?</t>
+        </is>
+      </c>
+      <c r="AF22" s="24" t="inlineStr">
+        <is>
+          <t>What do you need from God as you apply this truth to your life this week?</t>
+        </is>
+      </c>
+      <c r="AG22" s="24" t="inlineStr"/>
+      <c r="AH22" s="24" t="inlineStr"/>
+      <c r="AI22" s="24" t="inlineStr"/>
+      <c r="AJ22" s="24" t="inlineStr"/>
+      <c r="AK22" s="24" t="inlineStr"/>
+      <c r="AL22" s="24" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="AM22" s="24" t="inlineStr"/>
+      <c r="AN22" s="24" t="inlineStr">
+        <is>
+          <t>God’s glory returns and a river of life flows out. Where do you most need God’s presence and life right now?</t>
+        </is>
+      </c>
+      <c r="AO22" s="24" t="inlineStr">
+        <is>
+          <t>In Jesus the river of living water flows to you by the Spirit, and one day God will dwell with His people forever. Rest in His presence and thank Him.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>Nehemiah</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="inlineStr">
+        <is>
+          <t>8-10; 13</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>How the OT Ends</t>
+        </is>
+      </c>
+      <c r="E23" s="24" t="inlineStr">
+        <is>
+          <t>The exiles are finally home, the temple rebuilt, the Law read aloud, the people in tears of repentance renewing their vows to God. Surely this time it sticks. How does the Old Testament’s story actually end?</t>
+        </is>
+      </c>
+      <c r="F23" s="24" t="inlineStr">
+        <is>
+          <t>On an honest, unresolved note. In Nehemiah 8-10 the people hear the Law, grieve, rejoice, and bind themselves by oath to obey. But by Nehemiah 13 — after Nehemiah is away a while — they are breaking the very promises they made: the temple profaned, the Sabbath broken, intermarriage with the nations. The OT closes with God’s people back in the land but still with the same unchanged heart — the whole story leaning forward, aching for the New Covenant and the King who alone can save.</t>
+        </is>
+      </c>
+      <c r="G23" s="24" t="inlineStr">
+        <is>
+          <t>Context: ~440 BC, the very end of the OT narrative. The exiles have returned and rebuilt (the 2nd temple). Read how the people respond to the Law (Neh 8-9), what they commit to (Neh 10), and what has happened by Neh 13. Ask honestly: how does the OT story end — and what is it leaving us waiting for?</t>
+        </is>
+      </c>
+      <c r="H23" s="24" t="inlineStr">
+        <is>
+          <t>Nehemiah 8-9 | The Law read: weeping, joy and confession
+Nehemiah 10 | The covenant renewed by oath
+Nehemiah 13 | The relapse</t>
+        </is>
+      </c>
+      <c r="I23" s="24" t="inlineStr">
+        <is>
+          <t>Home from exile, God’s people hear the Law and renew the covenant — yet soon relapse into sin, so the OT ends still waiting for the Saviour who can change the heart.</t>
+        </is>
+      </c>
+      <c r="J23" s="24" t="inlineStr">
+        <is>
+          <t>Nehemiah 9:33 — Yet you have been righteous in all that has come upon us, for you have dealt faithfully and we have acted wickedly.</t>
+        </is>
+      </c>
+      <c r="K23" s="24" t="inlineStr">
+        <is>
+          <t>God’s people are **back in the land** under God’s word — the Law read publicly, the people assembled (Neh 8) — the outward restoration of the kingdom community.</t>
+        </is>
+      </c>
+      <c r="L23" s="24" t="inlineStr">
+        <is>
+          <t>Nehemiah 9 rehearses the whole story of God’s **faithful salvation** against Israel’s repeated rebellion — ‘you have been righteous… we have acted wickedly’ (9:33) — exposing that the problem was never God’s faithfulness but their hearts.</t>
+        </is>
+      </c>
+      <c r="M23" s="24" t="inlineStr">
+        <is>
+          <t>They **renew the covenant** by solemn oath (Neh 10) — yet Neh 13 shows them breaking it almost at once, leaving the OT’s promises unfulfilled and crying out for the **New Covenant** that can write the law on the heart.</t>
+        </is>
+      </c>
+      <c r="N23" s="24" t="inlineStr">
+        <is>
+          <t>God is faithful and righteous through the whole story — patient, forgiving, keeping His word to a people who keep failing — setting the stage for the only solution: a covenant that changes the heart.</t>
+        </is>
+      </c>
+      <c r="O23" s="24" t="inlineStr">
+        <is>
+          <t>Even after exile, miracle, Law and heartfelt vows, the people relapse into the same old sins (Neh 13). Resolutions and ceremonies cannot change the heart; the OT ends with the problem unsolved.</t>
+        </is>
+      </c>
+      <c r="P23" s="24" t="inlineStr">
+        <is>
+          <t>Luke 24:44-47; Jeremiah 31:31-34</t>
+        </is>
+      </c>
+      <c r="Q23" s="24" t="inlineStr">
+        <is>
+          <t>The OT ends unresolved on purpose — every rescue, king, temple and covenant has pointed beyond itself. It all ‘must be fulfilled’ in Jesus (Luke 24:44), who brings the New Covenant Jeremiah promised: forgiveness and a new heart the Law never could give.</t>
+        </is>
+      </c>
+      <c r="R23" s="24" t="inlineStr">
+        <is>
+          <t>How do you feel about how the whole Old Testament ends — home, but still unchanged?</t>
+        </is>
+      </c>
+      <c r="S23" s="24" t="inlineStr">
+        <is>
+          <t>Nehemiah 13 shows that heartfelt resolutions couldn’t fix the heart. Where do you see that pattern in your own walk — and where does it drive you?</t>
+        </is>
+      </c>
+      <c r="T23" s="24" t="inlineStr">
+        <is>
+          <t>How does seeing the OT end ‘waiting’ make you treasure Jesus and the New Covenant more?</t>
+        </is>
+      </c>
+      <c r="U23" s="24" t="inlineStr">
+        <is>
+          <t>wickedly</t>
+        </is>
+      </c>
+      <c r="V23" s="24" t="inlineStr">
+        <is>
+          <t>Nehemiah 9:33 — ‘You have dealt faithfully, and we have acted ___.’</t>
+        </is>
+      </c>
+      <c r="W23" s="24" t="inlineStr">
+        <is>
+          <t>fulfilled</t>
+        </is>
+      </c>
+      <c r="X23" s="24" t="inlineStr">
+        <is>
+          <t>Luke 24:44 — everything written about Jesus in the Law, the Prophets and the Psalms must be ___.</t>
+        </is>
+      </c>
+      <c r="Y23" s="24" t="inlineStr"/>
+      <c r="Z23" s="24" t="inlineStr">
+        <is>
+          <t>Promises</t>
+        </is>
+      </c>
+      <c r="AA23" s="24" t="inlineStr">
+        <is>
+          <t>• This is the end of the OT narrative — land yes, changed heart no. The deliberate anticlimax is the point: it sends us to the New Covenant (Jer 31) and to Jesus (Luke 24).
+• Chapters span Neh 8-10 and 13 (the prep summarised 8-9 as the response to the Law, 10 as the renewed covenant, 13 as the relapse).</t>
+        </is>
+      </c>
+      <c r="AB23" s="24" t="inlineStr">
+        <is>
+          <t>Thank God that the whole OT story was leaning toward Jesus; pray we would not trust our own resolutions but the Saviour and New Covenant who alone change the heart.</t>
+        </is>
+      </c>
+      <c r="AC23" s="24" t="inlineStr">
+        <is>
+          <t>As you reflect on How the OT Ends (Nehemiah 8-10; 13), what does this passage reveal about God’s character that you can praise Him for?</t>
+        </is>
+      </c>
+      <c r="AD23" s="24" t="inlineStr">
+        <is>
+          <t>In light of what you’ve studied, where have you fallen short of God’s design? Where have you resisted His good rule?</t>
+        </is>
+      </c>
+      <c r="AE23" s="24" t="inlineStr">
+        <is>
+          <t>What can you thank God for in light of this passage — especially how Christ fulfils what you’ve studied?</t>
+        </is>
+      </c>
+      <c r="AF23" s="24" t="inlineStr">
+        <is>
+          <t>What do you need from God as you apply this truth to your life this week?</t>
+        </is>
+      </c>
+      <c r="AG23" s="24" t="inlineStr"/>
+      <c r="AH23" s="24" t="inlineStr"/>
+      <c r="AI23" s="24" t="inlineStr"/>
+      <c r="AJ23" s="24" t="inlineStr"/>
+      <c r="AK23" s="24" t="inlineStr"/>
+      <c r="AL23" s="24" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="AM23" s="24" t="inlineStr"/>
+      <c r="AN23" s="24" t="inlineStr">
+        <is>
+          <t>The OT ends with God’s people home but unchanged. Where are you relying on resolutions instead of a new heart?</t>
+        </is>
+      </c>
+      <c r="AO23" s="24" t="inlineStr">
+        <is>
+          <t>The whole story was waiting for Jesus. Thank Him that in the New Covenant He gives what the Law never could — forgiveness and a changed heart.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="Z2:Z13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -3526,7 +5325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:P67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.5"/>
   <cols>
     <col width="8" customWidth="1" style="22" min="1" max="1"/>
@@ -5676,6 +7475,2076 @@
         </is>
       </c>
       <c r="P34" s="12" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="24" t="n">
+        <v>13</v>
+      </c>
+      <c r="B35" s="24" t="inlineStr">
+        <is>
+          <t>The Need for a King</t>
+        </is>
+      </c>
+      <c r="C35" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="24" t="inlineStr">
+        <is>
+          <t>Judges 1</t>
+        </is>
+      </c>
+      <c r="E35" s="24" t="inlineStr">
+        <is>
+          <t>The Failure of the Military Conquest</t>
+        </is>
+      </c>
+      <c r="F35" s="24" t="inlineStr">
+        <is>
+          <t>Read through Judges 1 and trace the progression of Israel’s conquest of Canaan (note v.10, v.19, v.20-21, v.28, v.33). What changes?</t>
+        </is>
+      </c>
+      <c r="G35" s="24" t="inlineStr">
+        <is>
+          <t>Watch the verbs shift — from destroying, to could not, to would not, to living among.</t>
+        </is>
+      </c>
+      <c r="H35" s="24" t="inlineStr">
+        <is>
+          <t>Israel slides from destroying the Canaanites completely (v.10), to being unable to (v.19), to choosing not to (v.21), to merely putting them to forced labour (v.28) — obedience decaying into compromise.</t>
+        </is>
+      </c>
+      <c r="I35" s="24" t="inlineStr">
+        <is>
+          <t>Why is this progression so serious? What had God commanded Israel to do on entering Canaan?</t>
+        </is>
+      </c>
+      <c r="J35" s="24" t="inlineStr">
+        <is>
+          <t>God called them to drive out the nations completely and leave nothing behind.</t>
+        </is>
+      </c>
+      <c r="K35" s="24" t="inlineStr">
+        <is>
+          <t>God had commanded Israel to drive the nations out completely; by stopping short and coexisting, they are directly disobeying Him.</t>
+        </is>
+      </c>
+      <c r="L35" s="24" t="inlineStr">
+        <is>
+          <t>What is the result of Israel’s compromise (v.34), and why is that significant?</t>
+        </is>
+      </c>
+      <c r="M35" s="24" t="inlineStr">
+        <is>
+          <t>Who ends up pressing whom? Think about the land as God’s promised blessing.</t>
+        </is>
+      </c>
+      <c r="N35" s="24" t="inlineStr">
+        <is>
+          <t>The tables turn — the Amorites press Israel back (v.34). The promised blessing of the land is going into reverse as the fruit of their disobedience.</t>
+        </is>
+      </c>
+      <c r="O35" s="24" t="inlineStr">
+        <is>
+          <t>Judges 1 records a conquest that fizzles: Israel’s obedience decays from destroying the nations, to tolerating them, to being pressed back by them. The promised blessing of the land starts slipping away as disobedience takes root.</t>
+        </is>
+      </c>
+      <c r="P35" s="24" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="24" t="n">
+        <v>13</v>
+      </c>
+      <c r="B36" s="24" t="inlineStr">
+        <is>
+          <t>The Need for a King</t>
+        </is>
+      </c>
+      <c r="C36" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" s="24" t="inlineStr">
+        <is>
+          <t>Judges 2</t>
+        </is>
+      </c>
+      <c r="E36" s="24" t="inlineStr">
+        <is>
+          <t>The Spiritual Failure &amp; the Cycle</t>
+        </is>
+      </c>
+      <c r="F36" s="24" t="inlineStr">
+        <is>
+          <t>Judges 2 interprets what really went wrong. What was Israel’s deeper problem (v.1-10)?</t>
+        </is>
+      </c>
+      <c r="G36" s="24" t="inlineStr">
+        <is>
+          <t>It’s more than disobedience — look especially at v.10.</t>
+        </is>
+      </c>
+      <c r="H36" s="24" t="inlineStr">
+        <is>
+          <t>They refused to tear down the Canaanite altars (v.2), but the deeper problem is a generation ‘who did not know the Lord’ (v.10) — they forgot God and what He had done.</t>
+        </is>
+      </c>
+      <c r="I36" s="24" t="inlineStr">
+        <is>
+          <t>Trace the cycle Israel falls into (v.11-23). What are its stages?</t>
+        </is>
+      </c>
+      <c r="J36" s="24" t="inlineStr">
+        <is>
+          <t>It repeats — and it spirals downward.</t>
+        </is>
+      </c>
+      <c r="K36" s="24" t="inlineStr">
+        <is>
+          <t>Rebellion → Retribution (God’s judgement) → Request (they cry out) → Rescue (God raises a judge) → Rest (peace while he lives) → Repeat — sinking lower each time.</t>
+        </is>
+      </c>
+      <c r="L36" s="24" t="inlineStr">
+        <is>
+          <t>What is a judge meant to do, and was it an effective, lasting solution? Why or why not?</t>
+        </is>
+      </c>
+      <c r="M36" s="24" t="inlineStr">
+        <is>
+          <t>See v.16-19. What happens when the judge dies — and did the people’s hearts actually change?</t>
+        </is>
+      </c>
+      <c r="N36" s="24" t="inlineStr">
+        <is>
+          <t>A judge is raised to save them (v.18), but only temporarily — the judges die and the people relapse, even worse (v.19), because they ‘would not listen’ (v.17). The real problem is the heart.</t>
+        </is>
+      </c>
+      <c r="O36" s="24" t="inlineStr">
+        <is>
+          <t>Judges 2 exposes the heart behind the failure: Israel forgot the Lord and fell into a downward cycle of rebellion and rescue. The judges brought only temporary relief — they die, the people won’t listen, and ‘everyone did what was right in his own eyes’ (21:25). A better, lasting Saviour-King is needed.</t>
+        </is>
+      </c>
+      <c r="P36" s="24" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="24" t="n">
+        <v>13</v>
+      </c>
+      <c r="B37" s="24" t="inlineStr">
+        <is>
+          <t>The Need for a King</t>
+        </is>
+      </c>
+      <c r="C37" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" s="24" t="inlineStr">
+        <is>
+          <t>1 Samuel 8; 13:14; Deuteronomy 17:14-20</t>
+        </is>
+      </c>
+      <c r="E37" s="24" t="inlineStr">
+        <is>
+          <t>The Need for a Righteous King</t>
+        </is>
+      </c>
+      <c r="F37" s="24" t="inlineStr">
+        <is>
+          <t>In 1 Samuel 8, what kind of king does Israel ask for, and what will he cost them?</t>
+        </is>
+      </c>
+      <c r="G37" s="24" t="inlineStr">
+        <is>
+          <t>See v.5, v.20 — who do they want to be like? And what does Samuel warn a king will do?</t>
+        </is>
+      </c>
+      <c r="H37" s="24" t="inlineStr">
+        <is>
+          <t>A king ‘like all the nations’ (v.5, 20) to fight their battles — rejecting God as king. Samuel warns such a king will only take and take from them.</t>
+        </is>
+      </c>
+      <c r="I37" s="24" t="inlineStr">
+        <is>
+          <t>From 1 Samuel 13:14 and Deuteronomy 17:14-20, what kind of king is God actually looking for?</t>
+        </is>
+      </c>
+      <c r="J37" s="24" t="inlineStr">
+        <is>
+          <t>‘A man after God’s own heart’ — and Deut 17 spells out how such a king lives.</t>
+        </is>
+      </c>
+      <c r="K37" s="24" t="inlineStr">
+        <is>
+          <t>A king God Himself chooses (Deut 17:15), a man after God’s own heart (1 Sam 13:14), who fears the Lord and keeps His law — a model of obedience for all Israel.</t>
+        </is>
+      </c>
+      <c r="L37" s="24" t="inlineStr">
+        <is>
+          <t>Judges and 1 Samuel leave Israel needing a righteous King. How does the NT answer that need (Acts 5:29-32)?</t>
+        </is>
+      </c>
+      <c r="M37" s="24" t="inlineStr">
+        <is>
+          <t>Whom did God raise up as Leader and Saviour?</t>
+        </is>
+      </c>
+      <c r="N37" s="24" t="inlineStr">
+        <is>
+          <t>God raised up Jesus as Leader and Saviour (Acts 5:31) — the truly righteous King who saves us by His death and deals with the heart the judges never could.</t>
+        </is>
+      </c>
+      <c r="O37" s="24" t="inlineStr">
+        <is>
+          <t>Israel’s answer to the cycle is a king — but a king ‘like the nations’ only takes and oppresses. God is looking for a righteous king of His own choosing, a man after His heart who fears God and keeps His law. That longing is finally answered in Jesus, the Leader and Saviour God raised up.</t>
+        </is>
+      </c>
+      <c r="P37" s="24" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="24" t="n">
+        <v>14</v>
+      </c>
+      <c r="B38" s="24" t="inlineStr">
+        <is>
+          <t>Davidic Covenant</t>
+        </is>
+      </c>
+      <c r="C38" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="24" t="inlineStr">
+        <is>
+          <t>Deuteronomy 17:14-20; 1 Samuel 8; 13; 15</t>
+        </is>
+      </c>
+      <c r="E38" s="24" t="inlineStr">
+        <is>
+          <t>The king the Lord wants (recap)</t>
+        </is>
+      </c>
+      <c r="F38" s="24" t="inlineStr">
+        <is>
+          <t>Pulling together Deut 17, 1 Samuel 8, 13 and 15 — what has the OT already said about the kind of king God wants (and doesn’t)?</t>
+        </is>
+      </c>
+      <c r="G38" s="24" t="inlineStr">
+        <is>
+          <t>Contrast the ‘king like the nations’ with the king who fears the Lord and obeys His word.</t>
+        </is>
+      </c>
+      <c r="H38" s="24" t="inlineStr">
+        <is>
+          <t>Not a self-serving king like the nations (1 Sam 8) or one who ignores God (1 Sam 13; 15), but a godly king who fears the Lord, keeps His commands and models obedience (Deut 17).</t>
+        </is>
+      </c>
+      <c r="I38" s="24" t="inlineStr">
+        <is>
+          <t>Saul was also God’s chosen king. Why does God prefer David (1 Sam 15:28; 13:14)?</t>
+        </is>
+      </c>
+      <c r="J38" s="24" t="inlineStr">
+        <is>
+          <t>God’s choice, plus the character of the man — a man after God’s own heart.</t>
+        </is>
+      </c>
+      <c r="K38" s="24" t="inlineStr">
+        <is>
+          <t>Kingship is God’s choice, but the king must share God’s heart. Saul was chosen yet rejected for disobeying; David is ‘better’ because he takes after the Lord’s own heart.</t>
+        </is>
+      </c>
+      <c r="L38" s="24" t="inlineStr"/>
+      <c r="M38" s="24" t="inlineStr"/>
+      <c r="N38" s="24" t="inlineStr"/>
+      <c r="O38" s="24" t="inlineStr">
+        <is>
+          <t>The OT has been sketching a ‘job description’ for God’s king: not the self-serving king of the nations, but a king of God’s own choosing who fears Him, obeys His word and models godliness for the people. Saul failed that test; the question is what God thinks of David.</t>
+        </is>
+      </c>
+      <c r="P38" s="24" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="24" t="n">
+        <v>14</v>
+      </c>
+      <c r="B39" s="24" t="inlineStr">
+        <is>
+          <t>Davidic Covenant</t>
+        </is>
+      </c>
+      <c r="C39" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>2 Samuel 7:1-17</t>
+        </is>
+      </c>
+      <c r="E39" s="24" t="inlineStr">
+        <is>
+          <t>God’s promise to David</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>David wants to build a house for the Lord. Why (v.1-2, 8-9)?</t>
+        </is>
+      </c>
+      <c r="G39" s="24" t="inlineStr">
+        <is>
+          <t>It flows from what God has already done for him.</t>
+        </is>
+      </c>
+      <c r="H39" s="24" t="inlineStr">
+        <is>
+          <t>It flows from gratitude: settled with rest from his enemies, David recognises all God has given him and wants to honour God in return.</t>
+        </is>
+      </c>
+      <c r="I39" s="24" t="inlineStr">
+        <is>
+          <t>God turns it around: instead of David building God a house, God will build David a ‘house’. What exactly does God promise (v.9-16)?</t>
+        </is>
+      </c>
+      <c r="J39" s="24" t="inlineStr">
+        <is>
+          <t>Notice the repeated ‘I will’. Compare the great name and the land with the Abrahamic and Sinai covenants.</t>
+        </is>
+      </c>
+      <c r="K39" s="24" t="inlineStr">
+        <is>
+          <t>A great name (v.9), a secure place for His people, and — beyond any building — an offspring whose throne and kingdom God will establish forever (v.16). The repeated ‘I will’ shows it rests on God’s faithfulness, not the king’s.</t>
+        </is>
+      </c>
+      <c r="L39" s="24" t="inlineStr">
+        <is>
+          <t>What does God repeatedly call David, and what does that reveal about the king God wants?</t>
+        </is>
+      </c>
+      <c r="M39" s="24" t="inlineStr">
+        <is>
+          <t>See ‘my servant’ — striking, at the very peak of David’s reign.</t>
+        </is>
+      </c>
+      <c r="N39" s="24" t="inlineStr">
+        <is>
+          <t>God calls David ‘my servant’, even at the height of his power — the king God wants is one who honours and serves Him.</t>
+        </is>
+      </c>
+      <c r="O39" s="24" t="inlineStr">
+        <is>
+          <t>David wants to build God a house; God promises instead to build David a ‘house’ — an everlasting throne and kingdom, secured by God’s own repeated ‘I will’. The faithful God will establish His forever-kingdom through the offspring of David, His servant-king.</t>
+        </is>
+      </c>
+      <c r="P39" s="24" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="24" t="n">
+        <v>14</v>
+      </c>
+      <c r="B40" s="24" t="inlineStr">
+        <is>
+          <t>Davidic Covenant</t>
+        </is>
+      </c>
+      <c r="C40" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" s="24" t="inlineStr">
+        <is>
+          <t>2 Samuel 7:18-29</t>
+        </is>
+      </c>
+      <c r="E40" s="24" t="inlineStr">
+        <is>
+          <t>David’s response</t>
+        </is>
+      </c>
+      <c r="F40" s="24" t="inlineStr">
+        <is>
+          <t>From the repetitions in David’s prayer, what kind of king is he?</t>
+        </is>
+      </c>
+      <c r="G40" s="24" t="inlineStr">
+        <is>
+          <t>How does David keep describing himself?</t>
+        </is>
+      </c>
+      <c r="H40" s="24" t="inlineStr">
+        <is>
+          <t>He repeatedly calls himself ‘your servant’ — humbled by grace, not a self-important king.</t>
+        </is>
+      </c>
+      <c r="I40" s="24" t="inlineStr">
+        <is>
+          <t>What does David keep asking God for in this prayer (v.25-29)?</t>
+        </is>
+      </c>
+      <c r="J40" s="24" t="inlineStr">
+        <is>
+          <t>He asks God to do what He has said — about the house.</t>
+        </is>
+      </c>
+      <c r="K40" s="24" t="inlineStr">
+        <is>
+          <t>He asks God to confirm and keep His word — to establish the ‘house’ (kingdom) He promised; David loves God’s house and pleads for it to last forever.</t>
+        </is>
+      </c>
+      <c r="L40" s="24" t="inlineStr">
+        <is>
+          <t>2 Samuel 7:19 calls this covenant ‘instruction/revelation for mankind’. Why does this promise reach beyond David?</t>
+        </is>
+      </c>
+      <c r="M40" s="24" t="inlineStr">
+        <is>
+          <t>Echo of Abraham — ‘in you all nations will be blessed’.</t>
+        </is>
+      </c>
+      <c r="N40" s="24" t="inlineStr">
+        <is>
+          <t>The forever-kingdom is for all nations, not just David’s line — echoing the Abrahamic promise that all nations will be blessed, reaching even to us today.</t>
+        </is>
+      </c>
+      <c r="O40" s="24" t="inlineStr">
+        <is>
+          <t>David responds as the servant-king God wants: humbled, calling himself ‘your servant’, loving God’s house and asking God simply to keep His promise. And the promise reaches beyond David — this forever-kingdom is God’s revelation for all mankind, pointing to the King still to come.</t>
+        </is>
+      </c>
+      <c r="P40" s="24" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="B41" s="24" t="inlineStr">
+        <is>
+          <t>The Temple</t>
+        </is>
+      </c>
+      <c r="C41" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="24" t="inlineStr">
+        <is>
+          <t>1 Kings 8:1-21</t>
+        </is>
+      </c>
+      <c r="E41" s="24" t="inlineStr">
+        <is>
+          <t>A house filled with the Lord’s presence</t>
+        </is>
+      </c>
+      <c r="F41" s="24" t="inlineStr">
+        <is>
+          <t>What do we see the people of Israel doing at the Temple (v.1-11)?</t>
+        </is>
+      </c>
+      <c r="G41" s="24" t="inlineStr">
+        <is>
+          <t>Assembling, sacrificing, moving the ark — and then something stops the priests.</t>
+        </is>
+      </c>
+      <c r="H41" s="24" t="inlineStr">
+        <is>
+          <t>Solomon assembles Israel and they sacrifice beyond counting as the ark is brought in (v.1-9); then the glory of the Lord fills the house so the priests cannot stand to minister (v.10-11).</t>
+        </is>
+      </c>
+      <c r="I41" s="24" t="inlineStr">
+        <is>
+          <t>What is inside the ark, and why does that matter (v.9)?</t>
+        </is>
+      </c>
+      <c r="J41" s="24" t="inlineStr">
+        <is>
+          <t>Only the two stone tablets from Horeb — think covenant and Exodus.</t>
+        </is>
+      </c>
+      <c r="K41" s="24" t="inlineStr">
+        <is>
+          <t>Only the two tablets from Horeb, where God made His covenant when He brought Israel out of Egypt (v.9) — the Temple’s significance is the Lord’s presence and covenant, not its grandeur.</t>
+        </is>
+      </c>
+      <c r="L41" s="24" t="inlineStr">
+        <is>
+          <t>According to Solomon (v.12-21), how has the Lord fulfilled His promise?</t>
+        </is>
+      </c>
+      <c r="M41" s="24" t="inlineStr">
+        <is>
+          <t>‘Your son... shall build the house for my name’ — has that happened?</t>
+        </is>
+      </c>
+      <c r="N41" s="24" t="inlineStr">
+        <is>
+          <t>God promised David that his son would build the house for His name (v.19); Solomon, David’s son, has now done so — the promise is fulfilled.</t>
+        </is>
+      </c>
+      <c r="O41" s="24" t="inlineStr">
+        <is>
+          <t>The ark is brought in and God’s glory fills the Temple — the Lord Himself comes to dwell with His people. The Temple’s true significance is His presence, not its splendour, and its completion shows God keeping His promise to David through Solomon.</t>
+        </is>
+      </c>
+      <c r="P41" s="24" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="B42" s="24" t="inlineStr">
+        <is>
+          <t>The Temple</t>
+        </is>
+      </c>
+      <c r="C42" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" s="24" t="inlineStr">
+        <is>
+          <t>1 Kings 8:22-53</t>
+        </is>
+      </c>
+      <c r="E42" s="24" t="inlineStr">
+        <is>
+          <t>A house where God hears His people</t>
+        </is>
+      </c>
+      <c r="F42" s="24" t="inlineStr">
+        <is>
+          <t>From Solomon’s prayer (v.22-30), what does he understand about God’s promises and about the Temple itself?</t>
+        </is>
+      </c>
+      <c r="G42" s="24" t="inlineStr">
+        <is>
+          <t>See v.23 (Exodus), v.25 (David), v.27 (can any house contain God?).</t>
+        </is>
+      </c>
+      <c r="H42" s="24" t="inlineStr">
+        <is>
+          <t>God faithfully remembers His promises (v.23) and David’s (v.25); yet even heaven cannot contain Him (v.27). The Temple is a place to pray toward, that God would hear and forgive (v.30).</t>
+        </is>
+      </c>
+      <c r="I42" s="24" t="inlineStr">
+        <is>
+          <t>Solomon makes seven requests (v.31-53). Across them all, what is the role of the house for Israel?</t>
+        </is>
+      </c>
+      <c r="J42" s="24" t="inlineStr">
+        <is>
+          <t>Whatever the trouble — sin, defeat, drought, famine, even exile — what do the people do, and what do they ask God to do?</t>
+        </is>
+      </c>
+      <c r="K42" s="24" t="inlineStr">
+        <is>
+          <t>In every case it is where God’s people — and even the foreigner — pray toward, so God will hear from heaven, forgive and restore them, through every trouble up to exile.</t>
+        </is>
+      </c>
+      <c r="L42" s="24" t="inlineStr">
+        <is>
+          <t>It’s striking that Solomon dwells on sin and exile at Israel’s peak. What does this reveal (see v.46)?</t>
+        </is>
+      </c>
+      <c r="M42" s="24" t="inlineStr">
+        <is>
+          <t>‘There is no one who does not sin.’</t>
+        </is>
+      </c>
+      <c r="N42" s="24" t="inlineStr">
+        <is>
+          <t>Even at Israel’s peak Solomon knows ‘there is no one who does not sin’ (v.46). The magnificent Temple cannot solve sin; he already anticipates exile — hinting it is not the forever-house.</t>
+        </is>
+      </c>
+      <c r="O42" s="24" t="inlineStr">
+        <is>
+          <t>Solomon’s prayer makes the Temple a house where God hears and forgives His praying people, through every trouble up to exile. Yet at Israel’s peak he keeps returning to sin — ‘there is no one who does not sin’ — showing the Temple cannot fix the heart, and pointing beyond itself.</t>
+        </is>
+      </c>
+      <c r="P42" s="24" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="B43" s="24" t="inlineStr">
+        <is>
+          <t>The Temple</t>
+        </is>
+      </c>
+      <c r="C43" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D43" s="24" t="inlineStr">
+        <is>
+          <t>1 Kings 8:54-66</t>
+        </is>
+      </c>
+      <c r="E43" s="24" t="inlineStr">
+        <is>
+          <t>Solomon blesses and consecrates the house</t>
+        </is>
+      </c>
+      <c r="F43" s="24" t="inlineStr">
+        <is>
+          <t>Solomon’s prayer raised the worrying prospect of Israel’s failure and exile. Why then does he still bless the people and lead a huge feast (v.54-66)?</t>
+        </is>
+      </c>
+      <c r="G43" s="24" t="inlineStr">
+        <is>
+          <t>Where does Solomon’s confidence come from (v.56-58)?</t>
+        </is>
+      </c>
+      <c r="H43" s="24" t="inlineStr">
+        <is>
+          <t>His confidence rests on God’s promises, not Israel’s performance: ‘Not one word has failed of all his good promise’ (v.56). The people rejoice for what God has done, not human works (v.66).</t>
+        </is>
+      </c>
+      <c r="I43" s="24" t="inlineStr"/>
+      <c r="J43" s="24" t="inlineStr"/>
+      <c r="K43" s="24" t="inlineStr"/>
+      <c r="L43" s="24" t="inlineStr"/>
+      <c r="M43" s="24" t="inlineStr"/>
+      <c r="N43" s="24" t="inlineStr"/>
+      <c r="O43" s="24" t="inlineStr">
+        <is>
+          <t>Solomon blesses Israel and feasts because God has kept every word of His promise and gives rest to His people. The joy is grounded in God’s faithfulness and goodness, not human achievement — yet the deeper problem of sin still waits for a greater King.</t>
+        </is>
+      </c>
+      <c r="P43" s="24" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="24" t="n">
+        <v>16</v>
+      </c>
+      <c r="B44" s="24" t="inlineStr">
+        <is>
+          <t>The Glory Departs</t>
+        </is>
+      </c>
+      <c r="C44" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel 8:1-17</t>
+        </is>
+      </c>
+      <c r="E44" s="24" t="inlineStr">
+        <is>
+          <t>Israel turns God’s sanctuary into a house of idols</t>
+        </is>
+      </c>
+      <c r="F44" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel is shown four ‘abominations’ in the Temple (v.1-17). What is happening in each, and why is it so serious?</t>
+        </is>
+      </c>
+      <c r="G44" s="24" t="inlineStr">
+        <is>
+          <t>An image of jealousy; elders with incense to idols; women weeping for Tammuz; men bowing to the sun — and where is all this happening?</t>
+        </is>
+      </c>
+      <c r="H44" s="24" t="inlineStr">
+        <is>
+          <t>An image of jealousy in God’s house; elders secretly burning incense to idols; women weeping for Tammuz; men worshipping the sun in the Holy of Holies. Israel has filled the very place of God’s presence with idols.</t>
+        </is>
+      </c>
+      <c r="I44" s="24" t="inlineStr">
+        <is>
+          <t>Coming straight after the glory-filled Temple of 1 Kings 8, how do you think God feels — and why?</t>
+        </is>
+      </c>
+      <c r="J44" s="24" t="inlineStr">
+        <is>
+          <t>His own house, His own people, His own presence — now filled with idols.</t>
+        </is>
+      </c>
+      <c r="K44" s="24" t="inlineStr">
+        <is>
+          <t>God is provoked to jealousy and grief: His own people defile His house and break His covenant in His very presence, even claiming He cannot see.</t>
+        </is>
+      </c>
+      <c r="L44" s="24" t="inlineStr"/>
+      <c r="M44" s="24" t="inlineStr"/>
+      <c r="N44" s="24" t="inlineStr"/>
+      <c r="O44" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel sees Israel filling God’s own Temple with idols — escalating abominations in the very place of His presence, while claiming the Lord does not see. The house of God’s glory has become a house of idols; the covenant is broken from the inside.</t>
+        </is>
+      </c>
+      <c r="P44" s="24" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="24" t="n">
+        <v>16</v>
+      </c>
+      <c r="B45" s="24" t="inlineStr">
+        <is>
+          <t>The Glory Departs</t>
+        </is>
+      </c>
+      <c r="C45" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel 8:18-9:11</t>
+        </is>
+      </c>
+      <c r="E45" s="24" t="inlineStr">
+        <is>
+          <t>Judgement for the abominations</t>
+        </is>
+      </c>
+      <c r="F45" s="24" t="inlineStr">
+        <is>
+          <t>What does God do after witnessing the abominations (8:18-9:11)?</t>
+        </is>
+      </c>
+      <c r="G45" s="24" t="inlineStr">
+        <is>
+          <t>Six men with weapons; a mark on the foreheads of those who grieve over the sin.</t>
+        </is>
+      </c>
+      <c r="H45" s="24" t="inlineStr">
+        <is>
+          <t>God brings judgement — men with weapons against the idolaters — though those who sigh and grieve over the sin are marked and spared (9:4). His holiness will not overlook sin, even His people’s.</t>
+        </is>
+      </c>
+      <c r="I45" s="24" t="inlineStr"/>
+      <c r="J45" s="24" t="inlineStr"/>
+      <c r="K45" s="24" t="inlineStr"/>
+      <c r="L45" s="24" t="inlineStr"/>
+      <c r="M45" s="24" t="inlineStr"/>
+      <c r="N45" s="24" t="inlineStr"/>
+      <c r="O45" s="24" t="inlineStr">
+        <is>
+          <t>God responds to the abominations with just judgement — He will not ignore sin, even His people’s. Yet even here mercy appears: those who grieve over the sin are marked and spared. Holiness and mercy meet in God’s response.</t>
+        </is>
+      </c>
+      <c r="P45" s="24" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="24" t="n">
+        <v>16</v>
+      </c>
+      <c r="B46" s="24" t="inlineStr">
+        <is>
+          <t>The Glory Departs</t>
+        </is>
+      </c>
+      <c r="C46" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D46" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel 10</t>
+        </is>
+      </c>
+      <c r="E46" s="24" t="inlineStr">
+        <is>
+          <t>The glory of God leaves the temple</t>
+        </is>
+      </c>
+      <c r="F46" s="24" t="inlineStr">
+        <is>
+          <t>Read Ezekiel 10:1-5, 18-19. What movements of God’s glory do you notice, and why describe the departure in stages rather than simply ‘God left’?</t>
+        </is>
+      </c>
+      <c r="G46" s="24" t="inlineStr">
+        <is>
+          <t>The glory moves from the cherubim, to the threshold, to the east gate — slowly, reluctantly.</t>
+        </is>
+      </c>
+      <c r="H46" s="24" t="inlineStr">
+        <is>
+          <t>The glory moves in stages — from the cherubim, to the threshold, to the east gate. The gradual, reluctant departure shows the Lord grieves to leave; it is no hasty abandonment.</t>
+        </is>
+      </c>
+      <c r="I46" s="24" t="inlineStr">
+        <is>
+          <t>Why is the departure of God’s glory such a devastating judgement — wouldn’t the destruction of Jerusalem itself be worse?</t>
+        </is>
+      </c>
+      <c r="J46" s="24" t="inlineStr">
+        <is>
+          <t>What was the whole point of the Temple, all the way back to Sinai and Eden?</t>
+        </is>
+      </c>
+      <c r="K46" s="24" t="inlineStr">
+        <is>
+          <t>The Temple existed for God’s presence with His people. To lose His presence is worse than losing the city — it is to lose the very thing that made them God’s people.</t>
+        </is>
+      </c>
+      <c r="L46" s="24" t="inlineStr"/>
+      <c r="M46" s="24" t="inlineStr"/>
+      <c r="N46" s="24" t="inlineStr"/>
+      <c r="O46" s="24" t="inlineStr">
+        <is>
+          <t>God’s glory leaves the Temple in slow, reluctant stages (Eze 10). Because the Temple existed for God’s presence with His people, the departure of His glory is a more devastating judgement than the destruction of the city itself.</t>
+        </is>
+      </c>
+      <c r="P46" s="24" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="24" t="n">
+        <v>16</v>
+      </c>
+      <c r="B47" s="24" t="inlineStr">
+        <is>
+          <t>The Glory Departs</t>
+        </is>
+      </c>
+      <c r="C47" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel 11</t>
+        </is>
+      </c>
+      <c r="E47" s="24" t="inlineStr">
+        <is>
+          <t>Impending judgement — and a glimmer of hope</t>
+        </is>
+      </c>
+      <c r="F47" s="24" t="inlineStr">
+        <is>
+          <t>Israel’s sin has driven God from His temple. Yet how does God show He has not abandoned His people (11:16)?</t>
+        </is>
+      </c>
+      <c r="G47" s="24" t="inlineStr">
+        <is>
+          <t>Where does God go with them?</t>
+        </is>
+      </c>
+      <c r="H47" s="24" t="inlineStr">
+        <is>
+          <t>Even as He sends them into exile, God promises to be a ‘sanctuary’ for them there (11:16) — He follows His people into exile rather than abandoning them.</t>
+        </is>
+      </c>
+      <c r="I47" s="24" t="inlineStr">
+        <is>
+          <t>How does God intend to restore Israel (11:17-20; cf. 36:26-27)? Why is this grace and hope — to the exiles and to us?</t>
+        </is>
+      </c>
+      <c r="J47" s="24" t="inlineStr">
+        <is>
+          <t>A heart of stone removed; a new heart and spirit given. Who receives that Spirit in the NT (John 14:15-17; 15:26)?</t>
+        </is>
+      </c>
+      <c r="K47" s="24" t="inlineStr">
+        <is>
+          <t>God will bring back a remnant and give them a new heart and spirit, removing the heart of stone (11:19). To us, this is the Spirit given in Christ (John 14-15) — doing what Israel never could.</t>
+        </is>
+      </c>
+      <c r="L47" s="24" t="inlineStr"/>
+      <c r="M47" s="24" t="inlineStr"/>
+      <c r="N47" s="24" t="inlineStr"/>
+      <c r="O47" s="24" t="inlineStr">
+        <is>
+          <t>God gives Israel over to judgement, yet does not abandon them — He follows them into exile and promises a new heart and a new spirit, removing the heart of stone so they can finally love and follow Him. That promise is fulfilled in the Holy Spirit given to believers in Christ.</t>
+        </is>
+      </c>
+      <c r="P47" s="24" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="B48" s="24" t="inlineStr">
+        <is>
+          <t>Clinging to the Promise</t>
+        </is>
+      </c>
+      <c r="C48" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="24" t="inlineStr">
+        <is>
+          <t>Psalm 89:1-4</t>
+        </is>
+      </c>
+      <c r="E48" s="24" t="inlineStr">
+        <is>
+          <t>Praising God’s promise of an eternal kingdom to David</t>
+        </is>
+      </c>
+      <c r="F48" s="24" t="inlineStr">
+        <is>
+          <t>What does the psalmist celebrate about God in these opening verses?</t>
+        </is>
+      </c>
+      <c r="G48" s="24" t="inlineStr">
+        <is>
+          <t>Note the words ‘steadfast love’ and ‘faithfulness’, and the covenant with David (v.3-4).</t>
+        </is>
+      </c>
+      <c r="H48" s="24" t="inlineStr">
+        <is>
+          <t>He sings of the Lord’s steadfast love and faithfulness ‘forever’, grounded in God’s covenant with David: an offspring and throne established for all generations (v.3-4).</t>
+        </is>
+      </c>
+      <c r="I48" s="24" t="inlineStr"/>
+      <c r="J48" s="24" t="inlineStr"/>
+      <c r="K48" s="24" t="inlineStr"/>
+      <c r="L48" s="24" t="inlineStr"/>
+      <c r="M48" s="24" t="inlineStr"/>
+      <c r="N48" s="24" t="inlineStr"/>
+      <c r="O48" s="24" t="inlineStr">
+        <is>
+          <t>The psalm begins in praise, anchored on God’s steadfast love and His covenant oath to David — an eternal throne. This promise is the ground the psalmist will cling to when everything else collapses.</t>
+        </is>
+      </c>
+      <c r="P48" s="24" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="B49" s="24" t="inlineStr">
+        <is>
+          <t>Clinging to the Promise</t>
+        </is>
+      </c>
+      <c r="C49" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" s="24" t="inlineStr">
+        <is>
+          <t>Psalm 89:5-18</t>
+        </is>
+      </c>
+      <c r="E49" s="24" t="inlineStr">
+        <is>
+          <t>Praising the God who strengthens the King</t>
+        </is>
+      </c>
+      <c r="F49" s="24" t="inlineStr">
+        <is>
+          <t>What kind of God is praised in vv.5-18, and how does that relate to the king?</t>
+        </is>
+      </c>
+      <c r="G49" s="24" t="inlineStr">
+        <is>
+          <t>Think of God’s power over creation and the heavens, and v.16-18 (‘our king belongs to the Lord’).</t>
+        </is>
+      </c>
+      <c r="H49" s="24" t="inlineStr">
+        <is>
+          <t>The incomparable God who rules the raging sea and the heavens — Israel’s strength and shield, whose power stands behind the king: ‘our king belongs to the Holy One of Israel’ (v.18).</t>
+        </is>
+      </c>
+      <c r="I49" s="24" t="inlineStr"/>
+      <c r="J49" s="24" t="inlineStr"/>
+      <c r="K49" s="24" t="inlineStr"/>
+      <c r="L49" s="24" t="inlineStr"/>
+      <c r="M49" s="24" t="inlineStr"/>
+      <c r="N49" s="24" t="inlineStr"/>
+      <c r="O49" s="24" t="inlineStr">
+        <is>
+          <t>The God who strengthens the king is the incomparable Lord of creation and the heavens. The king’s security rests entirely on this mighty God — which makes the later judgement all the more painful.</t>
+        </is>
+      </c>
+      <c r="P49" s="24" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="B50" s="24" t="inlineStr">
+        <is>
+          <t>Clinging to the Promise</t>
+        </is>
+      </c>
+      <c r="C50" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" s="24" t="inlineStr">
+        <is>
+          <t>Psalm 89:19-37</t>
+        </is>
+      </c>
+      <c r="E50" s="24" t="inlineStr">
+        <is>
+          <t>God’s steadfast love and forever-promise to David</t>
+        </is>
+      </c>
+      <c r="F50" s="24" t="inlineStr">
+        <is>
+          <t>What specifically does God promise David here, and how certain is it (vv.28-37)?</t>
+        </is>
+      </c>
+      <c r="G50" s="24" t="inlineStr">
+        <is>
+          <t>Look at ‘forever’, ‘as long as the heavens endure’, and the oath ‘I will not lie to David’.</t>
+        </is>
+      </c>
+      <c r="H50" s="24" t="inlineStr">
+        <is>
+          <t>Steadfast love kept forever and a throne as sure as sun and moon (v.29, 36-37); even if David’s sons sin, God disciplines them but will not remove His love or lie to David (v.33-35). Utterly certain.</t>
+        </is>
+      </c>
+      <c r="I50" s="24" t="inlineStr">
+        <is>
+          <t>What is the psalmist anchoring his hope on as he rehearses all this?</t>
+        </is>
+      </c>
+      <c r="J50" s="24" t="inlineStr">
+        <is>
+          <t>Why recount the promise in such detail?</t>
+        </is>
+      </c>
+      <c r="K50" s="24" t="inlineStr">
+        <is>
+          <t>On God’s own character and oath — His steadfast love and faithfulness — which he will throw back to God in the lament: You promised; remember it.</t>
+        </is>
+      </c>
+      <c r="L50" s="24" t="inlineStr"/>
+      <c r="M50" s="24" t="inlineStr"/>
+      <c r="N50" s="24" t="inlineStr"/>
+      <c r="O50" s="24" t="inlineStr">
+        <is>
+          <t>God’s promise to David is spelled out in its fullness and certainty — steadfast love that will not be removed, a throne as sure as sun and moon, sworn by God who cannot lie. The psalmist piles up the promise precisely so he can plead it when reality seems to contradict it.</t>
+        </is>
+      </c>
+      <c r="P50" s="24" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="B51" s="24" t="inlineStr">
+        <is>
+          <t>Clinging to the Promise</t>
+        </is>
+      </c>
+      <c r="C51" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="D51" s="24" t="inlineStr">
+        <is>
+          <t>Psalm 89:38-45</t>
+        </is>
+      </c>
+      <c r="E51" s="24" t="inlineStr">
+        <is>
+          <t>God has judged His King, kingdom and people</t>
+        </is>
+      </c>
+      <c r="F51" s="24" t="inlineStr">
+        <is>
+          <t>The tone turns sharply at v.38. What has God done, and who bears the brunt of it?</t>
+        </is>
+      </c>
+      <c r="G51" s="24" t="inlineStr">
+        <is>
+          <t>‘But now you have cast off and rejected…’ Note the language is aimed at the throne/king.</t>
+        </is>
+      </c>
+      <c r="H51" s="24" t="inlineStr">
+        <is>
+          <t>God has ‘cast off and rejected’, renounced the covenant, cast the king’s throne to the ground and shamed him (v.38-45). The judgement falls on the king, who bears the people — so what was promised ‘forever’ now looks shattered.</t>
+        </is>
+      </c>
+      <c r="I51" s="24" t="inlineStr"/>
+      <c r="J51" s="24" t="inlineStr"/>
+      <c r="K51" s="24" t="inlineStr"/>
+      <c r="L51" s="24" t="inlineStr"/>
+      <c r="M51" s="24" t="inlineStr"/>
+      <c r="N51" s="24" t="inlineStr"/>
+      <c r="O51" s="24" t="inlineStr">
+        <is>
+          <t>The promise collides with brutal reality: God has judged His king — rejected, defeated, shamed, his throne cast down. Because the king bears the people, their whole hope seems to collapse with him. This is the darkness the psalm refuses to hide.</t>
+        </is>
+      </c>
+      <c r="P51" s="24" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="B52" s="24" t="inlineStr">
+        <is>
+          <t>Clinging to the Promise</t>
+        </is>
+      </c>
+      <c r="C52" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="D52" s="24" t="inlineStr">
+        <is>
+          <t>Psalm 89:46-52</t>
+        </is>
+      </c>
+      <c r="E52" s="24" t="inlineStr">
+        <is>
+          <t>‘How long, O Lord?’ — pleading the promises</t>
+        </is>
+      </c>
+      <c r="F52" s="24" t="inlineStr">
+        <is>
+          <t>How does the psalmist respond to the darkness (vv.46-51)?</t>
+        </is>
+      </c>
+      <c r="G52" s="24" t="inlineStr">
+        <is>
+          <t>‘How long, O Lord?’ and ‘Lord, where is your steadfast love of old…?’</t>
+        </is>
+      </c>
+      <c r="H52" s="24" t="inlineStr">
+        <is>
+          <t>Not with despair but a clinging cry: ‘How long, O Lord?’ (v.46) and ‘where is your steadfast love of old… you swore to David?’ (v.49). ‘How long’ assumes it is a matter of when, not if.</t>
+        </is>
+      </c>
+      <c r="I52" s="24" t="inlineStr"/>
+      <c r="J52" s="24" t="inlineStr"/>
+      <c r="K52" s="24" t="inlineStr"/>
+      <c r="L52" s="24" t="inlineStr"/>
+      <c r="M52" s="24" t="inlineStr"/>
+      <c r="N52" s="24" t="inlineStr"/>
+      <c r="O52" s="24" t="inlineStr">
+        <is>
+          <t>The psalm ends not with resolution but with a clinging cry: ‘How long?’ and ‘remember your steadfast love to David.’ It is the honest prayer of faith in exile — pleading the promise, trusting it is a matter of when, not if. (v.52 closes Book 3 with ‘Blessed be the Lord forever’.)</t>
+        </is>
+      </c>
+      <c r="P52" s="24" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="24" t="n">
+        <v>18</v>
+      </c>
+      <c r="B53" s="24" t="inlineStr">
+        <is>
+          <t>God’s King Who Saves</t>
+        </is>
+      </c>
+      <c r="C53" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 9:1-7</t>
+        </is>
+      </c>
+      <c r="E53" s="24" t="inlineStr">
+        <is>
+          <t>The King is God Himself</t>
+        </is>
+      </c>
+      <c r="F53" s="24" t="inlineStr">
+        <is>
+          <t>Put yourself in Isaiah’s day. What is new or shocking about this King (esp. v.6)?</t>
+        </is>
+      </c>
+      <c r="G53" s="24" t="inlineStr">
+        <is>
+          <t>Read the four names in v.6 — ‘Wonderful Counsellor, Mighty God, Everlasting Father, Prince of Peace’.</t>
+        </is>
+      </c>
+      <c r="H53" s="24" t="inlineStr">
+        <is>
+          <t>David’s son is described in divine terms — ‘Mighty God’, ‘Everlasting Father’ (v.6). Nobody reading 2 Samuel 7 expected God Himself to be David’s son.</t>
+        </is>
+      </c>
+      <c r="I53" s="24" t="inlineStr">
+        <is>
+          <t>What does v.7 add about His kingdom?</t>
+        </is>
+      </c>
+      <c r="J53" s="24" t="inlineStr">
+        <is>
+          <t>‘Of the increase of his government and of peace there will be no end…’</t>
+        </is>
+      </c>
+      <c r="K53" s="24" t="inlineStr">
+        <is>
+          <t>An ever-increasing government and peace with no end, on David’s throne, upheld in justice forever — and ‘the zeal of the Lord of hosts will do this’: God Himself guarantees it.</t>
+        </is>
+      </c>
+      <c r="L53" s="24" t="inlineStr"/>
+      <c r="M53" s="24" t="inlineStr"/>
+      <c r="N53" s="24" t="inlineStr"/>
+      <c r="O53" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah stuns his hearers: the promised son of David is God Himself — Mighty God, Prince of Peace — whose just and peaceful reign will never end. What God swore to David ‘forever’, God Himself will accomplish.</t>
+        </is>
+      </c>
+      <c r="P53" s="24" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="24" t="n">
+        <v>18</v>
+      </c>
+      <c r="B54" s="24" t="inlineStr">
+        <is>
+          <t>God’s King Who Saves</t>
+        </is>
+      </c>
+      <c r="C54" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 11:1-16</t>
+        </is>
+      </c>
+      <c r="E54" s="24" t="inlineStr">
+        <is>
+          <t>The Spirit-anointed King who renews creation</t>
+        </is>
+      </c>
+      <c r="F54" s="24" t="inlineStr">
+        <is>
+          <t>How does the Spirit relate to this King (v.1-2), and how is that different from before?</t>
+        </is>
+      </c>
+      <c r="G54" s="24" t="inlineStr">
+        <is>
+          <t>Recall the judges, Saul and David — the Spirit ‘rushed upon’ them. What’s different here?</t>
+        </is>
+      </c>
+      <c r="H54" s="24" t="inlineStr">
+        <is>
+          <t>The Spirit ‘rests’ on Him permanently — unlike the judges and Saul, where the Spirit ‘rushed upon’ someone temporarily. That permanence marks the true Davidic King.</t>
+        </is>
+      </c>
+      <c r="I54" s="24" t="inlineStr">
+        <is>
+          <t>What is startlingly new about His reign in v.3-9?</t>
+        </is>
+      </c>
+      <c r="J54" s="24" t="inlineStr">
+        <is>
+          <t>Note the scale of His judging (whole earth) and the change to nature (wolf and lamb).</t>
+        </is>
+      </c>
+      <c r="K54" s="24" t="inlineStr">
+        <is>
+          <t>He judges the whole earth in righteousness (v.3-4) and changes creation itself — wolf with lamb, the earth ‘full of the knowledge of the Lord’ (v.6-9). He begins to undo the Fall.</t>
+        </is>
+      </c>
+      <c r="L54" s="24" t="inlineStr">
+        <is>
+          <t>What does v.16 (and v.13) add?</t>
+        </is>
+      </c>
+      <c r="M54" s="24" t="inlineStr">
+        <is>
+          <t>A ‘highway from Assyria’ — Exodus language, and peace between north and south.</t>
+        </is>
+      </c>
+      <c r="N54" s="24" t="inlineStr">
+        <is>
+          <t>A second ‘Exodus’ — a highway bringing exiles home and making peace between north and south (v.13, 16). God leads His people home again.</t>
+        </is>
+      </c>
+      <c r="O54" s="24" t="inlineStr">
+        <is>
+          <t>The King on whom the Spirit permanently rests judges the whole earth in righteousness, begins to reverse the Fall (creation at peace, full of the knowledge of the Lord), and leads a new Exodus home. The promise now stretches to all the earth.</t>
+        </is>
+      </c>
+      <c r="P54" s="24" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="24" t="n">
+        <v>18</v>
+      </c>
+      <c r="B55" s="24" t="inlineStr">
+        <is>
+          <t>God’s King Who Saves</t>
+        </is>
+      </c>
+      <c r="C55" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D55" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 25:1-12</t>
+        </is>
+      </c>
+      <c r="E55" s="24" t="inlineStr">
+        <is>
+          <t>A feast for all peoples; death swallowed up</t>
+        </is>
+      </c>
+      <c r="F55" s="24" t="inlineStr">
+        <is>
+          <t>What is shocking about the feast in v.6-7?</t>
+        </is>
+      </c>
+      <c r="G55" s="24" t="inlineStr">
+        <is>
+          <t>‘For all peoples’ — and compare Exodus 24 (eating before God).</t>
+        </is>
+      </c>
+      <c r="H55" s="24" t="inlineStr">
+        <is>
+          <t>A feast of rich food ‘for all peoples’ on God’s mountain (v.6) — echoing Exodus 24 but with no veil or barrier, and all nations drawn near, not just Israel.</t>
+        </is>
+      </c>
+      <c r="I55" s="24" t="inlineStr">
+        <is>
+          <t>What does v.7-8 promise, and why is it staggering?</t>
+        </is>
+      </c>
+      <c r="J55" s="24" t="inlineStr">
+        <is>
+          <t>What is ‘swallowed up forever’?</t>
+        </is>
+      </c>
+      <c r="K55" s="24" t="inlineStr">
+        <is>
+          <t>God swallows up death itself forever and wipes away every tear (v.7-8). The curse of Genesis 3 is reversed — and it is God Himself who does it.</t>
+        </is>
+      </c>
+      <c r="L55" s="24" t="inlineStr"/>
+      <c r="M55" s="24" t="inlineStr"/>
+      <c r="N55" s="24" t="inlineStr"/>
+      <c r="O55" s="24" t="inlineStr">
+        <is>
+          <t>On His mountain God spreads a feast for all peoples and swallows up death forever, wiping away every tear. The curse of Genesis 3 is undone — and the host is the Lord of hosts Himself.</t>
+        </is>
+      </c>
+      <c r="P55" s="24" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="24" t="n">
+        <v>18</v>
+      </c>
+      <c r="B56" s="24" t="inlineStr">
+        <is>
+          <t>God’s King Who Saves</t>
+        </is>
+      </c>
+      <c r="C56" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="D56" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 40:1-5</t>
+        </is>
+      </c>
+      <c r="E56" s="24" t="inlineStr">
+        <is>
+          <t>Comfort: iniquity pardoned, the Lord comes</t>
+        </is>
+      </c>
+      <c r="F56" s="24" t="inlineStr">
+        <is>
+          <t>Why is ‘her iniquity is pardoned’ (v.2) the deepest comfort for an exile?</t>
+        </is>
+      </c>
+      <c r="G56" s="24" t="inlineStr">
+        <is>
+          <t>What was exile the consequence of?</t>
+        </is>
+      </c>
+      <c r="H56" s="24" t="inlineStr">
+        <is>
+          <t>Exile was the consequence of iniquity; so if the iniquity itself is pardoned (v.2), the root problem — not just the symptoms — is finally dealt with.</t>
+        </is>
+      </c>
+      <c r="I56" s="24" t="inlineStr">
+        <is>
+          <t>Whose way is being prepared on the highway (v.3-5), and how far does it reach?</t>
+        </is>
+      </c>
+      <c r="J56" s="24" t="inlineStr">
+        <is>
+          <t>‘Prepare the way of the Lord’ — and ‘all flesh’.</t>
+        </is>
+      </c>
+      <c r="K56" s="24" t="inlineStr">
+        <is>
+          <t>The highway is for ‘all flesh’, and it is prepared for GOD Himself to come: ‘Prepare the way of the Lord’ (v.3-5). God comes in person to lead His people home.</t>
+        </is>
+      </c>
+      <c r="L56" s="24" t="inlineStr"/>
+      <c r="M56" s="24" t="inlineStr"/>
+      <c r="N56" s="24" t="inlineStr"/>
+      <c r="O56" s="24" t="inlineStr">
+        <is>
+          <t>The comfort of Isaiah 40 is that iniquity itself is pardoned — the root of exile dealt with — and that God Himself comes in person, for all flesh, to lead His people home. The pieces point to one King: God come to save.</t>
+        </is>
+      </c>
+      <c r="P56" s="24" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="24" t="n">
+        <v>19</v>
+      </c>
+      <c r="B57" s="24" t="inlineStr">
+        <is>
+          <t>The Suffering Servant</t>
+        </is>
+      </c>
+      <c r="C57" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 52:1-12</t>
+        </is>
+      </c>
+      <c r="E57" s="24" t="inlineStr">
+        <is>
+          <t>God’s coming salvation — good news proclaimed</t>
+        </is>
+      </c>
+      <c r="F57" s="24" t="inlineStr">
+        <is>
+          <t>What is the ‘good news’ the herald proclaims (v.7-10)?</t>
+        </is>
+      </c>
+      <c r="G57" s="24" t="inlineStr">
+        <is>
+          <t>‘How beautiful… the feet of him who brings good news’ — what is the message?</t>
+        </is>
+      </c>
+      <c r="H57" s="24" t="inlineStr">
+        <is>
+          <t>‘Your God reigns’ (v.7) — God is returning to Zion to comfort and redeem His people before all nations. Salvation is coming, and God Himself brings it.</t>
+        </is>
+      </c>
+      <c r="I57" s="24" t="inlineStr"/>
+      <c r="J57" s="24" t="inlineStr"/>
+      <c r="K57" s="24" t="inlineStr"/>
+      <c r="L57" s="24" t="inlineStr"/>
+      <c r="M57" s="24" t="inlineStr"/>
+      <c r="N57" s="24" t="inlineStr"/>
+      <c r="O57" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 52 heralds good news: ‘Your God reigns.’ God Himself is coming to redeem His people in sight of all the earth. The question the next verses answer is HOW — and it is utterly unexpected.</t>
+        </is>
+      </c>
+      <c r="P57" s="24" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="24" t="n">
+        <v>19</v>
+      </c>
+      <c r="B58" s="24" t="inlineStr">
+        <is>
+          <t>The Suffering Servant</t>
+        </is>
+      </c>
+      <c r="C58" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 52:13-53:12</t>
+        </is>
+      </c>
+      <c r="E58" s="24" t="inlineStr">
+        <is>
+          <t>The fourth Servant Song</t>
+        </is>
+      </c>
+      <c r="F58" s="24" t="inlineStr">
+        <is>
+          <t>What does the Lord say about this Servant (52:13-15)?</t>
+        </is>
+      </c>
+      <c r="G58" s="24" t="inlineStr">
+        <is>
+          <t>Note both ‘high and lifted up… exalted’ and ‘his appearance so marred’.</t>
+        </is>
+      </c>
+      <c r="H58" s="24" t="inlineStr">
+        <is>
+          <t>He will be exalted, ‘high and lifted up’ (language used of God in Isaiah), yet his appearance is marred beyond recognition (52:13-15). Exaltation and suffering held together.</t>
+        </is>
+      </c>
+      <c r="I58" s="24" t="inlineStr">
+        <is>
+          <t>How do people respond to the Servant, and what is actually happening to him (53:1-10)?</t>
+        </is>
+      </c>
+      <c r="J58" s="24" t="inlineStr">
+        <is>
+          <t>‘Despised and rejected’… but ‘pierced for OUR transgressions’. Who is he suffering for?</t>
+        </is>
+      </c>
+      <c r="K58" s="24" t="inlineStr">
+        <is>
+          <t>He is despised and assumed ‘stricken by God’ — but the truth is the opposite: ‘he was pierced for OUR transgressions… the Lord has laid on him the iniquity of us all’ (53:5-6). He suffers as our substitute.</t>
+        </is>
+      </c>
+      <c r="L58" s="24" t="inlineStr">
+        <is>
+          <t>How does the Lord describe what the Servant achieves in the end (53:11-12)?</t>
+        </is>
+      </c>
+      <c r="M58" s="24" t="inlineStr">
+        <is>
+          <t>‘Make many to be accounted righteous’; ‘bore the sin of many’.</t>
+        </is>
+      </c>
+      <c r="N58" s="24" t="inlineStr">
+        <is>
+          <t>‘By his knowledge the righteous one, my servant, makes many to be accounted righteous, and he shall bear their iniquities’ (v.11). He bears the sin of many and makes intercession for them.</t>
+        </is>
+      </c>
+      <c r="O58" s="24" t="inlineStr">
+        <is>
+          <t>The exalted Servant is the rejected one: pierced for our transgressions, carrying the iniquity the Lord laid on him, pouring out his soul to death as a substitute — so that he makes ‘many to be accounted righteous’. This is how God’s salvation comes.</t>
+        </is>
+      </c>
+      <c r="P58" s="24" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="24" t="n">
+        <v>19</v>
+      </c>
+      <c r="B59" s="24" t="inlineStr">
+        <is>
+          <t>The Suffering Servant</t>
+        </is>
+      </c>
+      <c r="C59" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D59" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 54</t>
+        </is>
+      </c>
+      <c r="E59" s="24" t="inlineStr">
+        <is>
+          <t>The response: ‘Sing!’</t>
+        </is>
+      </c>
+      <c r="F59" s="24" t="inlineStr">
+        <is>
+          <t>How are God’s people called to respond to the Servant Song (54:1)?</t>
+        </is>
+      </c>
+      <c r="G59" s="24" t="inlineStr">
+        <is>
+          <t>The ‘barren one’ is told to do what?</t>
+        </is>
+      </c>
+      <c r="H59" s="24" t="inlineStr">
+        <is>
+          <t>‘Sing!’ The barren one is told to break into song for her coming offspring (54:1) — echoing the Servant who, though poured out to death, ‘shall see his offspring’ (53:10).</t>
+        </is>
+      </c>
+      <c r="I59" s="24" t="inlineStr">
+        <is>
+          <t>What reasons does Isaiah 54 give God’s people to praise Him?</t>
+        </is>
+      </c>
+      <c r="J59" s="24" t="inlineStr">
+        <is>
+          <t>Look at v.5-8 (relationship restored), v.9-10 (steadfast love), v.17 (‘servants’).</t>
+        </is>
+      </c>
+      <c r="K59" s="24" t="inlineStr">
+        <is>
+          <t>A restored, everlasting relationship with God (v.5-8), a covenant of peace and steadfast love that will never depart (v.9-10), and His people now called His ‘servants’ (v.17).</t>
+        </is>
+      </c>
+      <c r="L59" s="24" t="inlineStr"/>
+      <c r="M59" s="24" t="inlineStr"/>
+      <c r="N59" s="24" t="inlineStr"/>
+      <c r="O59" s="24" t="inlineStr">
+        <is>
+          <t>Isaiah 54 is the response: Sing! Because of the Servant, the barren rejoice with offspring, the relationship with God is restored forever in a covenant of steadfast love, and God’s people become His ‘servants’ too. The only fitting answer to the cross is worship.</t>
+        </is>
+      </c>
+      <c r="P59" s="24" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="B60" s="24" t="inlineStr">
+        <is>
+          <t>The New Covenant</t>
+        </is>
+      </c>
+      <c r="C60" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="24" t="inlineStr">
+        <is>
+          <t>Jeremiah 31:27-30</t>
+        </is>
+      </c>
+      <c r="E60" s="24" t="inlineStr">
+        <is>
+          <t>‘The days are coming’ — hope and questions</t>
+        </is>
+      </c>
+      <c r="F60" s="24" t="inlineStr">
+        <is>
+          <t>How do verses 27-30 offer hope to a people in exile?</t>
+        </is>
+      </c>
+      <c r="G60" s="24" t="inlineStr">
+        <is>
+          <t>‘The days are coming’… God will ‘watch over them to build and to plant’ (v.28); and the proverb about sour grapes.</t>
+        </is>
+      </c>
+      <c r="H60" s="24" t="inlineStr">
+        <is>
+          <t>God promises a reversal: once He watched ‘to pluck up’, now He will watch ‘to build and to plant’ (v.28); and each person now deals with God directly (v.29-30). A fresh, personal start.</t>
+        </is>
+      </c>
+      <c r="I60" s="24" t="inlineStr">
+        <is>
+          <t>What questions might verses 27-30 raise?</t>
+        </is>
+      </c>
+      <c r="J60" s="24" t="inlineStr">
+        <is>
+          <t>If everyone still dies for their own sin, how will the deeper sin problem be solved?</t>
+        </is>
+      </c>
+      <c r="K60" s="24" t="inlineStr">
+        <is>
+          <t>If each still bears their own sin (v.30), how will the heart problem that wrecked every covenant be fixed? It leaves a question the next verses answer.</t>
+        </is>
+      </c>
+      <c r="L60" s="24" t="inlineStr"/>
+      <c r="M60" s="24" t="inlineStr"/>
+      <c r="N60" s="24" t="inlineStr"/>
+      <c r="O60" s="24" t="inlineStr">
+        <is>
+          <t>God promises to ‘build and plant’ His people again and open a new, personal chapter with them. But it leaves a question hanging — how will their sin itself be dealt with? — preparing the way for the New Covenant.</t>
+        </is>
+      </c>
+      <c r="P60" s="24" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="B61" s="24" t="inlineStr">
+        <is>
+          <t>The New Covenant</t>
+        </is>
+      </c>
+      <c r="C61" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D61" s="24" t="inlineStr">
+        <is>
+          <t>Jeremiah 31:31-37</t>
+        </is>
+      </c>
+      <c r="E61" s="24" t="inlineStr">
+        <is>
+          <t>The New Covenant</t>
+        </is>
+      </c>
+      <c r="F61" s="24" t="inlineStr">
+        <is>
+          <t>What does this New Covenant look like (v.31-34)?</t>
+        </is>
+      </c>
+      <c r="G61" s="24" t="inlineStr">
+        <is>
+          <t>Not like the old one — note where the law goes, who knows God, what happens to sin.</t>
+        </is>
+      </c>
+      <c r="H61" s="24" t="inlineStr">
+        <is>
+          <t>‘Not like’ the broken Sinai covenant: God writes His law on their hearts, is their God, all know Him, and — the foundation — ‘I will remember their sin no more’ (v.33-34).</t>
+        </is>
+      </c>
+      <c r="I61" s="24" t="inlineStr">
+        <is>
+          <t>How does this New Covenant develop from the previous covenants (cf. Gen 17:1-9; Ex 19:1-6; Deut 30:1-10)?</t>
+        </is>
+      </c>
+      <c r="J61" s="24" t="inlineStr">
+        <is>
+          <t>Same promise — ‘I will be their God, they my people’ — but now written on the heart, not just commanded.</t>
+        </is>
+      </c>
+      <c r="K61" s="24" t="inlineStr">
+        <is>
+          <t>It keeps the earlier covenants’ heart — ‘I will be their God and they my people’ — but what Sinai commanded from outside, God now writes inside, guaranteed by His own forgiveness.</t>
+        </is>
+      </c>
+      <c r="L61" s="24" t="inlineStr">
+        <is>
+          <t>How certain is this covenant (v.35-37)?</t>
+        </is>
+      </c>
+      <c r="M61" s="24" t="inlineStr">
+        <is>
+          <t>‘Thus says the Lord’ — compared to the fixed order of sun, moon and stars.</t>
+        </is>
+      </c>
+      <c r="N61" s="24" t="inlineStr">
+        <is>
+          <t>As certain as creation: only if the fixed order of sun, moon and stars failed would God cast off His people (v.35-37). It is as unbreakable as the God who made the universe.</t>
+        </is>
+      </c>
+      <c r="O61" s="24" t="inlineStr">
+        <is>
+          <t>God promises a New Covenant unlike the broken Sinai one: His law written on the heart, all knowing Him, sin forgiven and remembered no more. It fulfils the earlier covenants’ ‘I will be their God’ from the inside out — and is as sure as creation itself.</t>
+        </is>
+      </c>
+      <c r="P61" s="24" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="B62" s="24" t="inlineStr">
+        <is>
+          <t>The New Covenant</t>
+        </is>
+      </c>
+      <c r="C62" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D62" s="24" t="inlineStr">
+        <is>
+          <t>Jeremiah 31:38-40</t>
+        </is>
+      </c>
+      <c r="E62" s="24" t="inlineStr">
+        <is>
+          <t>God’s new holy city</t>
+        </is>
+      </c>
+      <c r="F62" s="24" t="inlineStr">
+        <is>
+          <t>What does God promise in verses 38-40?</t>
+        </is>
+      </c>
+      <c r="G62" s="24" t="inlineStr">
+        <is>
+          <t>The city rebuilt — and what is said about the once-defiled places?</t>
+        </is>
+      </c>
+      <c r="H62" s="24" t="inlineStr">
+        <is>
+          <t>God will rebuild the city for Himself, and even the once-defiled places (the valley of dead bodies and ashes) will be ‘sacred to the Lord’ forever. Nothing is beyond His renewing grace.</t>
+        </is>
+      </c>
+      <c r="I62" s="24" t="inlineStr"/>
+      <c r="J62" s="24" t="inlineStr"/>
+      <c r="K62" s="24" t="inlineStr"/>
+      <c r="L62" s="24" t="inlineStr"/>
+      <c r="M62" s="24" t="inlineStr"/>
+      <c r="N62" s="24" t="inlineStr"/>
+      <c r="O62" s="24" t="inlineStr">
+        <is>
+          <t>God promises a rebuilt, holy city where even the once-defiled places become ‘sacred to the Lord’ forever. The New Covenant ends not just with forgiven hearts but a wholly renewed place — a glimpse of the new creation to come.</t>
+        </is>
+      </c>
+      <c r="P62" s="24" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B63" s="24" t="inlineStr">
+        <is>
+          <t>The New Temple</t>
+        </is>
+      </c>
+      <c r="C63" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel 43:1-12</t>
+        </is>
+      </c>
+      <c r="E63" s="24" t="inlineStr">
+        <is>
+          <t>The glory of the Lord returns to the new temple</t>
+        </is>
+      </c>
+      <c r="F63" s="24" t="inlineStr">
+        <is>
+          <t>Track where God’s glory and Spirit go in v.1-5. What is significant about these locations (compare chapters 8-11)?</t>
+        </is>
+      </c>
+      <c r="G63" s="24" t="inlineStr">
+        <is>
+          <t>The glory comes from the EAST — where did it go in chapter 10-11? And the Spirit lifts Ezekiel as before.</t>
+        </is>
+      </c>
+      <c r="H63" s="24" t="inlineStr">
+        <is>
+          <t>The glory comes from the EAST — the very direction it left in chapters 10-11 — and fills the temple (a throwback to Exodus 40 and 1 Kings 8). The God who left in judgement returns in grace.</t>
+        </is>
+      </c>
+      <c r="I63" s="24" t="inlineStr">
+        <is>
+          <t>In 43:6-9, what is God’s message to His people?</t>
+        </is>
+      </c>
+      <c r="J63" s="24" t="inlineStr">
+        <is>
+          <t>What must stop, so that God can dwell with them forever?</t>
+        </is>
+      </c>
+      <c r="K63" s="24" t="inlineStr">
+        <is>
+          <t>‘This is the place of my throne… where I will dwell in the midst of Israel forever’ (43:7) — but they must put away the idolatry that defiled His house. Holiness befits His returned presence.</t>
+        </is>
+      </c>
+      <c r="L63" s="24" t="inlineStr">
+        <is>
+          <t>In 43:10-12, why does the Lord stress Israel being ‘ashamed’, and how does that relate to ‘knowing the design of the temple’?</t>
+        </is>
+      </c>
+      <c r="M63" s="24" t="inlineStr">
+        <is>
+          <t>Knowing the measurements/design stands for knowing and keeping God’s law.</t>
+        </is>
+      </c>
+      <c r="N63" s="24" t="inlineStr">
+        <is>
+          <t>Seeing God’s holy design is meant to make Israel ashamed of their sin; being shown the temple’s measurements is really about knowing and keeping God’s law (v.12). The temple teaches obedience.</t>
+        </is>
+      </c>
+      <c r="O63" s="24" t="inlineStr">
+        <is>
+          <t>The glory that departed to the east in chapters 8-11 returns from the east to fill the new temple: God will dwell with His people forever. Confronted with His holy design, Israel is to be ashamed of their sin and to know and keep His law — the temple itself teaching obedience.</t>
+        </is>
+      </c>
+      <c r="P63" s="24" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B64" s="24" t="inlineStr">
+        <is>
+          <t>The New Temple</t>
+        </is>
+      </c>
+      <c r="C64" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" s="24" t="inlineStr">
+        <is>
+          <t>Ezekiel 47:1-12</t>
+        </is>
+      </c>
+      <c r="E64" s="24" t="inlineStr">
+        <is>
+          <t>The river of life flows from the temple</t>
+        </is>
+      </c>
+      <c r="F64" s="24" t="inlineStr">
+        <is>
+          <t>What is the symbolism of water flowing out from the temple (v.1-6)?</t>
+        </is>
+      </c>
+      <c r="G64" s="24" t="inlineStr">
+        <is>
+          <t>Note the ‘physical impossible-ness’ — a river sourced from a building, deepening as it flows outward.</t>
+        </is>
+      </c>
+      <c r="H64" s="24" t="inlineStr">
+        <is>
+          <t>Water flows from under the temple and, impossibly, deepens the further it goes — ankles, knees, waist, then an uncrossable river (v.1-6). Life pours out of God’s presence and keeps growing.</t>
+        </is>
+      </c>
+      <c r="I64" s="24" t="inlineStr">
+        <is>
+          <t>Note the effects of the water (v.7-12). What is God showing His people?</t>
+        </is>
+      </c>
+      <c r="J64" s="24" t="inlineStr">
+        <is>
+          <t>A river through the desert (Arabah); the Dead Sea made fresh; trees for food and healing.</t>
+        </is>
+      </c>
+      <c r="K64" s="24" t="inlineStr">
+        <is>
+          <t>It heals everywhere it flows — even reviving the Dead Sea — with fish teeming and trees bearing fruit and leaves ‘for healing’ (v.7-12). God remakes a new creation, like Eden renewed.</t>
+        </is>
+      </c>
+      <c r="L64" s="24" t="inlineStr"/>
+      <c r="M64" s="24" t="inlineStr"/>
+      <c r="N64" s="24" t="inlineStr"/>
+      <c r="O64" s="24" t="inlineStr">
+        <is>
+          <t>From the temple flows an impossible, ever-deepening river that brings life and healing everywhere — even reviving the Dead Sea — remaking creation like Eden renewed. God’s presence pours life out into all the world, pointing to the Spirit’s living water and the river of life in the New Creation (Rev 22).</t>
+        </is>
+      </c>
+      <c r="P64" s="24" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B65" s="24" t="inlineStr">
+        <is>
+          <t>How the OT Ends</t>
+        </is>
+      </c>
+      <c r="C65" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="24" t="inlineStr">
+        <is>
+          <t>Nehemiah 8-9</t>
+        </is>
+      </c>
+      <c r="E65" s="24" t="inlineStr">
+        <is>
+          <t>The Law read: weeping, joy and confession</t>
+        </is>
+      </c>
+      <c r="F65" s="24" t="inlineStr">
+        <is>
+          <t>How do the people respond to the reading of the Law (Neh 8)?</t>
+        </is>
+      </c>
+      <c r="G65" s="24" t="inlineStr">
+        <is>
+          <t>Note both their weeping (8:9) and the call to rejoice (8:10-12).</t>
+        </is>
+      </c>
+      <c r="H65" s="24" t="inlineStr">
+        <is>
+          <t>They listen attentively and weep when they understand the Law (8:9), but are told ‘the joy of the Lord is your strength’ (8:10) and celebrate. God’s word brings both grief over sin and joy.</t>
+        </is>
+      </c>
+      <c r="I65" s="24" t="inlineStr">
+        <is>
+          <t>In the long confession of Nehemiah 9, how do they summarise the whole story of God and Israel?</t>
+        </is>
+      </c>
+      <c r="J65" s="24" t="inlineStr">
+        <is>
+          <t>See 9:33 — who was faithful, who was not?</t>
+        </is>
+      </c>
+      <c r="K65" s="24" t="inlineStr">
+        <is>
+          <t>Rehearsing the whole story, they confess: ‘you have dealt faithfully and we have acted wickedly’ (9:33). God kept faith; Israel rebelled — the real problem is their own hearts.</t>
+        </is>
+      </c>
+      <c r="L65" s="24" t="inlineStr"/>
+      <c r="M65" s="24" t="inlineStr"/>
+      <c r="N65" s="24" t="inlineStr"/>
+      <c r="O65" s="24" t="inlineStr">
+        <is>
+          <t>Hearing the Law, the returned people weep, then rejoice, then confess: through the whole story God was faithful and they were not (9:33). The problem the whole OT has exposed is named plainly — the human heart.</t>
+        </is>
+      </c>
+      <c r="P65" s="24" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B66" s="24" t="inlineStr">
+        <is>
+          <t>How the OT Ends</t>
+        </is>
+      </c>
+      <c r="C66" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" s="24" t="inlineStr">
+        <is>
+          <t>Nehemiah 10</t>
+        </is>
+      </c>
+      <c r="E66" s="24" t="inlineStr">
+        <is>
+          <t>The covenant renewed by oath</t>
+        </is>
+      </c>
+      <c r="F66" s="24" t="inlineStr">
+        <is>
+          <t>What do the people commit to in their renewed covenant (Neh 10)?</t>
+        </is>
+      </c>
+      <c r="G66" s="24" t="inlineStr">
+        <is>
+          <t>They bind themselves by ‘a curse and an oath’ — to do what?</t>
+        </is>
+      </c>
+      <c r="H66" s="24" t="inlineStr">
+        <is>
+          <t>They bind themselves by solemn oath to obey God’s Law — no intermarriage, keeping the Sabbath, and supporting the temple (10:28-39). A sincere, wholehearted recommitment.</t>
+        </is>
+      </c>
+      <c r="I66" s="24" t="inlineStr"/>
+      <c r="J66" s="24" t="inlineStr"/>
+      <c r="K66" s="24" t="inlineStr"/>
+      <c r="L66" s="24" t="inlineStr"/>
+      <c r="M66" s="24" t="inlineStr"/>
+      <c r="N66" s="24" t="inlineStr"/>
+      <c r="O66" s="24" t="inlineStr">
+        <is>
+          <t>The people make a sincere, solemn covenant to obey God — no intermarriage, keep the Sabbath, support the temple. Everything looks set right. The question is whether oaths can hold a heart that has failed every time before.</t>
+        </is>
+      </c>
+      <c r="P66" s="24" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B67" s="24" t="inlineStr">
+        <is>
+          <t>How the OT Ends</t>
+        </is>
+      </c>
+      <c r="C67" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D67" s="24" t="inlineStr">
+        <is>
+          <t>Nehemiah 13</t>
+        </is>
+      </c>
+      <c r="E67" s="24" t="inlineStr">
+        <is>
+          <t>The relapse</t>
+        </is>
+      </c>
+      <c r="F67" s="24" t="inlineStr">
+        <is>
+          <t>Nehemiah returns after being away (13:6). What surprises you about the people, given what they had sworn?</t>
+        </is>
+      </c>
+      <c r="G67" s="24" t="inlineStr">
+        <is>
+          <t>Look at the temple (13:4-9), the Sabbath (13:15-22), and marriages (13:23-27) — the very things they vowed in ch.10.</t>
+        </is>
+      </c>
+      <c r="H67" s="24" t="inlineStr">
+        <is>
+          <t>They have broken the very vows of chapter 10 — the temple profaned, the Sabbath violated, intermarriage again (13:4-27). Within a short time the heartfelt covenant has collapsed.</t>
+        </is>
+      </c>
+      <c r="I67" s="24" t="inlineStr">
+        <is>
+          <t>What does this ending reveal about the human heart — and what the OT is ultimately waiting for?</t>
+        </is>
+      </c>
+      <c r="J67" s="24" t="inlineStr">
+        <is>
+          <t>If Law, miracle, exile and sincere vows can’t fix it, what is needed?</t>
+        </is>
+      </c>
+      <c r="K67" s="24" t="inlineStr">
+        <is>
+          <t>No amount of Law or sincere resolution can change the heart — the problem since Genesis 3 is still unsolved. The OT ends home but unchanged, aching for the New Covenant and the Saviour-King, Jesus.</t>
+        </is>
+      </c>
+      <c r="L67" s="24" t="inlineStr"/>
+      <c r="M67" s="24" t="inlineStr"/>
+      <c r="N67" s="24" t="inlineStr"/>
+      <c r="O67" s="24" t="inlineStr">
+        <is>
+          <t>Barely after swearing the covenant, the people break it — profaned temple, broken Sabbath, intermarriage. The OT ends honestly: home, but with the same unchanged heart. The only hope left is the New Covenant and the Saviour the whole story has been pointing to — Jesus.</t>
+        </is>
+      </c>
+      <c r="P67" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>